<commit_message>
20260106: Update LVS/DRC for Drawin Layers except ESD.
</commit_message>
<xml_diff>
--- a/Document/TR-1um_Drawing_Layer_DR_Table.xlsx
+++ b/Document/TR-1um_Drawing_Layer_DR_Table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/okamura/Library/CloudStorage/Dropbox/91_OpenPDK/TR-1um/Document/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{328E9EA7-D8E4-844A-B5C4-2B6780DA8963}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0D650A9-9EB4-984E-AA72-A3602D397E13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="800" yWindow="760" windowWidth="29440" windowHeight="18880" xr2:uid="{7F1200E8-B51D-9446-A5CE-CEA05B5231B7}"/>
+    <workbookView xWindow="1780" yWindow="760" windowWidth="29440" windowHeight="18880" xr2:uid="{7F1200E8-B51D-9446-A5CE-CEA05B5231B7}"/>
   </bookViews>
   <sheets>
     <sheet name="TR-1um_Drawing_Layer_DR_Table" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="499" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="228">
   <si>
     <t>WN.W1</t>
   </si>
@@ -224,18 +224,6 @@
     <t>ERWLMN11</t>
   </si>
   <si>
-    <t>PO.W1</t>
-  </si>
-  <si>
-    <t>PO.S1</t>
-  </si>
-  <si>
-    <t>PO.AP</t>
-  </si>
-  <si>
-    <t>PO.AN</t>
-  </si>
-  <si>
     <t>CO.W1</t>
   </si>
   <si>
@@ -254,9 +242,6 @@
     <t>CO.PG</t>
   </si>
   <si>
-    <t>CO.PO</t>
-  </si>
-  <si>
     <t>CO.AD</t>
   </si>
   <si>
@@ -287,9 +272,6 @@
     <t>V1.M1</t>
   </si>
   <si>
-    <t>V1.PO</t>
-  </si>
-  <si>
     <t>V1.CO</t>
   </si>
   <si>
@@ -305,9 +287,6 @@
     <t>IP62 Rule Name</t>
   </si>
   <si>
-    <t>PO.R1</t>
-  </si>
-  <si>
     <t>AC.R1</t>
   </si>
   <si>
@@ -401,12 +380,6 @@
     <t>ER1507</t>
   </si>
   <si>
-    <t>PR.W1</t>
-  </si>
-  <si>
-    <t>PR.S1</t>
-  </si>
-  <si>
     <t>ERRS04</t>
   </si>
   <si>
@@ -440,9 +413,6 @@
     <t>M1.SW</t>
   </si>
   <si>
-    <t>AR.PO</t>
-  </si>
-  <si>
     <t>AR.PW</t>
   </si>
   <si>
@@ -509,9 +479,6 @@
     <t>DN</t>
   </si>
   <si>
-    <t>PO</t>
-  </si>
-  <si>
     <t>CO</t>
   </si>
   <si>
@@ -524,9 +491,6 @@
     <t>AR</t>
   </si>
   <si>
-    <t>PO(AR)</t>
-  </si>
-  <si>
     <t>CO(RR)</t>
   </si>
   <si>
@@ -572,9 +536,6 @@
     <t>DN.W1</t>
   </si>
   <si>
-    <t>PO(G)</t>
-  </si>
-  <si>
     <t>Donut</t>
   </si>
   <si>
@@ -626,9 +587,6 @@
     <t>AP+AR</t>
   </si>
   <si>
-    <t>Prohibited</t>
-  </si>
-  <si>
     <t>WN-AC/AR related</t>
   </si>
   <si>
@@ -653,24 +611,9 @@
     <t>AP+AC</t>
   </si>
   <si>
-    <t>AR/PR related</t>
-  </si>
-  <si>
-    <t>AP-PO</t>
-  </si>
-  <si>
-    <t>AN-PO</t>
-  </si>
-  <si>
     <t>ECmin</t>
   </si>
   <si>
-    <t>PO.EP</t>
-  </si>
-  <si>
-    <t>PO.EN</t>
-  </si>
-  <si>
     <t>ERMP06</t>
   </si>
   <si>
@@ -680,21 +623,12 @@
     <t>AN(C)</t>
   </si>
   <si>
-    <t>PR.L1</t>
-  </si>
-  <si>
-    <t>AA+PO+PR</t>
-  </si>
-  <si>
     <t>WN(M)</t>
   </si>
   <si>
     <t>CO(S)</t>
   </si>
   <si>
-    <t>PO-AN</t>
-  </si>
-  <si>
     <t>RS</t>
   </si>
   <si>
@@ -713,7 +647,79 @@
     <t>RR(L)</t>
   </si>
   <si>
-    <t>PO.R2</t>
+    <t>ERCSIO13</t>
+  </si>
+  <si>
+    <t>AC.GC</t>
+  </si>
+  <si>
+    <t>GC</t>
+  </si>
+  <si>
+    <t>AP-GC</t>
+  </si>
+  <si>
+    <t>GC-AN</t>
+  </si>
+  <si>
+    <t>AN-GC</t>
+  </si>
+  <si>
+    <t>GC.W1</t>
+  </si>
+  <si>
+    <t>GC.S1</t>
+  </si>
+  <si>
+    <t>GC.AP</t>
+  </si>
+  <si>
+    <t>GC.AN</t>
+  </si>
+  <si>
+    <t>GC.EP</t>
+  </si>
+  <si>
+    <t>GC.EN</t>
+  </si>
+  <si>
+    <t>GC(G)</t>
+  </si>
+  <si>
+    <t>CO.GC</t>
+  </si>
+  <si>
+    <t>AR.GC</t>
+  </si>
+  <si>
+    <t>GC(AR)</t>
+  </si>
+  <si>
+    <t>GC.R1</t>
+  </si>
+  <si>
+    <t>GC.R2</t>
+  </si>
+  <si>
+    <t>V1.GC</t>
+  </si>
+  <si>
+    <t>GRohibited</t>
+  </si>
+  <si>
+    <t>AA+GC+GR</t>
+  </si>
+  <si>
+    <t>AR/GR related</t>
+  </si>
+  <si>
+    <t>GR.W1</t>
+  </si>
+  <si>
+    <t>GR.L1</t>
+  </si>
+  <si>
+    <t>GR.S1</t>
   </si>
 </sst>
 </file>
@@ -1771,7 +1777,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4478C0F2-BA21-8B4B-B7C2-220C0E7FA6A8}">
-  <dimension ref="B2:H107"/>
+  <dimension ref="B2:H108"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="19" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.6640625" style="4" customWidth="1"/>
@@ -1786,10 +1792,10 @@
   <sheetData>
     <row r="2" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B2" s="22" t="s">
-        <v>203</v>
+        <v>189</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>196</v>
+        <v>222</v>
       </c>
       <c r="D2" s="23"/>
       <c r="E2" s="22"/>
@@ -1799,39 +1805,39 @@
     </row>
     <row r="3" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="1" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="C3" s="19" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="D3" s="19" t="s">
-        <v>176</v>
+        <v>164</v>
       </c>
       <c r="E3" s="20" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="F3" s="21" t="s">
-        <v>170</v>
+        <v>158</v>
       </c>
       <c r="G3" s="21" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="H3" s="20" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="5" t="s">
-        <v>201</v>
+        <v>187</v>
       </c>
       <c r="C4" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>190</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>172</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>204</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>185</v>
       </c>
       <c r="F4" s="6">
         <v>0</v>
@@ -1841,16 +1847,16 @@
     </row>
     <row r="5" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="5" t="s">
-        <v>202</v>
+        <v>188</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>195</v>
+        <v>182</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>185</v>
+        <v>172</v>
       </c>
       <c r="F5" s="6">
         <v>0</v>
@@ -1860,16 +1866,16 @@
     </row>
     <row r="6" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="5" t="s">
-        <v>186</v>
+        <v>173</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>185</v>
+        <v>172</v>
       </c>
       <c r="F6" s="6">
         <v>0</v>
@@ -1879,16 +1885,16 @@
     </row>
     <row r="7" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="5" t="s">
-        <v>187</v>
+        <v>174</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>185</v>
+        <v>172</v>
       </c>
       <c r="F7" s="6">
         <v>0</v>
@@ -1898,16 +1904,16 @@
     </row>
     <row r="8" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="5" t="s">
-        <v>188</v>
+        <v>175</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>185</v>
+        <v>172</v>
       </c>
       <c r="F8" s="6">
         <v>0</v>
@@ -1917,16 +1923,16 @@
     </row>
     <row r="9" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="5" t="s">
-        <v>189</v>
+        <v>176</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>185</v>
+        <v>172</v>
       </c>
       <c r="F9" s="6">
         <v>0</v>
@@ -1936,10 +1942,10 @@
     </row>
     <row r="10" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B10" s="22" t="s">
-        <v>203</v>
+        <v>189</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>197</v>
+        <v>183</v>
       </c>
       <c r="D10" s="23"/>
       <c r="E10" s="22"/>
@@ -1949,25 +1955,25 @@
     </row>
     <row r="11" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="1" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>176</v>
+        <v>164</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>170</v>
+        <v>158</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
     </row>
     <row r="12" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
@@ -1975,11 +1981,11 @@
         <v>0</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="D12" s="11"/>
       <c r="E12" s="5" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="F12" s="6">
         <v>8</v>
@@ -1994,13 +2000,13 @@
         <v>1</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="F13" s="6">
         <v>12</v>
@@ -2015,13 +2021,13 @@
         <v>2</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="F14" s="6">
         <v>9.5</v>
@@ -2036,13 +2042,13 @@
         <v>3</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="F15" s="6">
         <v>12</v>
@@ -2057,13 +2063,13 @@
         <v>4</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="F16" s="6">
         <v>9.5</v>
@@ -2078,13 +2084,13 @@
         <v>5</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="F17" s="6">
         <v>8</v>
@@ -2099,13 +2105,13 @@
         <v>6</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="F18" s="6">
         <v>12</v>
@@ -2120,13 +2126,13 @@
         <v>7</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="F19" s="6">
         <v>5</v>
@@ -2141,13 +2147,13 @@
         <v>8</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="F20" s="6">
         <v>10</v>
@@ -2162,13 +2168,13 @@
         <v>21</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="F21" s="9">
         <v>4</v>
@@ -2183,13 +2189,13 @@
         <v>22</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="D22" s="13" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="F22" s="9">
         <v>10</v>
@@ -2204,13 +2210,13 @@
         <v>23</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="F23" s="9">
         <v>5</v>
@@ -2225,13 +2231,13 @@
         <v>24</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="F24" s="9">
         <v>4</v>
@@ -2246,11 +2252,11 @@
         <v>31</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="D25" s="11"/>
       <c r="E25" s="5" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="F25" s="6">
         <v>28.5</v>
@@ -2259,7 +2265,7 @@
         <v>120</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
     </row>
     <row r="26" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
@@ -2267,13 +2273,13 @@
         <v>32</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>58</v>
@@ -2288,13 +2294,13 @@
         <v>33</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="F27" s="6" t="s">
         <v>58</v>
@@ -2309,13 +2315,13 @@
         <v>34</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="F28" s="6">
         <v>3</v>
@@ -2330,13 +2336,13 @@
         <v>35</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="F29" s="6">
         <v>2.8</v>
@@ -2348,997 +2354,1001 @@
     </row>
     <row r="30" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="5" t="s">
-        <v>90</v>
+        <v>204</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>179</v>
+        <v>137</v>
       </c>
       <c r="F30" s="6">
+        <v>1.4</v>
+      </c>
+      <c r="G30" s="6"/>
+      <c r="H30" s="5" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="31" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B31" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C31" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="D31" s="11" t="s">
+        <v>194</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="F31" s="6">
         <v>0</v>
       </c>
-      <c r="G30" s="6"/>
-      <c r="H30" s="5"/>
-    </row>
-    <row r="31" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B31" s="22" t="s">
-        <v>203</v>
-      </c>
-      <c r="C31" s="18" t="s">
-        <v>198</v>
-      </c>
-      <c r="D31" s="23"/>
-      <c r="E31" s="22"/>
-      <c r="F31" s="24"/>
-      <c r="G31" s="24"/>
-      <c r="H31" s="22"/>
-    </row>
-    <row r="32" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="F32" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="G32" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="H32" s="1" t="s">
-        <v>88</v>
-      </c>
+      <c r="G31" s="6"/>
+      <c r="H31" s="5"/>
+    </row>
+    <row r="32" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B32" s="22" t="s">
+        <v>189</v>
+      </c>
+      <c r="C32" s="18" t="s">
+        <v>184</v>
+      </c>
+      <c r="D32" s="23"/>
+      <c r="E32" s="22"/>
+      <c r="F32" s="24"/>
+      <c r="G32" s="24"/>
+      <c r="H32" s="22"/>
     </row>
     <row r="33" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B33" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="C33" s="13" t="s">
-        <v>151</v>
-      </c>
-      <c r="D33" s="13"/>
-      <c r="E33" s="8" t="s">
-        <v>144</v>
-      </c>
-      <c r="F33" s="9">
-        <v>1.4</v>
-      </c>
-      <c r="G33" s="9"/>
-      <c r="H33" s="8" t="s">
-        <v>56</v>
+      <c r="B33" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="G33" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="H33" s="1" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="34" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B34" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>151</v>
-      </c>
-      <c r="D34" s="13" t="s">
-        <v>151</v>
-      </c>
+        <v>141</v>
+      </c>
+      <c r="D34" s="13"/>
       <c r="E34" s="8" t="s">
-        <v>145</v>
+        <v>134</v>
       </c>
       <c r="F34" s="9">
         <v>1.4</v>
       </c>
       <c r="G34" s="9"/>
       <c r="H34" s="8" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="35" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B35" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="D35" s="13" t="s">
-        <v>154</v>
+        <v>141</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="F35" s="9">
-        <v>2.8</v>
+        <v>1.4</v>
       </c>
       <c r="G35" s="9"/>
       <c r="H35" s="8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="36" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B36" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="D36" s="13" t="s">
-        <v>206</v>
+        <v>144</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="F36" s="9">
-        <v>3.4</v>
-      </c>
-      <c r="G36" s="9">
-        <v>60</v>
-      </c>
+        <v>2.8</v>
+      </c>
+      <c r="G36" s="9"/>
       <c r="H36" s="8" t="s">
-        <v>124</v>
+        <v>57</v>
       </c>
     </row>
     <row r="37" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B37" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C37" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="D37" s="13" t="s">
+        <v>206</v>
+      </c>
+      <c r="E37" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="C37" s="13" t="s">
-        <v>152</v>
-      </c>
-      <c r="D37" s="13" t="s">
-        <v>218</v>
-      </c>
-      <c r="E37" s="8" t="s">
-        <v>150</v>
-      </c>
       <c r="F37" s="9">
-        <v>1</v>
+        <v>3.4</v>
       </c>
       <c r="G37" s="9">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="H37" s="8" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
     </row>
     <row r="38" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B38" s="8" t="s">
-        <v>16</v>
+        <v>126</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
       <c r="D38" s="13" t="s">
-        <v>171</v>
+        <v>207</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="F38" s="9">
-        <v>7</v>
-      </c>
-      <c r="G38" s="9"/>
+        <v>1</v>
+      </c>
+      <c r="G38" s="9">
+        <v>30</v>
+      </c>
       <c r="H38" s="8" t="s">
-        <v>25</v>
+        <v>115</v>
       </c>
     </row>
     <row r="39" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B39" s="8" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>153</v>
-      </c>
-      <c r="D39" s="13"/>
+        <v>141</v>
+      </c>
+      <c r="D39" s="13" t="s">
+        <v>159</v>
+      </c>
       <c r="E39" s="8" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="F39" s="9">
-        <v>2.8</v>
+        <v>7</v>
       </c>
       <c r="G39" s="9"/>
-      <c r="H39" s="8"/>
+      <c r="H39" s="8" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="40" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B40" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>153</v>
-      </c>
-      <c r="D40" s="13" t="s">
-        <v>153</v>
-      </c>
+        <v>143</v>
+      </c>
+      <c r="D40" s="13"/>
       <c r="E40" s="8" t="s">
-        <v>145</v>
-      </c>
-      <c r="F40" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="G40" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="H40" s="8" t="s">
-        <v>58</v>
-      </c>
+        <v>134</v>
+      </c>
+      <c r="F40" s="9">
+        <v>2.8</v>
+      </c>
+      <c r="G40" s="9"/>
+      <c r="H40" s="8"/>
     </row>
     <row r="41" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B41" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="D41" s="13" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>145</v>
-      </c>
-      <c r="F41" s="9">
-        <v>2.8</v>
-      </c>
-      <c r="G41" s="9"/>
+        <v>135</v>
+      </c>
+      <c r="F41" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="G41" s="9" t="s">
+        <v>58</v>
+      </c>
       <c r="H41" s="8" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
     </row>
     <row r="42" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B42" s="8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="D42" s="13" t="s">
-        <v>154</v>
+        <v>141</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="F42" s="9">
         <v>2.8</v>
       </c>
       <c r="G42" s="9"/>
       <c r="H42" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="43" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B43" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C43" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="D43" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E43" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="F43" s="9">
+        <v>2.8</v>
+      </c>
+      <c r="G43" s="9"/>
+      <c r="H43" s="8" t="s">
         <v>54</v>
-      </c>
-    </row>
-    <row r="43" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B43" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="C43" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="D43" s="11"/>
-      <c r="E43" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="F43" s="6">
-        <v>1.4</v>
-      </c>
-      <c r="G43" s="6"/>
-      <c r="H43" s="5" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="44" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B44" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C44" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="D44" s="11" t="s">
-        <v>154</v>
-      </c>
+        <v>144</v>
+      </c>
+      <c r="D44" s="11"/>
       <c r="E44" s="5" t="s">
-        <v>145</v>
+        <v>134</v>
       </c>
       <c r="F44" s="6">
         <v>1.4</v>
       </c>
       <c r="G44" s="6"/>
       <c r="H44" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="45" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B45" s="5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C45" s="11" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="D45" s="11" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="F45" s="6">
-        <v>2.8</v>
+        <v>1.4</v>
       </c>
       <c r="G45" s="6"/>
       <c r="H45" s="5" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="46" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B46" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C46" s="11" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="D46" s="11" t="s">
-        <v>207</v>
+        <v>141</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="F46" s="6">
-        <v>3.4</v>
-      </c>
-      <c r="G46" s="6">
-        <v>60</v>
-      </c>
+        <v>2.8</v>
+      </c>
+      <c r="G46" s="6"/>
       <c r="H46" s="5" t="s">
-        <v>124</v>
+        <v>59</v>
       </c>
     </row>
     <row r="47" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B47" s="5" t="s">
-        <v>140</v>
+        <v>44</v>
       </c>
       <c r="C47" s="11" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>218</v>
+        <v>208</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
       <c r="F47" s="6">
-        <v>1</v>
+        <v>3.4</v>
       </c>
       <c r="G47" s="6">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="H47" s="5" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
     </row>
     <row r="48" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B48" s="5" t="s">
-        <v>17</v>
+        <v>130</v>
       </c>
       <c r="C48" s="11" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="D48" s="11" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="F48" s="6">
-        <v>5</v>
-      </c>
-      <c r="G48" s="6"/>
+        <v>1</v>
+      </c>
+      <c r="G48" s="6">
+        <v>30</v>
+      </c>
       <c r="H48" s="5" t="s">
-        <v>26</v>
+        <v>115</v>
       </c>
     </row>
     <row r="49" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B49" s="5" t="s">
-        <v>177</v>
+        <v>17</v>
       </c>
       <c r="C49" s="11" t="s">
-        <v>156</v>
-      </c>
-      <c r="D49" s="11"/>
+        <v>144</v>
+      </c>
+      <c r="D49" s="11" t="s">
+        <v>195</v>
+      </c>
       <c r="E49" s="5" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="F49" s="6">
-        <v>2.8</v>
+        <v>5</v>
       </c>
       <c r="G49" s="6"/>
-      <c r="H49" s="5"/>
+      <c r="H49" s="5" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="50" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B50" s="5" t="s">
-        <v>50</v>
+        <v>165</v>
       </c>
       <c r="C50" s="11" t="s">
-        <v>156</v>
-      </c>
-      <c r="D50" s="11" t="s">
-        <v>156</v>
-      </c>
+        <v>146</v>
+      </c>
+      <c r="D50" s="11"/>
       <c r="E50" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="F50" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="G50" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="H50" s="5" t="s">
-        <v>58</v>
-      </c>
+        <v>134</v>
+      </c>
+      <c r="F50" s="6">
+        <v>2.8</v>
+      </c>
+      <c r="G50" s="6"/>
+      <c r="H50" s="5"/>
     </row>
     <row r="51" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B51" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C51" s="11" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="F51" s="6">
-        <v>2.8</v>
-      </c>
-      <c r="G51" s="6"/>
+        <v>135</v>
+      </c>
+      <c r="F51" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="G51" s="6" t="s">
+        <v>58</v>
+      </c>
       <c r="H51" s="5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="52" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B52" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C52" s="11" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>154</v>
+        <v>141</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="F52" s="6">
         <v>2.8</v>
       </c>
       <c r="G52" s="6"/>
       <c r="H52" s="5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="53" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B53" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C53" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="D53" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="E53" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F53" s="6">
+        <v>2.8</v>
+      </c>
+      <c r="G53" s="6"/>
+      <c r="H53" s="5" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="53" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B53" s="22" t="s">
-        <v>203</v>
-      </c>
-      <c r="C53" s="18" t="s">
-        <v>199</v>
-      </c>
-      <c r="D53" s="23"/>
-      <c r="E53" s="22"/>
-      <c r="F53" s="24"/>
-      <c r="G53" s="24"/>
-      <c r="H53" s="22"/>
-    </row>
-    <row r="54" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B54" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="C54" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="D54" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="E54" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="F54" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="G54" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="H54" s="1" t="s">
-        <v>88</v>
-      </c>
+    <row r="54" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B54" s="22" t="s">
+        <v>189</v>
+      </c>
+      <c r="C54" s="18" t="s">
+        <v>185</v>
+      </c>
+      <c r="D54" s="23"/>
+      <c r="E54" s="22"/>
+      <c r="F54" s="24"/>
+      <c r="G54" s="24"/>
+      <c r="H54" s="22"/>
     </row>
     <row r="55" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B55" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="C55" s="13" t="s">
-        <v>157</v>
-      </c>
-      <c r="D55" s="13"/>
-      <c r="E55" s="8" t="s">
-        <v>144</v>
-      </c>
-      <c r="F55" s="9">
-        <v>1</v>
-      </c>
-      <c r="G55" s="9">
-        <v>30</v>
-      </c>
-      <c r="H55" s="8" t="s">
-        <v>91</v>
+      <c r="B55" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="F55" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="G55" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="H55" s="1" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="56" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B56" s="8" t="s">
-        <v>63</v>
+        <v>209</v>
       </c>
       <c r="C56" s="13" t="s">
-        <v>157</v>
-      </c>
-      <c r="D56" s="13" t="s">
-        <v>157</v>
-      </c>
+        <v>205</v>
+      </c>
+      <c r="D56" s="13"/>
       <c r="E56" s="8" t="s">
-        <v>145</v>
+        <v>134</v>
       </c>
       <c r="F56" s="9">
-        <v>1.2</v>
-      </c>
-      <c r="G56" s="9"/>
+        <v>1</v>
+      </c>
+      <c r="G56" s="9">
+        <v>30</v>
+      </c>
       <c r="H56" s="8" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
     </row>
     <row r="57" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B57" s="8" t="s">
-        <v>64</v>
+        <v>210</v>
       </c>
       <c r="C57" s="13" t="s">
-        <v>157</v>
+        <v>205</v>
       </c>
       <c r="D57" s="13" t="s">
-        <v>151</v>
+        <v>205</v>
       </c>
       <c r="E57" s="8" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="F57" s="9">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="G57" s="9"/>
       <c r="H57" s="8" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
     </row>
     <row r="58" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B58" s="8" t="s">
-        <v>65</v>
+        <v>211</v>
       </c>
       <c r="C58" s="13" t="s">
-        <v>157</v>
+        <v>205</v>
       </c>
       <c r="D58" s="13" t="s">
-        <v>154</v>
+        <v>141</v>
       </c>
       <c r="E58" s="8" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="F58" s="9">
         <v>0.4</v>
       </c>
       <c r="G58" s="9"/>
       <c r="H58" s="8" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
     </row>
     <row r="59" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B59" s="8" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="C59" s="13" t="s">
-        <v>152</v>
+        <v>205</v>
       </c>
       <c r="D59" s="13" t="s">
-        <v>157</v>
+        <v>144</v>
       </c>
       <c r="E59" s="8" t="s">
-        <v>208</v>
+        <v>135</v>
       </c>
       <c r="F59" s="9">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="G59" s="9"/>
       <c r="H59" s="8" t="s">
-        <v>211</v>
+        <v>87</v>
       </c>
     </row>
     <row r="60" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B60" s="8" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="C60" s="13" t="s">
-        <v>155</v>
+        <v>142</v>
       </c>
       <c r="D60" s="13" t="s">
-        <v>157</v>
+        <v>205</v>
       </c>
       <c r="E60" s="8" t="s">
-        <v>208</v>
+        <v>191</v>
       </c>
       <c r="F60" s="9">
         <v>1.2</v>
       </c>
       <c r="G60" s="9"/>
       <c r="H60" s="8" t="s">
-        <v>212</v>
+        <v>192</v>
       </c>
     </row>
     <row r="61" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B61" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="C61" s="11" t="s">
-        <v>158</v>
-      </c>
-      <c r="D61" s="11"/>
-      <c r="E61" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="F61" s="6">
-        <v>1</v>
-      </c>
-      <c r="G61" s="6"/>
-      <c r="H61" s="5" t="s">
-        <v>95</v>
+      <c r="B61" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="C61" s="13" t="s">
+        <v>145</v>
+      </c>
+      <c r="D61" s="13" t="s">
+        <v>205</v>
+      </c>
+      <c r="E61" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="F61" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="G61" s="9"/>
+      <c r="H61" s="8" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="62" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B62" s="5" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="C62" s="11" t="s">
-        <v>158</v>
-      </c>
-      <c r="D62" s="11" t="s">
-        <v>158</v>
-      </c>
+        <v>147</v>
+      </c>
+      <c r="D62" s="11"/>
       <c r="E62" s="5" t="s">
-        <v>145</v>
+        <v>134</v>
       </c>
       <c r="F62" s="6">
         <v>1</v>
       </c>
       <c r="G62" s="6"/>
       <c r="H62" s="5" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="63" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B63" s="5" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="C63" s="11" t="s">
-        <v>159</v>
-      </c>
-      <c r="D63" s="11"/>
+        <v>147</v>
+      </c>
+      <c r="D63" s="11" t="s">
+        <v>147</v>
+      </c>
       <c r="E63" s="5" t="s">
-        <v>174</v>
+        <v>135</v>
       </c>
       <c r="F63" s="6">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="G63" s="6"/>
       <c r="H63" s="5" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
     </row>
     <row r="64" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B64" s="5" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="C64" s="11" t="s">
-        <v>159</v>
-      </c>
-      <c r="D64" s="11" t="s">
-        <v>190</v>
-      </c>
+        <v>148</v>
+      </c>
+      <c r="D64" s="11"/>
       <c r="E64" s="5" t="s">
-        <v>147</v>
+        <v>162</v>
       </c>
       <c r="F64" s="6">
         <v>1.2</v>
       </c>
       <c r="G64" s="6"/>
       <c r="H64" s="5" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
     </row>
     <row r="65" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B65" s="5" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C65" s="11" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="D65" s="11" t="s">
-        <v>151</v>
+        <v>177</v>
       </c>
       <c r="E65" s="5" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="F65" s="6">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="G65" s="6"/>
       <c r="H65" s="5" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="66" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B66" s="5" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C66" s="11" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="D66" s="11" t="s">
-        <v>154</v>
+        <v>141</v>
       </c>
       <c r="E66" s="5" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="F66" s="6">
         <v>0.8</v>
       </c>
       <c r="G66" s="6"/>
       <c r="H66" s="5" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
     </row>
     <row r="67" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B67" s="5" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="C67" s="11" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="D67" s="11" t="s">
-        <v>178</v>
+        <v>144</v>
       </c>
       <c r="E67" s="5" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="F67" s="6">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="G67" s="6"/>
       <c r="H67" s="5" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
     </row>
     <row r="68" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B68" s="5" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C68" s="11" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="D68" s="11" t="s">
-        <v>157</v>
+        <v>215</v>
       </c>
       <c r="E68" s="5" t="s">
-        <v>147</v>
+        <v>135</v>
       </c>
       <c r="F68" s="6">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="G68" s="6"/>
       <c r="H68" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="69" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B69" s="22" t="s">
-        <v>203</v>
-      </c>
-      <c r="C69" s="18" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="69" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B69" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="C69" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="D69" s="11" t="s">
         <v>205</v>
       </c>
-      <c r="D69" s="23"/>
-      <c r="E69" s="22"/>
-      <c r="F69" s="24"/>
-      <c r="G69" s="24"/>
-      <c r="H69" s="22"/>
-    </row>
-    <row r="70" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B70" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="C70" s="16" t="s">
-        <v>175</v>
-      </c>
-      <c r="D70" s="16" t="s">
-        <v>176</v>
-      </c>
-      <c r="E70" s="15" t="s">
-        <v>143</v>
-      </c>
-      <c r="F70" s="17" t="s">
-        <v>170</v>
-      </c>
-      <c r="G70" s="17" t="s">
-        <v>132</v>
-      </c>
-      <c r="H70" s="15" t="s">
-        <v>88</v>
-      </c>
+      <c r="E69" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="F69" s="6">
+        <v>0.8</v>
+      </c>
+      <c r="G69" s="6"/>
+      <c r="H69" s="5" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="70" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B70" s="22" t="s">
+        <v>189</v>
+      </c>
+      <c r="C70" s="18" t="s">
+        <v>224</v>
+      </c>
+      <c r="D70" s="23"/>
+      <c r="E70" s="22"/>
+      <c r="F70" s="24"/>
+      <c r="G70" s="24"/>
+      <c r="H70" s="22"/>
     </row>
     <row r="71" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B71" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C71" s="13" t="s">
-        <v>220</v>
-      </c>
-      <c r="D71" s="13" t="s">
-        <v>224</v>
-      </c>
-      <c r="E71" s="8" t="s">
-        <v>146</v>
-      </c>
-      <c r="F71" s="9">
-        <v>2.8</v>
-      </c>
-      <c r="G71" s="9">
-        <v>20</v>
-      </c>
-      <c r="H71" s="8" t="s">
-        <v>124</v>
+      <c r="B71" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="C71" s="16" t="s">
+        <v>163</v>
+      </c>
+      <c r="D71" s="16" t="s">
+        <v>164</v>
+      </c>
+      <c r="E71" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="F71" s="17" t="s">
+        <v>158</v>
+      </c>
+      <c r="G71" s="17" t="s">
+        <v>123</v>
+      </c>
+      <c r="H71" s="15" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="72" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B72" s="8" t="s">
-        <v>125</v>
+        <v>20</v>
       </c>
       <c r="C72" s="13" t="s">
-        <v>220</v>
+        <v>198</v>
       </c>
       <c r="D72" s="13" t="s">
-        <v>221</v>
+        <v>202</v>
       </c>
       <c r="E72" s="8" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
       <c r="F72" s="9">
-        <v>13</v>
+        <v>2.8</v>
       </c>
       <c r="G72" s="9">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="H72" s="8" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
     </row>
     <row r="73" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B73" s="8" t="s">
-        <v>134</v>
+        <v>116</v>
       </c>
       <c r="C73" s="13" t="s">
-        <v>157</v>
+        <v>198</v>
       </c>
       <c r="D73" s="13" t="s">
-        <v>161</v>
+        <v>199</v>
       </c>
       <c r="E73" s="8" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="F73" s="9">
-        <v>1</v>
-      </c>
-      <c r="G73" s="9"/>
+        <v>13</v>
+      </c>
+      <c r="G73" s="9">
+        <v>100</v>
+      </c>
       <c r="H73" s="8" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
     </row>
     <row r="74" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B74" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="C74" s="13" t="s">
+        <v>205</v>
+      </c>
+      <c r="D74" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="E74" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="C74" s="13" t="s">
-        <v>162</v>
-      </c>
-      <c r="D74" s="13"/>
-      <c r="E74" s="8" t="s">
-        <v>144</v>
-      </c>
       <c r="F74" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G74" s="9"/>
       <c r="H74" s="8" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
     </row>
     <row r="75" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B75" s="8" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="C75" s="13" t="s">
-        <v>161</v>
-      </c>
-      <c r="D75" s="13" t="s">
-        <v>194</v>
-      </c>
+        <v>218</v>
+      </c>
+      <c r="D75" s="13"/>
       <c r="E75" s="8" t="s">
-        <v>193</v>
+        <v>134</v>
       </c>
       <c r="F75" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G75" s="9"/>
-      <c r="H75" s="8"/>
+      <c r="H75" s="8" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="76" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B76" s="8" t="s">
-        <v>65</v>
+        <v>122</v>
       </c>
       <c r="C76" s="13" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="D76" s="13" t="s">
-        <v>154</v>
+        <v>181</v>
       </c>
       <c r="E76" s="8" t="s">
-        <v>145</v>
-      </c>
-      <c r="F76" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="G76" s="9" t="s">
-        <v>58</v>
-      </c>
+        <v>180</v>
+      </c>
+      <c r="F76" s="9">
+        <v>1</v>
+      </c>
+      <c r="G76" s="9"/>
       <c r="H76" s="8"/>
     </row>
     <row r="77" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B77" s="8" t="s">
-        <v>89</v>
+        <v>212</v>
       </c>
       <c r="C77" s="13" t="s">
-        <v>161</v>
+        <v>218</v>
       </c>
       <c r="D77" s="13" t="s">
-        <v>162</v>
+        <v>144</v>
       </c>
       <c r="E77" s="8" t="s">
-        <v>179</v>
-      </c>
-      <c r="F77" s="9">
-        <v>0</v>
-      </c>
-      <c r="G77" s="9"/>
+        <v>135</v>
+      </c>
+      <c r="F77" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="G77" s="9" t="s">
+        <v>58</v>
+      </c>
       <c r="H77" s="8"/>
     </row>
     <row r="78" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B78" s="8" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="C78" s="13" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="D78" s="13" t="s">
-        <v>180</v>
-      </c>
-      <c r="E78" s="8"/>
+        <v>218</v>
+      </c>
+      <c r="E78" s="8" t="s">
+        <v>166</v>
+      </c>
       <c r="F78" s="9">
         <v>0</v>
       </c>
@@ -3346,594 +3356,611 @@
       <c r="H78" s="8"/>
     </row>
     <row r="79" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B79" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="C79" s="11" t="s">
-        <v>219</v>
-      </c>
-      <c r="D79" s="11" t="s">
-        <v>223</v>
-      </c>
-      <c r="E79" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="F79" s="6">
-        <v>4</v>
-      </c>
-      <c r="G79" s="6">
-        <v>20</v>
-      </c>
-      <c r="H79" s="5" t="s">
-        <v>124</v>
-      </c>
+      <c r="B79" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="C79" s="13" t="s">
+        <v>205</v>
+      </c>
+      <c r="D79" s="13" t="s">
+        <v>167</v>
+      </c>
+      <c r="E79" s="8"/>
+      <c r="F79" s="9">
+        <v>0</v>
+      </c>
+      <c r="G79" s="9"/>
+      <c r="H79" s="8"/>
     </row>
     <row r="80" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B80" s="5" t="s">
-        <v>214</v>
+        <v>225</v>
       </c>
       <c r="C80" s="11" t="s">
-        <v>219</v>
+        <v>197</v>
       </c>
       <c r="D80" s="11" t="s">
-        <v>222</v>
+        <v>201</v>
       </c>
       <c r="E80" s="5" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
       <c r="F80" s="6">
+        <v>4</v>
+      </c>
+      <c r="G80" s="6">
         <v>20</v>
       </c>
-      <c r="G80" s="6">
-        <v>100</v>
-      </c>
       <c r="H80" s="5" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
     </row>
     <row r="81" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B81" s="5" t="s">
-        <v>122</v>
+        <v>226</v>
       </c>
       <c r="C81" s="11" t="s">
-        <v>219</v>
+        <v>197</v>
       </c>
       <c r="D81" s="11" t="s">
-        <v>219</v>
+        <v>200</v>
       </c>
       <c r="E81" s="5" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="F81" s="6">
+        <v>20</v>
+      </c>
+      <c r="G81" s="6">
+        <v>100</v>
+      </c>
+      <c r="H81" s="5" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="82" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B82" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="C82" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="D82" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="E82" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F82" s="6">
         <v>2</v>
       </c>
-      <c r="G81" s="6"/>
-      <c r="H81" s="5" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="82" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B82" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="C82" s="13" t="s">
-        <v>163</v>
-      </c>
-      <c r="D82" s="13"/>
-      <c r="E82" s="8" t="s">
-        <v>144</v>
-      </c>
-      <c r="F82" s="9">
-        <v>1</v>
-      </c>
-      <c r="G82" s="9"/>
-      <c r="H82" s="8"/>
+      <c r="G82" s="6"/>
+      <c r="H82" s="5" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="83" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B83" s="8" t="s">
-        <v>127</v>
+        <v>117</v>
       </c>
       <c r="C83" s="13" t="s">
-        <v>181</v>
+        <v>151</v>
       </c>
       <c r="D83" s="13"/>
       <c r="E83" s="8" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
       <c r="F83" s="9">
         <v>1</v>
       </c>
-      <c r="G83" s="9">
-        <v>97.5</v>
-      </c>
-      <c r="H83" s="8" t="s">
-        <v>184</v>
-      </c>
+      <c r="G83" s="9"/>
+      <c r="H83" s="8"/>
     </row>
     <row r="84" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B84" s="8" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="C84" s="13" t="s">
-        <v>163</v>
-      </c>
-      <c r="D84" s="13" t="s">
-        <v>182</v>
-      </c>
+        <v>168</v>
+      </c>
+      <c r="D84" s="13"/>
       <c r="E84" s="8" t="s">
-        <v>147</v>
+        <v>136</v>
       </c>
       <c r="F84" s="9">
-        <v>1.5</v>
-      </c>
-      <c r="G84" s="9"/>
-      <c r="H84" s="8"/>
+        <v>1</v>
+      </c>
+      <c r="G84" s="9">
+        <v>97.5</v>
+      </c>
+      <c r="H84" s="8" t="s">
+        <v>171</v>
+      </c>
     </row>
     <row r="85" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B85" s="8" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="C85" s="13" t="s">
-        <v>163</v>
+        <v>151</v>
       </c>
       <c r="D85" s="13" t="s">
-        <v>183</v>
+        <v>169</v>
       </c>
       <c r="E85" s="8" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="F85" s="9">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="G85" s="9"/>
       <c r="H85" s="8"/>
     </row>
     <row r="86" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B86" s="8" t="s">
-        <v>74</v>
+        <v>120</v>
       </c>
       <c r="C86" s="13" t="s">
-        <v>164</v>
-      </c>
-      <c r="D86" s="13"/>
+        <v>151</v>
+      </c>
+      <c r="D86" s="13" t="s">
+        <v>170</v>
+      </c>
       <c r="E86" s="8" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="F86" s="9">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="G86" s="9"/>
-      <c r="H86" s="8" t="s">
-        <v>105</v>
-      </c>
+      <c r="H86" s="8"/>
     </row>
     <row r="87" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B87" s="8" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="C87" s="13" t="s">
-        <v>164</v>
-      </c>
-      <c r="D87" s="13" t="s">
-        <v>164</v>
-      </c>
+        <v>152</v>
+      </c>
+      <c r="D87" s="13"/>
       <c r="E87" s="8" t="s">
-        <v>145</v>
+        <v>134</v>
       </c>
       <c r="F87" s="9">
         <v>1.2</v>
       </c>
       <c r="G87" s="9"/>
       <c r="H87" s="8" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
     </row>
     <row r="88" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B88" s="8" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="C88" s="13" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="D88" s="13" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="E88" s="8" t="s">
-        <v>147</v>
+        <v>135</v>
       </c>
       <c r="F88" s="9">
-        <v>2.9</v>
+        <v>1.2</v>
       </c>
       <c r="G88" s="9"/>
       <c r="H88" s="8" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
     </row>
     <row r="89" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B89" s="8" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C89" s="13" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="D89" s="13" t="s">
-        <v>154</v>
+        <v>139</v>
       </c>
       <c r="E89" s="8" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="F89" s="9">
-        <v>1.2</v>
+        <v>2.9</v>
       </c>
       <c r="G89" s="9"/>
       <c r="H89" s="8" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="90" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B90" s="22" t="s">
-        <v>203</v>
-      </c>
-      <c r="C90" s="18" t="s">
-        <v>200</v>
-      </c>
-      <c r="D90" s="23"/>
-      <c r="E90" s="22"/>
-      <c r="F90" s="24"/>
-      <c r="G90" s="24"/>
-      <c r="H90" s="22"/>
-    </row>
-    <row r="91" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B91" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="C91" s="16" t="s">
-        <v>175</v>
-      </c>
-      <c r="D91" s="16" t="s">
-        <v>176</v>
-      </c>
-      <c r="E91" s="15" t="s">
-        <v>143</v>
-      </c>
-      <c r="F91" s="17" t="s">
-        <v>170</v>
-      </c>
-      <c r="G91" s="17" t="s">
-        <v>132</v>
-      </c>
-      <c r="H91" s="15" t="s">
-        <v>88</v>
-      </c>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="90" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B90" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="C90" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="D90" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E90" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="F90" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="G90" s="9"/>
+      <c r="H90" s="8" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="91" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B91" s="22" t="s">
+        <v>189</v>
+      </c>
+      <c r="C91" s="18" t="s">
+        <v>186</v>
+      </c>
+      <c r="D91" s="23"/>
+      <c r="E91" s="22"/>
+      <c r="F91" s="24"/>
+      <c r="G91" s="24"/>
+      <c r="H91" s="22"/>
     </row>
     <row r="92" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B92" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="C92" s="11" t="s">
-        <v>165</v>
-      </c>
-      <c r="D92" s="11"/>
-      <c r="E92" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="F92" s="6">
-        <v>1.8</v>
-      </c>
-      <c r="G92" s="6"/>
-      <c r="H92" s="5" t="s">
-        <v>109</v>
+      <c r="B92" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="C92" s="16" t="s">
+        <v>163</v>
+      </c>
+      <c r="D92" s="16" t="s">
+        <v>164</v>
+      </c>
+      <c r="E92" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="F92" s="17" t="s">
+        <v>158</v>
+      </c>
+      <c r="G92" s="17" t="s">
+        <v>123</v>
+      </c>
+      <c r="H92" s="15" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="93" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B93" s="5" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="C93" s="11" t="s">
-        <v>165</v>
-      </c>
-      <c r="D93" s="11" t="s">
-        <v>165</v>
-      </c>
+        <v>153</v>
+      </c>
+      <c r="D93" s="11"/>
       <c r="E93" s="5" t="s">
-        <v>145</v>
+        <v>134</v>
       </c>
       <c r="F93" s="6">
-        <v>1.4</v>
+        <v>1.8</v>
       </c>
       <c r="G93" s="6"/>
       <c r="H93" s="5" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
     </row>
     <row r="94" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B94" s="5" t="s">
-        <v>141</v>
+        <v>74</v>
       </c>
       <c r="C94" s="11" t="s">
-        <v>166</v>
+        <v>153</v>
       </c>
       <c r="D94" s="11" t="s">
-        <v>166</v>
+        <v>153</v>
       </c>
       <c r="E94" s="5" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="F94" s="6">
-        <v>10</v>
+        <v>1.4</v>
       </c>
       <c r="G94" s="6"/>
       <c r="H94" s="5" t="s">
-        <v>142</v>
+        <v>103</v>
       </c>
     </row>
     <row r="95" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B95" s="5" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="C95" s="11" t="s">
-        <v>165</v>
+        <v>154</v>
       </c>
       <c r="D95" s="11" t="s">
-        <v>217</v>
+        <v>154</v>
       </c>
       <c r="E95" s="5" t="s">
-        <v>160</v>
+        <v>135</v>
       </c>
       <c r="F95" s="6">
-        <v>0.8</v>
+        <v>10</v>
       </c>
       <c r="G95" s="6"/>
       <c r="H95" s="5" t="s">
-        <v>116</v>
+        <v>132</v>
       </c>
     </row>
     <row r="96" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B96" s="5" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="C96" s="11" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="D96" s="11" t="s">
-        <v>164</v>
+        <v>196</v>
       </c>
       <c r="E96" s="5" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="F96" s="6">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="G96" s="6"/>
       <c r="H96" s="5" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="97" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B97" s="5" t="s">
-        <v>192</v>
+        <v>128</v>
       </c>
       <c r="C97" s="11" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="D97" s="11" t="s">
-        <v>184</v>
+        <v>152</v>
       </c>
       <c r="E97" s="5" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="F97" s="6">
         <v>1.2</v>
       </c>
       <c r="G97" s="6"/>
       <c r="H97" s="5" t="s">
-        <v>191</v>
+        <v>101</v>
       </c>
     </row>
     <row r="98" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B98" s="5" t="s">
-        <v>133</v>
+        <v>179</v>
       </c>
       <c r="C98" s="11" t="s">
-        <v>167</v>
+        <v>153</v>
       </c>
       <c r="D98" s="11" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="E98" s="5" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="F98" s="6">
-        <v>2</v>
+        <v>1.2</v>
       </c>
       <c r="G98" s="6"/>
       <c r="H98" s="5" t="s">
-        <v>117</v>
+        <v>178</v>
       </c>
     </row>
     <row r="99" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B99" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="C99" s="13" t="s">
-        <v>168</v>
-      </c>
-      <c r="D99" s="13"/>
-      <c r="E99" s="8" t="s">
-        <v>174</v>
-      </c>
-      <c r="F99" s="9">
-        <v>1.4</v>
-      </c>
-      <c r="G99" s="9"/>
-      <c r="H99" s="8" t="s">
-        <v>111</v>
+      <c r="B99" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C99" s="11" t="s">
+        <v>155</v>
+      </c>
+      <c r="D99" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="E99" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F99" s="6">
+        <v>2</v>
+      </c>
+      <c r="G99" s="6"/>
+      <c r="H99" s="5" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="100" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B100" s="8" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="C100" s="13" t="s">
-        <v>168</v>
-      </c>
-      <c r="D100" s="13" t="s">
-        <v>168</v>
-      </c>
+        <v>156</v>
+      </c>
+      <c r="D100" s="13"/>
       <c r="E100" s="8" t="s">
-        <v>145</v>
+        <v>162</v>
       </c>
       <c r="F100" s="9">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="G100" s="9"/>
       <c r="H100" s="8" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
     </row>
     <row r="101" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B101" s="8" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="C101" s="13" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="D101" s="13" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
       <c r="E101" s="8" t="s">
-        <v>147</v>
+        <v>135</v>
       </c>
       <c r="F101" s="9">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="G101" s="9"/>
       <c r="H101" s="8" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
     </row>
     <row r="102" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B102" s="8" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="C102" s="13" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="D102" s="13" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="E102" s="8" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="F102" s="9">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="G102" s="9"/>
       <c r="H102" s="8" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
     </row>
     <row r="103" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B103" s="8" t="s">
-        <v>84</v>
+        <v>221</v>
       </c>
       <c r="C103" s="13" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="D103" s="13" t="s">
-        <v>158</v>
+        <v>205</v>
       </c>
       <c r="E103" s="8" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="F103" s="9">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="G103" s="9"/>
       <c r="H103" s="8" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
     </row>
     <row r="104" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B104" s="8" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="C104" s="13" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="D104" s="13" t="s">
-        <v>184</v>
+        <v>147</v>
       </c>
       <c r="E104" s="8" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="F104" s="9">
-        <v>1.4</v>
+        <v>1</v>
       </c>
       <c r="G104" s="9"/>
       <c r="H104" s="8" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
     </row>
     <row r="105" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B105" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="C105" s="11" t="s">
-        <v>169</v>
-      </c>
-      <c r="D105" s="11"/>
-      <c r="E105" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="F105" s="6">
-        <v>3</v>
-      </c>
-      <c r="G105" s="6"/>
-      <c r="H105" s="5" t="s">
+      <c r="B105" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="C105" s="13" t="s">
+        <v>156</v>
+      </c>
+      <c r="D105" s="13" t="s">
+        <v>171</v>
+      </c>
+      <c r="E105" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="F105" s="9">
+        <v>1.4</v>
+      </c>
+      <c r="G105" s="9"/>
+      <c r="H105" s="8" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="106" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B106" s="5" t="s">
-        <v>130</v>
+        <v>80</v>
       </c>
       <c r="C106" s="11" t="s">
-        <v>169</v>
-      </c>
-      <c r="D106" s="11" t="s">
-        <v>169</v>
-      </c>
+        <v>157</v>
+      </c>
+      <c r="D106" s="11"/>
       <c r="E106" s="5" t="s">
-        <v>145</v>
+        <v>134</v>
       </c>
       <c r="F106" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G106" s="6"/>
       <c r="H106" s="5" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
     </row>
     <row r="107" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B107" s="5" t="s">
-        <v>139</v>
+        <v>121</v>
       </c>
       <c r="C107" s="11" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="D107" s="11" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="E107" s="5" t="s">
-        <v>160</v>
+        <v>135</v>
       </c>
       <c r="F107" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G107" s="6"/>
       <c r="H107" s="5" t="s">
-        <v>115</v>
+        <v>107</v>
+      </c>
+    </row>
+    <row r="108" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B108" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="C108" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="D108" s="11" t="s">
+        <v>156</v>
+      </c>
+      <c r="E108" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="F108" s="6">
+        <v>1</v>
+      </c>
+      <c r="G108" s="6"/>
+      <c r="H108" s="5" t="s">
+        <v>108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
20260107: USE pin name for extracted.
</commit_message>
<xml_diff>
--- a/Document/TR-1um_Drawing_Layer_DR_Table.xlsx
+++ b/Document/TR-1um_Drawing_Layer_DR_Table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/okamura/Library/CloudStorage/Dropbox/91_OpenPDK/TR-1um/Document/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0D650A9-9EB4-984E-AA72-A3602D397E13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{359213D5-6771-1342-9B21-AB98D47C92BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1780" yWindow="760" windowWidth="29440" windowHeight="18880" xr2:uid="{7F1200E8-B51D-9446-A5CE-CEA05B5231B7}"/>
+    <workbookView xWindow="1760" yWindow="760" windowWidth="29440" windowHeight="18880" xr2:uid="{7F1200E8-B51D-9446-A5CE-CEA05B5231B7}"/>
   </bookViews>
   <sheets>
     <sheet name="TR-1um_Drawing_Layer_DR_Table" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="671" uniqueCount="291">
   <si>
     <t>WN.W1</t>
   </si>
@@ -720,6 +720,195 @@
   </si>
   <si>
     <t>GR.S1</t>
+  </si>
+  <si>
+    <t>ESD related</t>
+  </si>
+  <si>
+    <t>APE.WM</t>
+  </si>
+  <si>
+    <t>APE.LM</t>
+  </si>
+  <si>
+    <t>ANE.WM</t>
+  </si>
+  <si>
+    <t>ANE.LM</t>
+  </si>
+  <si>
+    <t>APE.AN</t>
+  </si>
+  <si>
+    <t>APE</t>
+  </si>
+  <si>
+    <t>APE.XY</t>
+  </si>
+  <si>
+    <t>ANE.AP</t>
+  </si>
+  <si>
+    <t>ANE.XY</t>
+  </si>
+  <si>
+    <t>ANE</t>
+  </si>
+  <si>
+    <t>COE.W1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CO(E) </t>
+  </si>
+  <si>
+    <t>COE.S1</t>
+  </si>
+  <si>
+    <t>CDE.GC</t>
+  </si>
+  <si>
+    <t>CD(E)</t>
+  </si>
+  <si>
+    <t>CSE.GC</t>
+  </si>
+  <si>
+    <t>CS(E)</t>
+  </si>
+  <si>
+    <t>ERMPE04/ERMNE08</t>
+  </si>
+  <si>
+    <t>ERMPE03/ERMNE09</t>
+  </si>
+  <si>
+    <t>COE.AP</t>
+  </si>
+  <si>
+    <t>ERMPE05/ERMPE31</t>
+  </si>
+  <si>
+    <t>COE.AN</t>
+  </si>
+  <si>
+    <t>ERMNE10/ERMNE32</t>
+  </si>
+  <si>
+    <t>APE.CO</t>
+  </si>
+  <si>
+    <t>ANE.CO</t>
+  </si>
+  <si>
+    <t>ERWLMN15</t>
+  </si>
+  <si>
+    <t>ERWLMPE16</t>
+  </si>
+  <si>
+    <t>ERMPE12/ERMNE13</t>
+  </si>
+  <si>
+    <t>ERMPE13/ERMNE15</t>
+  </si>
+  <si>
+    <t>ERMPE06</t>
+  </si>
+  <si>
+    <t>ERMNE15</t>
+  </si>
+  <si>
+    <t>ERWLMN14</t>
+  </si>
+  <si>
+    <t>ERWLMPE15</t>
+  </si>
+  <si>
+    <t>PAD related</t>
+  </si>
+  <si>
+    <t>PO.W1</t>
+  </si>
+  <si>
+    <t>PO</t>
+  </si>
+  <si>
+    <t>PO.S1</t>
+  </si>
+  <si>
+    <t>PO.M1</t>
+  </si>
+  <si>
+    <t>M1(P)</t>
+  </si>
+  <si>
+    <t>PO.M2</t>
+  </si>
+  <si>
+    <t>M2(P)</t>
+  </si>
+  <si>
+    <t>V1.M2</t>
+  </si>
+  <si>
+    <t>PO.AN</t>
+  </si>
+  <si>
+    <t>PO.AP</t>
+  </si>
+  <si>
+    <t>PO.GC</t>
+  </si>
+  <si>
+    <t>M2.PE</t>
+  </si>
+  <si>
+    <t>Extention</t>
+  </si>
+  <si>
+    <t>M2.PW</t>
+  </si>
+  <si>
+    <t>M1.PE</t>
+  </si>
+  <si>
+    <t>M1.PW</t>
+  </si>
+  <si>
+    <t>ER1809</t>
+  </si>
+  <si>
+    <t>ER1810</t>
+  </si>
+  <si>
+    <t>ER1703</t>
+  </si>
+  <si>
+    <t>ER1704</t>
+  </si>
+  <si>
+    <t>ER1801</t>
+  </si>
+  <si>
+    <t>ER1802</t>
+  </si>
+  <si>
+    <t>ER1808</t>
+  </si>
+  <si>
+    <t>ER1807</t>
+  </si>
+  <si>
+    <t>ER1811</t>
+  </si>
+  <si>
+    <t>ER1812</t>
+  </si>
+  <si>
+    <t>ER1803</t>
+  </si>
+  <si>
+    <t>ER1804</t>
   </si>
 </sst>
 </file>
@@ -764,7 +953,7 @@
       <family val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -792,6 +981,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD9D9D9"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.89999084444715716"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
@@ -823,7 +1018,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -895,6 +1090,18 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1777,7 +1984,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4478C0F2-BA21-8B4B-B7C2-220C0E7FA6A8}">
-  <dimension ref="B2:H108"/>
+  <dimension ref="B2:H143"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="19" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.6640625" style="4" customWidth="1"/>
@@ -3963,8 +4170,728 @@
         <v>108</v>
       </c>
     </row>
+    <row r="109" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B109" s="22" t="s">
+        <v>189</v>
+      </c>
+      <c r="C109" s="18" t="s">
+        <v>228</v>
+      </c>
+      <c r="D109" s="23"/>
+      <c r="E109" s="22"/>
+      <c r="F109" s="24"/>
+      <c r="G109" s="24"/>
+      <c r="H109" s="22"/>
+    </row>
+    <row r="110" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B110" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="C110" s="16" t="s">
+        <v>163</v>
+      </c>
+      <c r="D110" s="16" t="s">
+        <v>164</v>
+      </c>
+      <c r="E110" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="F110" s="17" t="s">
+        <v>158</v>
+      </c>
+      <c r="G110" s="17" t="s">
+        <v>123</v>
+      </c>
+      <c r="H110" s="15" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="111" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B111" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="C111" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="D111" s="13" t="s">
+        <v>206</v>
+      </c>
+      <c r="E111" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="F111" s="9">
+        <v>11</v>
+      </c>
+      <c r="G111" s="9">
+        <v>60</v>
+      </c>
+      <c r="H111" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="112" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B112" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="C112" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="D112" s="13" t="s">
+        <v>207</v>
+      </c>
+      <c r="E112" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="F112" s="9">
+        <v>2</v>
+      </c>
+      <c r="G112" s="9">
+        <v>30</v>
+      </c>
+      <c r="H112" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="113" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B113" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="C113" s="13" t="s">
+        <v>234</v>
+      </c>
+      <c r="D113" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E113" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="F113" s="9">
+        <v>10</v>
+      </c>
+      <c r="G113" s="9"/>
+      <c r="H113" s="8" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="114" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B114" s="8" t="s">
+        <v>235</v>
+      </c>
+      <c r="C114" s="13" t="s">
+        <v>234</v>
+      </c>
+      <c r="D114" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="E114" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="F114" s="9">
+        <v>1.4</v>
+      </c>
+      <c r="G114" s="9"/>
+      <c r="H114" s="8" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="115" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B115" s="8" t="s">
+        <v>252</v>
+      </c>
+      <c r="C115" s="13" t="s">
+        <v>234</v>
+      </c>
+      <c r="D115" s="13" t="s">
+        <v>147</v>
+      </c>
+      <c r="E115" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="F115" s="9">
+        <v>2</v>
+      </c>
+      <c r="G115" s="9"/>
+      <c r="H115" s="8" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="116" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B116" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="C116" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="D116" s="11" t="s">
+        <v>208</v>
+      </c>
+      <c r="E116" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="F116" s="6">
+        <v>11</v>
+      </c>
+      <c r="G116" s="6">
+        <v>60</v>
+      </c>
+      <c r="H116" s="5" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="117" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B117" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="C117" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="D117" s="11" t="s">
+        <v>207</v>
+      </c>
+      <c r="E117" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="F117" s="6">
+        <v>2</v>
+      </c>
+      <c r="G117" s="6">
+        <v>30</v>
+      </c>
+      <c r="H117" s="5" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="118" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B118" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="C118" s="11" t="s">
+        <v>238</v>
+      </c>
+      <c r="D118" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="E118" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F118" s="6">
+        <v>10</v>
+      </c>
+      <c r="G118" s="6"/>
+      <c r="H118" s="5" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="119" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B119" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="C119" s="11" t="s">
+        <v>238</v>
+      </c>
+      <c r="D119" s="11" t="s">
+        <v>181</v>
+      </c>
+      <c r="E119" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="F119" s="6">
+        <v>1.4</v>
+      </c>
+      <c r="G119" s="6"/>
+      <c r="H119" s="5" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="120" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B120" s="5" t="s">
+        <v>253</v>
+      </c>
+      <c r="C120" s="11" t="s">
+        <v>238</v>
+      </c>
+      <c r="D120" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="E120" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F120" s="6">
+        <v>2</v>
+      </c>
+      <c r="G120" s="6"/>
+      <c r="H120" s="5" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="121" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B121" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="C121" s="13" t="s">
+        <v>240</v>
+      </c>
+      <c r="D121" s="13"/>
+      <c r="E121" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="F121" s="9">
+        <v>3</v>
+      </c>
+      <c r="G121" s="9"/>
+      <c r="H121" s="8" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="122" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B122" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="C122" s="13" t="s">
+        <v>240</v>
+      </c>
+      <c r="D122" s="13"/>
+      <c r="E122" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="F122" s="9">
+        <v>1.6</v>
+      </c>
+      <c r="G122" s="9"/>
+      <c r="H122" s="8" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="123" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B123" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="C123" s="13" t="s">
+        <v>243</v>
+      </c>
+      <c r="D123" s="13" t="s">
+        <v>205</v>
+      </c>
+      <c r="E123" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="F123" s="9">
+        <v>7</v>
+      </c>
+      <c r="G123" s="9"/>
+      <c r="H123" s="8" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="124" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B124" s="8" t="s">
+        <v>244</v>
+      </c>
+      <c r="C124" s="13" t="s">
+        <v>245</v>
+      </c>
+      <c r="D124" s="13" t="s">
+        <v>205</v>
+      </c>
+      <c r="E124" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="F124" s="9">
+        <v>3</v>
+      </c>
+      <c r="G124" s="9"/>
+      <c r="H124" s="8" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="125" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B125" s="8" t="s">
+        <v>248</v>
+      </c>
+      <c r="C125" s="13" t="s">
+        <v>240</v>
+      </c>
+      <c r="D125" s="13" t="s">
+        <v>141</v>
+      </c>
+      <c r="E125" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="F125" s="9">
+        <v>4</v>
+      </c>
+      <c r="G125" s="9"/>
+      <c r="H125" s="8" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="126" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B126" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="C126" s="13" t="s">
+        <v>240</v>
+      </c>
+      <c r="D126" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E126" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="F126" s="9">
+        <v>4</v>
+      </c>
+      <c r="G126" s="9"/>
+      <c r="H126" s="8" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="127" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B127" s="22" t="s">
+        <v>189</v>
+      </c>
+      <c r="C127" s="18" t="s">
+        <v>262</v>
+      </c>
+      <c r="D127" s="23"/>
+      <c r="E127" s="22"/>
+      <c r="F127" s="24"/>
+      <c r="G127" s="24"/>
+      <c r="H127" s="22"/>
+    </row>
+    <row r="128" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B128" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="C128" s="16" t="s">
+        <v>163</v>
+      </c>
+      <c r="D128" s="16" t="s">
+        <v>164</v>
+      </c>
+      <c r="E128" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="F128" s="17" t="s">
+        <v>158</v>
+      </c>
+      <c r="G128" s="17" t="s">
+        <v>123</v>
+      </c>
+      <c r="H128" s="15" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="129" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B129" s="25" t="s">
+        <v>263</v>
+      </c>
+      <c r="C129" s="26" t="s">
+        <v>264</v>
+      </c>
+      <c r="D129" s="26"/>
+      <c r="E129" s="25" t="s">
+        <v>134</v>
+      </c>
+      <c r="F129" s="28">
+        <v>70</v>
+      </c>
+      <c r="G129" s="27"/>
+      <c r="H129" s="25" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="130" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B130" s="25" t="s">
+        <v>265</v>
+      </c>
+      <c r="C130" s="26" t="s">
+        <v>264</v>
+      </c>
+      <c r="D130" s="26"/>
+      <c r="E130" s="25" t="s">
+        <v>135</v>
+      </c>
+      <c r="F130" s="28">
+        <v>64</v>
+      </c>
+      <c r="G130" s="27"/>
+      <c r="H130" s="25" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="131" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B131" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="C131" s="11" t="s">
+        <v>264</v>
+      </c>
+      <c r="D131" s="11" t="s">
+        <v>269</v>
+      </c>
+      <c r="E131" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="F131" s="6">
+        <v>5</v>
+      </c>
+      <c r="G131" s="6"/>
+      <c r="H131" s="5" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="132" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B132" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="C132" s="11" t="s">
+        <v>264</v>
+      </c>
+      <c r="D132" s="11" t="s">
+        <v>267</v>
+      </c>
+      <c r="E132" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="F132" s="6">
+        <v>5</v>
+      </c>
+      <c r="G132" s="6"/>
+      <c r="H132" s="5" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="133" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B133" s="25" t="s">
+        <v>270</v>
+      </c>
+      <c r="C133" s="26" t="s">
+        <v>156</v>
+      </c>
+      <c r="D133" s="26" t="s">
+        <v>269</v>
+      </c>
+      <c r="E133" s="25" t="s">
+        <v>137</v>
+      </c>
+      <c r="F133" s="28">
+        <v>15</v>
+      </c>
+      <c r="G133" s="27"/>
+      <c r="H133" s="25" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="134" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B134" s="25" t="s">
+        <v>77</v>
+      </c>
+      <c r="C134" s="26" t="s">
+        <v>156</v>
+      </c>
+      <c r="D134" s="26" t="s">
+        <v>267</v>
+      </c>
+      <c r="E134" s="25" t="s">
+        <v>137</v>
+      </c>
+      <c r="F134" s="28">
+        <v>15</v>
+      </c>
+      <c r="G134" s="27"/>
+      <c r="H134" s="25" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="135" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B135" s="5" t="s">
+        <v>272</v>
+      </c>
+      <c r="C135" s="11" t="s">
+        <v>264</v>
+      </c>
+      <c r="D135" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="E135" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F135" s="6">
+        <v>14</v>
+      </c>
+      <c r="G135" s="6"/>
+      <c r="H135" s="5" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="136" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B136" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="C136" s="11" t="s">
+        <v>264</v>
+      </c>
+      <c r="D136" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="E136" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F136" s="6">
+        <v>14</v>
+      </c>
+      <c r="G136" s="6"/>
+      <c r="H136" s="5" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="137" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B137" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="C137" s="11" t="s">
+        <v>264</v>
+      </c>
+      <c r="D137" s="11" t="s">
+        <v>205</v>
+      </c>
+      <c r="E137" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F137" s="6">
+        <v>14</v>
+      </c>
+      <c r="G137" s="6"/>
+      <c r="H137" s="5" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="138" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B138" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="C138" s="11" t="s">
+        <v>264</v>
+      </c>
+      <c r="D138" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="E138" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F138" s="6">
+        <v>14</v>
+      </c>
+      <c r="G138" s="6"/>
+      <c r="H138" s="25" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="139" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B139" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="C139" s="11" t="s">
+        <v>264</v>
+      </c>
+      <c r="D139" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="E139" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F139" s="6">
+        <v>14</v>
+      </c>
+      <c r="G139" s="6"/>
+      <c r="H139" s="25" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="140" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B140" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="C140" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="D140" s="11" t="s">
+        <v>275</v>
+      </c>
+      <c r="E140" s="5"/>
+      <c r="F140" s="6">
+        <v>19</v>
+      </c>
+      <c r="G140" s="6"/>
+      <c r="H140" s="5" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="141" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B141" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="C141" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="D141" s="11" t="s">
+        <v>275</v>
+      </c>
+      <c r="E141" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="F141" s="6">
+        <v>40</v>
+      </c>
+      <c r="G141" s="6"/>
+      <c r="H141" s="5" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="142" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B142" s="5" t="s">
+        <v>277</v>
+      </c>
+      <c r="C142" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="D142" s="11" t="s">
+        <v>275</v>
+      </c>
+      <c r="E142" s="5"/>
+      <c r="F142" s="6">
+        <v>19</v>
+      </c>
+      <c r="G142" s="6"/>
+      <c r="H142" s="5" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="143" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B143" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="C143" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="D143" s="11" t="s">
+        <v>275</v>
+      </c>
+      <c r="E143" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="F143" s="6">
+        <v>40</v>
+      </c>
+      <c r="G143" s="6"/>
+      <c r="H143" s="5" t="s">
+        <v>290</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="50" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
20250107: Update DRC (ESD/PAD) document
</commit_message>
<xml_diff>
--- a/Document/TR-1um_Drawing_Layer_DR_Table.xlsx
+++ b/Document/TR-1um_Drawing_Layer_DR_Table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/okamura/Library/CloudStorage/Dropbox/91_OpenPDK/TR-1um/Document/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{359213D5-6771-1342-9B21-AB98D47C92BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E015A33D-DF6B-394F-A61F-B88E677DA75E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1760" yWindow="760" windowWidth="29440" windowHeight="18880" xr2:uid="{7F1200E8-B51D-9446-A5CE-CEA05B5231B7}"/>
+    <workbookView xWindow="800" yWindow="760" windowWidth="29440" windowHeight="18880" xr2:uid="{7F1200E8-B51D-9446-A5CE-CEA05B5231B7}"/>
   </bookViews>
   <sheets>
     <sheet name="TR-1um_Drawing_Layer_DR_Table" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="671" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="666" uniqueCount="292">
   <si>
     <t>WN.W1</t>
   </si>
@@ -848,9 +848,6 @@
     <t>M2(P)</t>
   </si>
   <si>
-    <t>V1.M2</t>
-  </si>
-  <si>
     <t>PO.AN</t>
   </si>
   <si>
@@ -899,16 +896,22 @@
     <t>ER1807</t>
   </si>
   <si>
-    <t>ER1811</t>
-  </si>
-  <si>
-    <t>ER1812</t>
-  </si>
-  <si>
     <t>ER1803</t>
   </si>
   <si>
     <t>ER1804</t>
+  </si>
+  <si>
+    <t>PO.V1</t>
+  </si>
+  <si>
+    <t>ER1811/ER1703</t>
+  </si>
+  <si>
+    <t>M2.PO</t>
+  </si>
+  <si>
+    <t>M1.PO</t>
   </si>
 </sst>
 </file>
@@ -1984,7 +1987,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4478C0F2-BA21-8B4B-B7C2-220C0E7FA6A8}">
-  <dimension ref="B2:H143"/>
+  <dimension ref="B2:H142"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="19" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.6640625" style="4" customWidth="1"/>
@@ -4598,7 +4601,7 @@
       </c>
       <c r="G129" s="27"/>
       <c r="H129" s="25" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="130" spans="2:8" ht="20" x14ac:dyDescent="0.2">
@@ -4617,102 +4620,102 @@
       </c>
       <c r="G130" s="27"/>
       <c r="H130" s="25" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="131" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B131" s="5" t="s">
-        <v>268</v>
+        <v>290</v>
       </c>
       <c r="C131" s="11" t="s">
+        <v>269</v>
+      </c>
+      <c r="D131" s="11" t="s">
         <v>264</v>
       </c>
-      <c r="D131" s="11" t="s">
-        <v>269</v>
-      </c>
       <c r="E131" s="5" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="F131" s="6">
         <v>5</v>
       </c>
       <c r="G131" s="6"/>
       <c r="H131" s="5" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="132" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B132" s="5" t="s">
-        <v>266</v>
+        <v>291</v>
       </c>
       <c r="C132" s="11" t="s">
+        <v>267</v>
+      </c>
+      <c r="D132" s="11" t="s">
         <v>264</v>
       </c>
-      <c r="D132" s="11" t="s">
-        <v>267</v>
-      </c>
       <c r="E132" s="5" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="F132" s="6">
         <v>5</v>
       </c>
       <c r="G132" s="6"/>
       <c r="H132" s="5" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="133" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B133" s="25" t="s">
-        <v>270</v>
+        <v>288</v>
       </c>
       <c r="C133" s="26" t="s">
+        <v>264</v>
+      </c>
+      <c r="D133" s="26" t="s">
         <v>156</v>
-      </c>
-      <c r="D133" s="26" t="s">
-        <v>269</v>
       </c>
       <c r="E133" s="25" t="s">
         <v>137</v>
       </c>
       <c r="F133" s="28">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G133" s="27"/>
       <c r="H133" s="25" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="134" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B134" s="25" t="s">
-        <v>77</v>
-      </c>
-      <c r="C134" s="26" t="s">
-        <v>156</v>
-      </c>
-      <c r="D134" s="26" t="s">
-        <v>267</v>
-      </c>
-      <c r="E134" s="25" t="s">
-        <v>137</v>
-      </c>
-      <c r="F134" s="28">
-        <v>15</v>
-      </c>
-      <c r="G134" s="27"/>
-      <c r="H134" s="25" t="s">
-        <v>288</v>
+      <c r="B134" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="C134" s="11" t="s">
+        <v>264</v>
+      </c>
+      <c r="D134" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="E134" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F134" s="6">
+        <v>14</v>
+      </c>
+      <c r="G134" s="6"/>
+      <c r="H134" s="5" t="s">
+        <v>284</v>
       </c>
     </row>
     <row r="135" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B135" s="5" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="C135" s="11" t="s">
         <v>264</v>
       </c>
       <c r="D135" s="11" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="E135" s="5" t="s">
         <v>135</v>
@@ -4722,18 +4725,18 @@
       </c>
       <c r="G135" s="6"/>
       <c r="H135" s="5" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="136" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B136" s="5" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C136" s="11" t="s">
         <v>264</v>
       </c>
       <c r="D136" s="11" t="s">
-        <v>144</v>
+        <v>205</v>
       </c>
       <c r="E136" s="5" t="s">
         <v>135</v>
@@ -4748,13 +4751,13 @@
     </row>
     <row r="137" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B137" s="5" t="s">
-        <v>273</v>
+        <v>266</v>
       </c>
       <c r="C137" s="11" t="s">
         <v>264</v>
       </c>
       <c r="D137" s="11" t="s">
-        <v>205</v>
+        <v>153</v>
       </c>
       <c r="E137" s="5" t="s">
         <v>135</v>
@@ -4763,19 +4766,19 @@
         <v>14</v>
       </c>
       <c r="G137" s="6"/>
-      <c r="H137" s="5" t="s">
-        <v>286</v>
+      <c r="H137" s="25" t="s">
+        <v>282</v>
       </c>
     </row>
     <row r="138" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B138" s="5" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C138" s="11" t="s">
         <v>264</v>
       </c>
       <c r="D138" s="11" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="E138" s="5" t="s">
         <v>135</v>
@@ -4790,42 +4793,42 @@
     </row>
     <row r="139" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B139" s="5" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="C139" s="11" t="s">
-        <v>264</v>
+        <v>157</v>
       </c>
       <c r="D139" s="11" t="s">
-        <v>157</v>
-      </c>
-      <c r="E139" s="5" t="s">
-        <v>135</v>
-      </c>
+        <v>274</v>
+      </c>
+      <c r="E139" s="5"/>
       <c r="F139" s="6">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="G139" s="6"/>
-      <c r="H139" s="25" t="s">
-        <v>284</v>
+      <c r="H139" s="5" t="s">
+        <v>286</v>
       </c>
     </row>
     <row r="140" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B140" s="5" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C140" s="11" t="s">
         <v>157</v>
       </c>
       <c r="D140" s="11" t="s">
-        <v>275</v>
-      </c>
-      <c r="E140" s="5"/>
+        <v>274</v>
+      </c>
+      <c r="E140" s="5" t="s">
+        <v>134</v>
+      </c>
       <c r="F140" s="6">
-        <v>19</v>
+        <v>40</v>
       </c>
       <c r="G140" s="6"/>
       <c r="H140" s="5" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
     </row>
     <row r="141" spans="2:8" ht="20" x14ac:dyDescent="0.2">
@@ -4836,17 +4839,15 @@
         <v>157</v>
       </c>
       <c r="D141" s="11" t="s">
-        <v>275</v>
-      </c>
-      <c r="E141" s="5" t="s">
-        <v>134</v>
-      </c>
+        <v>274</v>
+      </c>
+      <c r="E141" s="5"/>
       <c r="F141" s="6">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="G141" s="6"/>
       <c r="H141" s="5" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
     </row>
     <row r="142" spans="2:8" ht="20" x14ac:dyDescent="0.2">
@@ -4857,36 +4858,17 @@
         <v>157</v>
       </c>
       <c r="D142" s="11" t="s">
-        <v>275</v>
-      </c>
-      <c r="E142" s="5"/>
+        <v>274</v>
+      </c>
+      <c r="E142" s="5" t="s">
+        <v>134</v>
+      </c>
       <c r="F142" s="6">
-        <v>19</v>
+        <v>40</v>
       </c>
       <c r="G142" s="6"/>
       <c r="H142" s="5" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="143" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B143" s="5" t="s">
-        <v>278</v>
-      </c>
-      <c r="C143" s="11" t="s">
-        <v>157</v>
-      </c>
-      <c r="D143" s="11" t="s">
-        <v>275</v>
-      </c>
-      <c r="E143" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="F143" s="6">
-        <v>40</v>
-      </c>
-      <c r="G143" s="6"/>
-      <c r="H143" s="5" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
20250108: Update DRC (ESD/PAD)
</commit_message>
<xml_diff>
--- a/Document/TR-1um_Drawing_Layer_DR_Table.xlsx
+++ b/Document/TR-1um_Drawing_Layer_DR_Table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/okamura/Library/CloudStorage/Dropbox/91_OpenPDK/TR-1um/Document/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E015A33D-DF6B-394F-A61F-B88E677DA75E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE0B6A12-3D26-294A-97DB-4A7BD4673915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="800" yWindow="760" windowWidth="29440" windowHeight="18880" xr2:uid="{7F1200E8-B51D-9446-A5CE-CEA05B5231B7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="666" uniqueCount="292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="690" uniqueCount="306">
   <si>
     <t>WN.W1</t>
   </si>
@@ -704,9 +704,6 @@
     <t>V1.GC</t>
   </si>
   <si>
-    <t>GRohibited</t>
-  </si>
-  <si>
     <t>AA+GC+GR</t>
   </si>
   <si>
@@ -860,9 +857,6 @@
     <t>M2.PE</t>
   </si>
   <si>
-    <t>Extention</t>
-  </si>
-  <si>
     <t>M2.PW</t>
   </si>
   <si>
@@ -912,6 +906,54 @@
   </si>
   <si>
     <t>M1.PO</t>
+  </si>
+  <si>
+    <t>NMOSE</t>
+  </si>
+  <si>
+    <t>PMOSE</t>
+  </si>
+  <si>
+    <t>APE-GC</t>
+  </si>
+  <si>
+    <t>ANE-GC</t>
+  </si>
+  <si>
+    <t>GC-ANE</t>
+  </si>
+  <si>
+    <t>EXTW</t>
+  </si>
+  <si>
+    <t>EXTL</t>
+  </si>
+  <si>
+    <t>PO.Z1</t>
+  </si>
+  <si>
+    <t>PO.Z2</t>
+  </si>
+  <si>
+    <t>Electrical</t>
+  </si>
+  <si>
+    <t>ANT</t>
+  </si>
+  <si>
+    <t>Prohibited</t>
+  </si>
+  <si>
+    <t>PO.Z3</t>
+  </si>
+  <si>
+    <t>Exist</t>
+  </si>
+  <si>
+    <t>V1(P)</t>
+  </si>
+  <si>
+    <t>GC+GR</t>
   </si>
 </sst>
 </file>
@@ -1136,7 +1178,7 @@
     <xdr:to>
       <xdr:col>12</xdr:col>
       <xdr:colOff>636012</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>13</xdr:row>
       <xdr:rowOff>165275</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -1987,7 +2029,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4478C0F2-BA21-8B4B-B7C2-220C0E7FA6A8}">
-  <dimension ref="B2:H142"/>
+  <dimension ref="B2:H149"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="19" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.6640625" style="4" customWidth="1"/>
@@ -2005,7 +2047,7 @@
         <v>189</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>222</v>
+        <v>301</v>
       </c>
       <c r="D2" s="23"/>
       <c r="E2" s="22"/>
@@ -2082,7 +2124,7 @@
         <v>147</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>172</v>
@@ -2150,151 +2192,145 @@
       <c r="G9" s="6"/>
       <c r="H9" s="5"/>
     </row>
-    <row r="10" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B10" s="22" t="s">
-        <v>189</v>
-      </c>
-      <c r="C10" s="18" t="s">
-        <v>183</v>
-      </c>
-      <c r="D10" s="23"/>
-      <c r="E10" s="22"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="24"/>
-      <c r="H10" s="22"/>
+    <row r="10" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B10" s="5" t="s">
+        <v>297</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>263</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="F10" s="6">
+        <v>0</v>
+      </c>
+      <c r="G10" s="6"/>
+      <c r="H10" s="5"/>
     </row>
     <row r="11" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>82</v>
-      </c>
+      <c r="B11" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>263</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="F11" s="6">
+        <v>0</v>
+      </c>
+      <c r="G11" s="6"/>
+      <c r="H11" s="5"/>
     </row>
     <row r="12" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="5" t="s">
+        <v>302</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>263</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>304</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>303</v>
+      </c>
+      <c r="F12" s="6">
         <v>0</v>
       </c>
-      <c r="C12" s="11" t="s">
-        <v>159</v>
-      </c>
-      <c r="D12" s="11"/>
-      <c r="E12" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="F12" s="6">
-        <v>8</v>
-      </c>
       <c r="G12" s="6"/>
-      <c r="H12" s="5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C13" s="12" t="s">
-        <v>159</v>
-      </c>
-      <c r="D13" s="12" t="s">
-        <v>159</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="F13" s="6">
-        <v>12</v>
-      </c>
-      <c r="G13" s="6"/>
-      <c r="H13" s="5" t="s">
-        <v>10</v>
-      </c>
+      <c r="H12" s="5"/>
+    </row>
+    <row r="13" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B13" s="22" t="s">
+        <v>189</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>183</v>
+      </c>
+      <c r="D13" s="23"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="24"/>
+      <c r="G13" s="24"/>
+      <c r="H13" s="22"/>
     </row>
     <row r="14" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="C14" s="12" t="s">
-        <v>159</v>
-      </c>
-      <c r="D14" s="12" t="s">
-        <v>160</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="F14" s="6">
-        <v>9.5</v>
-      </c>
-      <c r="G14" s="6"/>
-      <c r="H14" s="7" t="s">
-        <v>12</v>
+      <c r="B14" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="15" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C15" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="C15" s="11" t="s">
         <v>159</v>
       </c>
-      <c r="D15" s="12" t="s">
-        <v>161</v>
-      </c>
+      <c r="D15" s="11"/>
       <c r="E15" s="5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F15" s="6">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G15" s="6"/>
-      <c r="H15" s="7" t="s">
-        <v>13</v>
+      <c r="H15" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="16" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="5" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>135</v>
       </c>
       <c r="F16" s="6">
-        <v>9.5</v>
+        <v>12</v>
       </c>
       <c r="G16" s="6"/>
-      <c r="H16" s="7" t="s">
-        <v>11</v>
+      <c r="H16" s="5" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="5" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D17" s="12" t="s">
         <v>160</v>
@@ -2303,19 +2339,19 @@
         <v>135</v>
       </c>
       <c r="F17" s="6">
-        <v>8</v>
+        <v>9.5</v>
       </c>
       <c r="G17" s="6"/>
       <c r="H17" s="7" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="18" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="5" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D18" s="12" t="s">
         <v>161</v>
@@ -2328,123 +2364,123 @@
       </c>
       <c r="G18" s="6"/>
       <c r="H18" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="5" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>141</v>
+        <v>161</v>
       </c>
       <c r="E19" s="5" t="s">
         <v>135</v>
       </c>
       <c r="F19" s="6">
-        <v>5</v>
+        <v>9.5</v>
       </c>
       <c r="G19" s="6"/>
       <c r="H19" s="7" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
     <row r="20" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>160</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>160</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F20" s="6">
         <v>8</v>
-      </c>
-      <c r="C20" s="12" t="s">
-        <v>159</v>
-      </c>
-      <c r="D20" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="F20" s="6">
-        <v>10</v>
       </c>
       <c r="G20" s="6"/>
       <c r="H20" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B21" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>161</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>161</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F21" s="6">
+        <v>12</v>
+      </c>
+      <c r="G21" s="6"/>
+      <c r="H21" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B22" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>159</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F22" s="6">
+        <v>5</v>
+      </c>
+      <c r="G22" s="6"/>
+      <c r="H22" s="7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="23" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B23" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>159</v>
+      </c>
+      <c r="D23" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F23" s="6">
+        <v>10</v>
+      </c>
+      <c r="G23" s="6"/>
+      <c r="H23" s="7" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="21" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="C21" s="13" t="s">
-        <v>138</v>
-      </c>
-      <c r="D21" s="13" t="s">
-        <v>150</v>
-      </c>
-      <c r="E21" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="F21" s="9">
-        <v>4</v>
-      </c>
-      <c r="G21" s="9"/>
-      <c r="H21" s="8" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="22" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C22" s="13" t="s">
-        <v>150</v>
-      </c>
-      <c r="D22" s="13" t="s">
-        <v>160</v>
-      </c>
-      <c r="E22" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="F22" s="9">
-        <v>10</v>
-      </c>
-      <c r="G22" s="9"/>
-      <c r="H22" s="8" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="23" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B23" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C23" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="D23" s="13" t="s">
-        <v>160</v>
-      </c>
-      <c r="E23" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="F23" s="9">
-        <v>5</v>
-      </c>
-      <c r="G23" s="9"/>
-      <c r="H23" s="8" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="24" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="8" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C24" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="D24" s="13" t="s">
         <v>150</v>
-      </c>
-      <c r="D24" s="13" t="s">
-        <v>144</v>
       </c>
       <c r="E24" s="8" t="s">
         <v>135</v>
@@ -2454,924 +2490,924 @@
       </c>
       <c r="G24" s="9"/>
       <c r="H24" s="8" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="25" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B25" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="D25" s="13" t="s">
+        <v>160</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="F25" s="9">
+        <v>10</v>
+      </c>
+      <c r="G25" s="9"/>
+      <c r="H25" s="8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="26" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B26" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="D26" s="13" t="s">
+        <v>160</v>
+      </c>
+      <c r="E26" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="F26" s="9">
+        <v>5</v>
+      </c>
+      <c r="G26" s="9"/>
+      <c r="H26" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="27" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B27" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="D27" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="F27" s="9">
+        <v>4</v>
+      </c>
+      <c r="G27" s="9"/>
+      <c r="H27" s="8" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="25" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C25" s="11" t="s">
-        <v>139</v>
-      </c>
-      <c r="D25" s="11"/>
-      <c r="E25" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="F25" s="6">
-        <v>28.5</v>
-      </c>
-      <c r="G25" s="6">
-        <v>120</v>
-      </c>
-      <c r="H25" s="5" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="26" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C26" s="11" t="s">
-        <v>139</v>
-      </c>
-      <c r="D26" s="11" t="s">
-        <v>139</v>
-      </c>
-      <c r="E26" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="F26" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="G26" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="H26" s="5"/>
-    </row>
-    <row r="27" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C27" s="11" t="s">
-        <v>139</v>
-      </c>
-      <c r="D27" s="11" t="s">
-        <v>161</v>
-      </c>
-      <c r="E27" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="F27" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="G27" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="H27" s="5"/>
     </row>
     <row r="28" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="5" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>144</v>
-      </c>
-      <c r="D28" s="11" t="s">
-        <v>161</v>
-      </c>
+        <v>139</v>
+      </c>
+      <c r="D28" s="11"/>
       <c r="E28" s="5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F28" s="6">
-        <v>3</v>
-      </c>
-      <c r="G28" s="6"/>
+        <v>28.5</v>
+      </c>
+      <c r="G28" s="6">
+        <v>120</v>
+      </c>
       <c r="H28" s="5" t="s">
-        <v>36</v>
+        <v>115</v>
       </c>
     </row>
     <row r="29" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="5" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C29" s="11" t="s">
         <v>139</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="E29" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="F29" s="6">
-        <v>2.8</v>
-      </c>
-      <c r="G29" s="6"/>
-      <c r="H29" s="5" t="s">
-        <v>37</v>
-      </c>
+      <c r="F29" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="G29" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="H29" s="5"/>
     </row>
     <row r="30" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="5" t="s">
-        <v>204</v>
+        <v>33</v>
       </c>
       <c r="C30" s="11" t="s">
         <v>139</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>205</v>
+        <v>161</v>
       </c>
       <c r="E30" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="F30" s="6">
-        <v>1.4</v>
-      </c>
-      <c r="G30" s="6"/>
-      <c r="H30" s="5" t="s">
-        <v>203</v>
-      </c>
+      <c r="F30" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="G30" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="H30" s="5"/>
     </row>
     <row r="31" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C31" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="D31" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="F31" s="6">
+        <v>3</v>
+      </c>
+      <c r="G31" s="6"/>
+      <c r="H31" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="32" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B32" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C32" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="D32" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F32" s="6">
+        <v>2.8</v>
+      </c>
+      <c r="G32" s="6"/>
+      <c r="H32" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="33" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B33" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="C33" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="D33" s="11" t="s">
+        <v>205</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="F33" s="6">
+        <v>1.4</v>
+      </c>
+      <c r="G33" s="6"/>
+      <c r="H33" s="5" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="34" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B34" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="C31" s="11" t="s">
+      <c r="C34" s="11" t="s">
         <v>139</v>
       </c>
-      <c r="D31" s="11" t="s">
+      <c r="D34" s="11" t="s">
         <v>194</v>
       </c>
-      <c r="E31" s="5" t="s">
+      <c r="E34" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="F31" s="6">
+      <c r="F34" s="6">
         <v>0</v>
       </c>
-      <c r="G31" s="6"/>
-      <c r="H31" s="5"/>
-    </row>
-    <row r="32" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B32" s="22" t="s">
+      <c r="G34" s="6"/>
+      <c r="H34" s="5"/>
+    </row>
+    <row r="35" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B35" s="22" t="s">
         <v>189</v>
       </c>
-      <c r="C32" s="18" t="s">
+      <c r="C35" s="18" t="s">
         <v>184</v>
       </c>
-      <c r="D32" s="23"/>
-      <c r="E32" s="22"/>
-      <c r="F32" s="24"/>
-      <c r="G32" s="24"/>
-      <c r="H32" s="22"/>
-    </row>
-    <row r="33" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B33" s="1" t="s">
+      <c r="D35" s="23"/>
+      <c r="E35" s="22"/>
+      <c r="F35" s="24"/>
+      <c r="G35" s="24"/>
+      <c r="H35" s="22"/>
+    </row>
+    <row r="36" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B36" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="C33" s="2" t="s">
+      <c r="C36" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="D33" s="2" t="s">
+      <c r="D36" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="E33" s="1" t="s">
+      <c r="E36" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="F33" s="3" t="s">
+      <c r="F36" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="G33" s="3" t="s">
+      <c r="G36" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="H33" s="1" t="s">
+      <c r="H36" s="1" t="s">
         <v>82</v>
-      </c>
-    </row>
-    <row r="34" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B34" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="C34" s="13" t="s">
-        <v>141</v>
-      </c>
-      <c r="D34" s="13"/>
-      <c r="E34" s="8" t="s">
-        <v>134</v>
-      </c>
-      <c r="F34" s="9">
-        <v>1.4</v>
-      </c>
-      <c r="G34" s="9"/>
-      <c r="H34" s="8" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="35" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B35" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="C35" s="13" t="s">
-        <v>141</v>
-      </c>
-      <c r="D35" s="13" t="s">
-        <v>141</v>
-      </c>
-      <c r="E35" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="F35" s="9">
-        <v>1.4</v>
-      </c>
-      <c r="G35" s="9"/>
-      <c r="H35" s="8" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="36" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B36" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="C36" s="13" t="s">
-        <v>141</v>
-      </c>
-      <c r="D36" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E36" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="F36" s="9">
-        <v>2.8</v>
-      </c>
-      <c r="G36" s="9"/>
-      <c r="H36" s="8" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="37" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B37" s="8" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>142</v>
-      </c>
-      <c r="D37" s="13" t="s">
-        <v>206</v>
-      </c>
+        <v>141</v>
+      </c>
+      <c r="D37" s="13"/>
       <c r="E37" s="8" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F37" s="9">
-        <v>3.4</v>
-      </c>
-      <c r="G37" s="9">
-        <v>60</v>
-      </c>
+        <v>1.4</v>
+      </c>
+      <c r="G37" s="9"/>
       <c r="H37" s="8" t="s">
-        <v>115</v>
+        <v>56</v>
       </c>
     </row>
     <row r="38" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B38" s="8" t="s">
-        <v>126</v>
+        <v>39</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D38" s="13" t="s">
-        <v>207</v>
+        <v>141</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="F38" s="9">
-        <v>1</v>
-      </c>
-      <c r="G38" s="9">
-        <v>30</v>
-      </c>
+        <v>1.4</v>
+      </c>
+      <c r="G38" s="9"/>
       <c r="H38" s="8" t="s">
-        <v>115</v>
+        <v>55</v>
       </c>
     </row>
     <row r="39" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B39" s="8" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="C39" s="13" t="s">
         <v>141</v>
       </c>
       <c r="D39" s="13" t="s">
-        <v>159</v>
+        <v>144</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F39" s="9">
-        <v>7</v>
+        <v>2.8</v>
       </c>
       <c r="G39" s="9"/>
       <c r="H39" s="8" t="s">
-        <v>25</v>
+        <v>57</v>
       </c>
     </row>
     <row r="40" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B40" s="8" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>143</v>
-      </c>
-      <c r="D40" s="13"/>
+        <v>142</v>
+      </c>
+      <c r="D40" s="13" t="s">
+        <v>206</v>
+      </c>
       <c r="E40" s="8" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F40" s="9">
-        <v>2.8</v>
-      </c>
-      <c r="G40" s="9"/>
-      <c r="H40" s="8"/>
+        <v>3.4</v>
+      </c>
+      <c r="G40" s="9">
+        <v>60</v>
+      </c>
+      <c r="H40" s="8" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="41" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B41" s="8" t="s">
-        <v>47</v>
+        <v>126</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D41" s="13" t="s">
-        <v>143</v>
+        <v>207</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="F41" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="G41" s="9" t="s">
-        <v>58</v>
+        <v>140</v>
+      </c>
+      <c r="F41" s="9">
+        <v>1</v>
+      </c>
+      <c r="G41" s="9">
+        <v>30</v>
       </c>
       <c r="H41" s="8" t="s">
-        <v>58</v>
+        <v>115</v>
       </c>
     </row>
     <row r="42" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B42" s="8" t="s">
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D42" s="13" t="s">
-        <v>141</v>
+        <v>159</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F42" s="9">
-        <v>2.8</v>
+        <v>7</v>
       </c>
       <c r="G42" s="9"/>
       <c r="H42" s="8" t="s">
-        <v>53</v>
+        <v>25</v>
       </c>
     </row>
     <row r="43" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B43" s="8" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C43" s="13" t="s">
         <v>143</v>
       </c>
-      <c r="D43" s="13" t="s">
-        <v>144</v>
-      </c>
+      <c r="D43" s="13"/>
       <c r="E43" s="8" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F43" s="9">
         <v>2.8</v>
       </c>
       <c r="G43" s="9"/>
-      <c r="H43" s="8" t="s">
+      <c r="H43" s="8"/>
+    </row>
+    <row r="44" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B44" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C44" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="D44" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="E44" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="F44" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="G44" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="H44" s="8" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="45" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B45" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C45" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="D45" s="13" t="s">
+        <v>141</v>
+      </c>
+      <c r="E45" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="F45" s="9">
+        <v>2.8</v>
+      </c>
+      <c r="G45" s="9"/>
+      <c r="H45" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="46" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B46" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C46" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="D46" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E46" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="F46" s="9">
+        <v>2.8</v>
+      </c>
+      <c r="G46" s="9"/>
+      <c r="H46" s="8" t="s">
         <v>54</v>
-      </c>
-    </row>
-    <row r="44" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B44" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="C44" s="11" t="s">
-        <v>144</v>
-      </c>
-      <c r="D44" s="11"/>
-      <c r="E44" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="F44" s="6">
-        <v>1.4</v>
-      </c>
-      <c r="G44" s="6"/>
-      <c r="H44" s="5" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="45" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B45" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="C45" s="11" t="s">
-        <v>144</v>
-      </c>
-      <c r="D45" s="11" t="s">
-        <v>144</v>
-      </c>
-      <c r="E45" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="F45" s="6">
-        <v>1.4</v>
-      </c>
-      <c r="G45" s="6"/>
-      <c r="H45" s="5" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="46" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B46" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="C46" s="11" t="s">
-        <v>144</v>
-      </c>
-      <c r="D46" s="11" t="s">
-        <v>141</v>
-      </c>
-      <c r="E46" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="F46" s="6">
-        <v>2.8</v>
-      </c>
-      <c r="G46" s="6"/>
-      <c r="H46" s="5" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="47" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B47" s="5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C47" s="11" t="s">
-        <v>145</v>
-      </c>
-      <c r="D47" s="11" t="s">
-        <v>208</v>
-      </c>
+        <v>144</v>
+      </c>
+      <c r="D47" s="11"/>
       <c r="E47" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F47" s="6">
-        <v>3.4</v>
-      </c>
-      <c r="G47" s="6">
-        <v>60</v>
-      </c>
+        <v>1.4</v>
+      </c>
+      <c r="G47" s="6"/>
       <c r="H47" s="5" t="s">
-        <v>115</v>
+        <v>56</v>
       </c>
     </row>
     <row r="48" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B48" s="5" t="s">
-        <v>130</v>
+        <v>43</v>
       </c>
       <c r="C48" s="11" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D48" s="11" t="s">
-        <v>207</v>
+        <v>144</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="F48" s="6">
-        <v>1</v>
-      </c>
-      <c r="G48" s="6">
-        <v>30</v>
-      </c>
+        <v>1.4</v>
+      </c>
+      <c r="G48" s="6"/>
       <c r="H48" s="5" t="s">
-        <v>115</v>
+        <v>55</v>
       </c>
     </row>
     <row r="49" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B49" s="5" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="C49" s="11" t="s">
         <v>144</v>
       </c>
       <c r="D49" s="11" t="s">
-        <v>195</v>
+        <v>141</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F49" s="6">
-        <v>5</v>
+        <v>2.8</v>
       </c>
       <c r="G49" s="6"/>
       <c r="H49" s="5" t="s">
-        <v>26</v>
+        <v>59</v>
       </c>
     </row>
     <row r="50" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B50" s="5" t="s">
-        <v>165</v>
+        <v>44</v>
       </c>
       <c r="C50" s="11" t="s">
-        <v>146</v>
-      </c>
-      <c r="D50" s="11"/>
+        <v>145</v>
+      </c>
+      <c r="D50" s="11" t="s">
+        <v>208</v>
+      </c>
       <c r="E50" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F50" s="6">
-        <v>2.8</v>
-      </c>
-      <c r="G50" s="6"/>
-      <c r="H50" s="5"/>
+        <v>3.4</v>
+      </c>
+      <c r="G50" s="6">
+        <v>60</v>
+      </c>
+      <c r="H50" s="5" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="51" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B51" s="5" t="s">
-        <v>50</v>
+        <v>130</v>
       </c>
       <c r="C51" s="11" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>146</v>
+        <v>207</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="F51" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="G51" s="6" t="s">
-        <v>58</v>
+        <v>140</v>
+      </c>
+      <c r="F51" s="6">
+        <v>1</v>
+      </c>
+      <c r="G51" s="6">
+        <v>30</v>
       </c>
       <c r="H51" s="5" t="s">
-        <v>58</v>
+        <v>115</v>
       </c>
     </row>
     <row r="52" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B52" s="5" t="s">
-        <v>51</v>
+        <v>17</v>
       </c>
       <c r="C52" s="11" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>141</v>
+        <v>195</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F52" s="6">
-        <v>2.8</v>
+        <v>5</v>
       </c>
       <c r="G52" s="6"/>
       <c r="H52" s="5" t="s">
-        <v>60</v>
+        <v>26</v>
       </c>
     </row>
     <row r="53" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B53" s="5" t="s">
-        <v>52</v>
+        <v>165</v>
       </c>
       <c r="C53" s="11" t="s">
         <v>146</v>
       </c>
-      <c r="D53" s="11" t="s">
-        <v>144</v>
-      </c>
+      <c r="D53" s="11"/>
       <c r="E53" s="5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F53" s="6">
         <v>2.8</v>
       </c>
       <c r="G53" s="6"/>
-      <c r="H53" s="5" t="s">
+      <c r="H53" s="5"/>
+    </row>
+    <row r="54" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B54" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C54" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="D54" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="E54" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F54" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="G54" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="H54" s="5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="55" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B55" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C55" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="D55" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="E55" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F55" s="6">
+        <v>2.8</v>
+      </c>
+      <c r="G55" s="6"/>
+      <c r="H55" s="5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="56" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B56" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C56" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="D56" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="E56" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F56" s="6">
+        <v>2.8</v>
+      </c>
+      <c r="G56" s="6"/>
+      <c r="H56" s="5" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="54" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B54" s="22" t="s">
+    <row r="57" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B57" s="22" t="s">
         <v>189</v>
       </c>
-      <c r="C54" s="18" t="s">
+      <c r="C57" s="18" t="s">
         <v>185</v>
       </c>
-      <c r="D54" s="23"/>
-      <c r="E54" s="22"/>
-      <c r="F54" s="24"/>
-      <c r="G54" s="24"/>
-      <c r="H54" s="22"/>
-    </row>
-    <row r="55" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B55" s="1" t="s">
+      <c r="D57" s="23"/>
+      <c r="E57" s="22"/>
+      <c r="F57" s="24"/>
+      <c r="G57" s="24"/>
+      <c r="H57" s="22"/>
+    </row>
+    <row r="58" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B58" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="C55" s="2" t="s">
+      <c r="C58" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="D55" s="2" t="s">
+      <c r="D58" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="E55" s="1" t="s">
+      <c r="E58" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="F55" s="3" t="s">
+      <c r="F58" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="G55" s="3" t="s">
+      <c r="G58" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="H55" s="1" t="s">
+      <c r="H58" s="1" t="s">
         <v>82</v>
-      </c>
-    </row>
-    <row r="56" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B56" s="8" t="s">
-        <v>209</v>
-      </c>
-      <c r="C56" s="13" t="s">
-        <v>205</v>
-      </c>
-      <c r="D56" s="13"/>
-      <c r="E56" s="8" t="s">
-        <v>134</v>
-      </c>
-      <c r="F56" s="9">
-        <v>1</v>
-      </c>
-      <c r="G56" s="9">
-        <v>30</v>
-      </c>
-      <c r="H56" s="8" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="57" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B57" s="8" t="s">
-        <v>210</v>
-      </c>
-      <c r="C57" s="13" t="s">
-        <v>205</v>
-      </c>
-      <c r="D57" s="13" t="s">
-        <v>205</v>
-      </c>
-      <c r="E57" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="F57" s="9">
-        <v>1.2</v>
-      </c>
-      <c r="G57" s="9"/>
-      <c r="H57" s="8" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="58" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B58" s="8" t="s">
-        <v>211</v>
-      </c>
-      <c r="C58" s="13" t="s">
-        <v>205</v>
-      </c>
-      <c r="D58" s="13" t="s">
-        <v>141</v>
-      </c>
-      <c r="E58" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="F58" s="9">
-        <v>0.4</v>
-      </c>
-      <c r="G58" s="9"/>
-      <c r="H58" s="8" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="59" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B59" s="8" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C59" s="13" t="s">
         <v>205</v>
       </c>
-      <c r="D59" s="13" t="s">
-        <v>144</v>
-      </c>
+      <c r="D59" s="13"/>
       <c r="E59" s="8" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F59" s="9">
-        <v>0.4</v>
-      </c>
-      <c r="G59" s="9"/>
+        <v>1</v>
+      </c>
+      <c r="G59" s="9">
+        <v>30</v>
+      </c>
       <c r="H59" s="8" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="60" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B60" s="8" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C60" s="13" t="s">
-        <v>142</v>
+        <v>205</v>
       </c>
       <c r="D60" s="13" t="s">
         <v>205</v>
       </c>
       <c r="E60" s="8" t="s">
-        <v>191</v>
+        <v>135</v>
       </c>
       <c r="F60" s="9">
         <v>1.2</v>
       </c>
       <c r="G60" s="9"/>
       <c r="H60" s="8" t="s">
-        <v>192</v>
+        <v>85</v>
       </c>
     </row>
     <row r="61" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B61" s="8" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C61" s="13" t="s">
-        <v>145</v>
+        <v>205</v>
       </c>
       <c r="D61" s="13" t="s">
-        <v>205</v>
+        <v>141</v>
       </c>
       <c r="E61" s="8" t="s">
-        <v>191</v>
+        <v>135</v>
       </c>
       <c r="F61" s="9">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="G61" s="9"/>
       <c r="H61" s="8" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="62" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B62" s="8" t="s">
+        <v>212</v>
+      </c>
+      <c r="C62" s="13" t="s">
+        <v>205</v>
+      </c>
+      <c r="D62" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E62" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="F62" s="9">
+        <v>0.4</v>
+      </c>
+      <c r="G62" s="9"/>
+      <c r="H62" s="8" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="63" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B63" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="C63" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="D63" s="13" t="s">
+        <v>205</v>
+      </c>
+      <c r="E63" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="F63" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="G63" s="9"/>
+      <c r="H63" s="8" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="64" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B64" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="C64" s="13" t="s">
+        <v>145</v>
+      </c>
+      <c r="D64" s="13" t="s">
+        <v>205</v>
+      </c>
+      <c r="E64" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="F64" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="G64" s="9"/>
+      <c r="H64" s="8" t="s">
         <v>193</v>
-      </c>
-    </row>
-    <row r="62" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B62" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="C62" s="11" t="s">
-        <v>147</v>
-      </c>
-      <c r="D62" s="11"/>
-      <c r="E62" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="F62" s="6">
-        <v>1</v>
-      </c>
-      <c r="G62" s="6"/>
-      <c r="H62" s="5" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="63" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B63" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="C63" s="11" t="s">
-        <v>147</v>
-      </c>
-      <c r="D63" s="11" t="s">
-        <v>147</v>
-      </c>
-      <c r="E63" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="F63" s="6">
-        <v>1</v>
-      </c>
-      <c r="G63" s="6"/>
-      <c r="H63" s="5" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="64" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B64" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="C64" s="11" t="s">
-        <v>148</v>
-      </c>
-      <c r="D64" s="11"/>
-      <c r="E64" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="F64" s="6">
-        <v>1.2</v>
-      </c>
-      <c r="G64" s="6"/>
-      <c r="H64" s="5" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="65" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B65" s="5" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="C65" s="11" t="s">
-        <v>148</v>
-      </c>
-      <c r="D65" s="11" t="s">
-        <v>177</v>
-      </c>
+        <v>147</v>
+      </c>
+      <c r="D65" s="11"/>
       <c r="E65" s="5" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="F65" s="6">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="G65" s="6"/>
       <c r="H65" s="5" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
     </row>
     <row r="66" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B66" s="5" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C66" s="11" t="s">
         <v>147</v>
       </c>
       <c r="D66" s="11" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="E66" s="5" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F66" s="6">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="G66" s="6"/>
       <c r="H66" s="5" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="67" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B67" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C67" s="11" t="s">
-        <v>147</v>
-      </c>
-      <c r="D67" s="11" t="s">
-        <v>144</v>
-      </c>
+        <v>148</v>
+      </c>
+      <c r="D67" s="11"/>
       <c r="E67" s="5" t="s">
-        <v>137</v>
+        <v>162</v>
       </c>
       <c r="F67" s="6">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="G67" s="6"/>
       <c r="H67" s="5" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="68" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B68" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C68" s="11" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D68" s="11" t="s">
-        <v>215</v>
+        <v>177</v>
       </c>
       <c r="E68" s="5" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F68" s="6">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="G68" s="6"/>
       <c r="H68" s="5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="69" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B69" s="5" t="s">
-        <v>216</v>
+        <v>66</v>
       </c>
       <c r="C69" s="11" t="s">
         <v>147</v>
       </c>
       <c r="D69" s="11" t="s">
-        <v>205</v>
+        <v>141</v>
       </c>
       <c r="E69" s="5" t="s">
         <v>137</v>
@@ -3381,343 +3417,347 @@
       </c>
       <c r="G69" s="6"/>
       <c r="H69" s="5" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="70" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B70" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C70" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="D70" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="E70" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="F70" s="6">
+        <v>0.8</v>
+      </c>
+      <c r="G70" s="6"/>
+      <c r="H70" s="5" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="71" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B71" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C71" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="D71" s="11" t="s">
+        <v>215</v>
+      </c>
+      <c r="E71" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F71" s="6">
+        <v>1</v>
+      </c>
+      <c r="G71" s="6"/>
+      <c r="H71" s="5" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="72" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B72" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="C72" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="D72" s="11" t="s">
+        <v>305</v>
+      </c>
+      <c r="E72" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="F72" s="6">
+        <v>0.8</v>
+      </c>
+      <c r="G72" s="6"/>
+      <c r="H72" s="5" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="70" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B70" s="22" t="s">
+    <row r="73" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B73" s="22" t="s">
         <v>189</v>
       </c>
-      <c r="C70" s="18" t="s">
-        <v>224</v>
-      </c>
-      <c r="D70" s="23"/>
-      <c r="E70" s="22"/>
-      <c r="F70" s="24"/>
-      <c r="G70" s="24"/>
-      <c r="H70" s="22"/>
-    </row>
-    <row r="71" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B71" s="15" t="s">
+      <c r="C73" s="18" t="s">
+        <v>223</v>
+      </c>
+      <c r="D73" s="23"/>
+      <c r="E73" s="22"/>
+      <c r="F73" s="24"/>
+      <c r="G73" s="24"/>
+      <c r="H73" s="22"/>
+    </row>
+    <row r="74" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B74" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="C71" s="16" t="s">
+      <c r="C74" s="16" t="s">
         <v>163</v>
       </c>
-      <c r="D71" s="16" t="s">
+      <c r="D74" s="16" t="s">
         <v>164</v>
       </c>
-      <c r="E71" s="15" t="s">
+      <c r="E74" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="F71" s="17" t="s">
+      <c r="F74" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="G71" s="17" t="s">
+      <c r="G74" s="17" t="s">
         <v>123</v>
       </c>
-      <c r="H71" s="15" t="s">
+      <c r="H74" s="15" t="s">
         <v>82</v>
-      </c>
-    </row>
-    <row r="72" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B72" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C72" s="13" t="s">
-        <v>198</v>
-      </c>
-      <c r="D72" s="13" t="s">
-        <v>202</v>
-      </c>
-      <c r="E72" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="F72" s="9">
-        <v>2.8</v>
-      </c>
-      <c r="G72" s="9">
-        <v>20</v>
-      </c>
-      <c r="H72" s="8" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="73" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B73" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="C73" s="13" t="s">
-        <v>198</v>
-      </c>
-      <c r="D73" s="13" t="s">
-        <v>199</v>
-      </c>
-      <c r="E73" s="8" t="s">
-        <v>140</v>
-      </c>
-      <c r="F73" s="9">
-        <v>13</v>
-      </c>
-      <c r="G73" s="9">
-        <v>100</v>
-      </c>
-      <c r="H73" s="8" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="74" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B74" s="8" t="s">
-        <v>217</v>
-      </c>
-      <c r="C74" s="13" t="s">
-        <v>205</v>
-      </c>
-      <c r="D74" s="13" t="s">
-        <v>150</v>
-      </c>
-      <c r="E74" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="F74" s="9">
-        <v>1</v>
-      </c>
-      <c r="G74" s="9"/>
-      <c r="H74" s="8" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="75" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B75" s="8" t="s">
-        <v>125</v>
+        <v>20</v>
       </c>
       <c r="C75" s="13" t="s">
-        <v>218</v>
-      </c>
-      <c r="D75" s="13"/>
+        <v>198</v>
+      </c>
+      <c r="D75" s="13" t="s">
+        <v>202</v>
+      </c>
       <c r="E75" s="8" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F75" s="9">
-        <v>2</v>
-      </c>
-      <c r="G75" s="9"/>
+        <v>2.8</v>
+      </c>
+      <c r="G75" s="9">
+        <v>20</v>
+      </c>
       <c r="H75" s="8" t="s">
-        <v>97</v>
+        <v>115</v>
       </c>
     </row>
     <row r="76" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B76" s="8" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="C76" s="13" t="s">
-        <v>150</v>
+        <v>198</v>
       </c>
       <c r="D76" s="13" t="s">
-        <v>181</v>
+        <v>199</v>
       </c>
       <c r="E76" s="8" t="s">
-        <v>180</v>
+        <v>140</v>
       </c>
       <c r="F76" s="9">
-        <v>1</v>
-      </c>
-      <c r="G76" s="9"/>
-      <c r="H76" s="8"/>
+        <v>13</v>
+      </c>
+      <c r="G76" s="9">
+        <v>100</v>
+      </c>
+      <c r="H76" s="8" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="77" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B77" s="8" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="C77" s="13" t="s">
-        <v>218</v>
+        <v>205</v>
       </c>
       <c r="D77" s="13" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="E77" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="F77" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="G77" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="H77" s="8"/>
+      <c r="F77" s="9">
+        <v>1</v>
+      </c>
+      <c r="G77" s="9"/>
+      <c r="H77" s="8" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="78" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B78" s="8" t="s">
-        <v>219</v>
+        <v>125</v>
       </c>
       <c r="C78" s="13" t="s">
-        <v>150</v>
-      </c>
-      <c r="D78" s="13" t="s">
         <v>218</v>
       </c>
+      <c r="D78" s="13"/>
       <c r="E78" s="8" t="s">
-        <v>166</v>
+        <v>134</v>
       </c>
       <c r="F78" s="9">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G78" s="9"/>
-      <c r="H78" s="8"/>
+      <c r="H78" s="8" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="79" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B79" s="8" t="s">
-        <v>220</v>
+        <v>122</v>
       </c>
       <c r="C79" s="13" t="s">
-        <v>205</v>
+        <v>150</v>
       </c>
       <c r="D79" s="13" t="s">
-        <v>167</v>
-      </c>
-      <c r="E79" s="8"/>
+        <v>181</v>
+      </c>
+      <c r="E79" s="8" t="s">
+        <v>180</v>
+      </c>
       <c r="F79" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G79" s="9"/>
       <c r="H79" s="8"/>
     </row>
     <row r="80" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B80" s="5" t="s">
+      <c r="B80" s="8" t="s">
+        <v>212</v>
+      </c>
+      <c r="C80" s="13" t="s">
+        <v>218</v>
+      </c>
+      <c r="D80" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E80" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="F80" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="G80" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="H80" s="8"/>
+    </row>
+    <row r="81" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B81" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="C81" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="D81" s="13" t="s">
+        <v>218</v>
+      </c>
+      <c r="E81" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="F81" s="9">
+        <v>0</v>
+      </c>
+      <c r="G81" s="9"/>
+      <c r="H81" s="8"/>
+    </row>
+    <row r="82" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B82" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="C82" s="13" t="s">
+        <v>205</v>
+      </c>
+      <c r="D82" s="13" t="s">
+        <v>167</v>
+      </c>
+      <c r="E82" s="8"/>
+      <c r="F82" s="9">
+        <v>0</v>
+      </c>
+      <c r="G82" s="9"/>
+      <c r="H82" s="8"/>
+    </row>
+    <row r="83" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B83" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="C83" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="D83" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="E83" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="F83" s="6">
+        <v>4</v>
+      </c>
+      <c r="G83" s="6">
+        <v>20</v>
+      </c>
+      <c r="H83" s="5" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="84" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B84" s="5" t="s">
         <v>225</v>
       </c>
-      <c r="C80" s="11" t="s">
+      <c r="C84" s="11" t="s">
         <v>197</v>
       </c>
-      <c r="D80" s="11" t="s">
-        <v>201</v>
-      </c>
-      <c r="E80" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="F80" s="6">
-        <v>4</v>
-      </c>
-      <c r="G80" s="6">
+      <c r="D84" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="E84" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="F84" s="6">
         <v>20</v>
       </c>
-      <c r="H80" s="5" t="s">
+      <c r="G84" s="6">
+        <v>100</v>
+      </c>
+      <c r="H84" s="5" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="81" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B81" s="5" t="s">
+    <row r="85" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B85" s="5" t="s">
         <v>226</v>
       </c>
-      <c r="C81" s="11" t="s">
+      <c r="C85" s="11" t="s">
         <v>197</v>
       </c>
-      <c r="D81" s="11" t="s">
-        <v>200</v>
-      </c>
-      <c r="E81" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="F81" s="6">
-        <v>20</v>
-      </c>
-      <c r="G81" s="6">
-        <v>100</v>
-      </c>
-      <c r="H81" s="5" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="82" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B82" s="5" t="s">
-        <v>227</v>
-      </c>
-      <c r="C82" s="11" t="s">
+      <c r="D85" s="11" t="s">
         <v>197</v>
       </c>
-      <c r="D82" s="11" t="s">
-        <v>197</v>
-      </c>
-      <c r="E82" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="F82" s="6">
+      <c r="E85" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F85" s="6">
         <v>2</v>
       </c>
-      <c r="G82" s="6"/>
-      <c r="H82" s="5" t="s">
+      <c r="G85" s="6"/>
+      <c r="H85" s="5" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="83" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B83" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="C83" s="13" t="s">
-        <v>151</v>
-      </c>
-      <c r="D83" s="13"/>
-      <c r="E83" s="8" t="s">
-        <v>134</v>
-      </c>
-      <c r="F83" s="9">
-        <v>1</v>
-      </c>
-      <c r="G83" s="9"/>
-      <c r="H83" s="8"/>
-    </row>
-    <row r="84" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B84" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="C84" s="13" t="s">
-        <v>168</v>
-      </c>
-      <c r="D84" s="13"/>
-      <c r="E84" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="F84" s="9">
-        <v>1</v>
-      </c>
-      <c r="G84" s="9">
-        <v>97.5</v>
-      </c>
-      <c r="H84" s="8" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="85" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B85" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="C85" s="13" t="s">
-        <v>151</v>
-      </c>
-      <c r="D85" s="13" t="s">
-        <v>169</v>
-      </c>
-      <c r="E85" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="F85" s="9">
-        <v>1.5</v>
-      </c>
-      <c r="G85" s="9"/>
-      <c r="H85" s="8"/>
     </row>
     <row r="86" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B86" s="8" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C86" s="13" t="s">
         <v>151</v>
       </c>
-      <c r="D86" s="13" t="s">
-        <v>170</v>
-      </c>
+      <c r="D86" s="13"/>
       <c r="E86" s="8" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="F86" s="9">
         <v>1</v>
@@ -3727,1037 +3767,1037 @@
     </row>
     <row r="87" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B87" s="8" t="s">
-        <v>69</v>
+        <v>118</v>
       </c>
       <c r="C87" s="13" t="s">
-        <v>152</v>
+        <v>168</v>
       </c>
       <c r="D87" s="13"/>
       <c r="E87" s="8" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F87" s="9">
-        <v>1.2</v>
-      </c>
-      <c r="G87" s="9"/>
+        <v>1</v>
+      </c>
+      <c r="G87" s="9">
+        <v>97.5</v>
+      </c>
       <c r="H87" s="8" t="s">
-        <v>98</v>
+        <v>171</v>
       </c>
     </row>
     <row r="88" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B88" s="8" t="s">
-        <v>70</v>
+        <v>119</v>
       </c>
       <c r="C88" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D88" s="13" t="s">
-        <v>152</v>
+        <v>169</v>
       </c>
       <c r="E88" s="8" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F88" s="9">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="G88" s="9"/>
-      <c r="H88" s="8" t="s">
-        <v>99</v>
-      </c>
+      <c r="H88" s="8"/>
     </row>
     <row r="89" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B89" s="8" t="s">
-        <v>71</v>
+        <v>120</v>
       </c>
       <c r="C89" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D89" s="13" t="s">
-        <v>139</v>
+        <v>170</v>
       </c>
       <c r="E89" s="8" t="s">
         <v>137</v>
       </c>
       <c r="F89" s="9">
-        <v>2.9</v>
+        <v>1</v>
       </c>
       <c r="G89" s="9"/>
-      <c r="H89" s="8" t="s">
-        <v>100</v>
-      </c>
+      <c r="H89" s="8"/>
     </row>
     <row r="90" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B90" s="8" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C90" s="13" t="s">
         <v>152</v>
       </c>
-      <c r="D90" s="13" t="s">
-        <v>144</v>
-      </c>
+      <c r="D90" s="13"/>
       <c r="E90" s="8" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="F90" s="9">
         <v>1.2</v>
       </c>
       <c r="G90" s="9"/>
       <c r="H90" s="8" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="91" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B91" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="C91" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="D91" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="E91" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="F91" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="G91" s="9"/>
+      <c r="H91" s="8" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="92" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B92" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="C92" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="D92" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="E92" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="F92" s="9">
+        <v>2.9</v>
+      </c>
+      <c r="G92" s="9"/>
+      <c r="H92" s="8" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="93" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B93" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="C93" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="D93" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E93" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="F93" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="G93" s="9"/>
+      <c r="H93" s="8" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="91" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B91" s="22" t="s">
+    <row r="94" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B94" s="22" t="s">
         <v>189</v>
       </c>
-      <c r="C91" s="18" t="s">
+      <c r="C94" s="18" t="s">
         <v>186</v>
       </c>
-      <c r="D91" s="23"/>
-      <c r="E91" s="22"/>
-      <c r="F91" s="24"/>
-      <c r="G91" s="24"/>
-      <c r="H91" s="22"/>
-    </row>
-    <row r="92" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B92" s="15" t="s">
+      <c r="D94" s="23"/>
+      <c r="E94" s="22"/>
+      <c r="F94" s="24"/>
+      <c r="G94" s="24"/>
+      <c r="H94" s="22"/>
+    </row>
+    <row r="95" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B95" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="C92" s="16" t="s">
+      <c r="C95" s="16" t="s">
         <v>163</v>
       </c>
-      <c r="D92" s="16" t="s">
+      <c r="D95" s="16" t="s">
         <v>164</v>
       </c>
-      <c r="E92" s="15" t="s">
+      <c r="E95" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="F92" s="17" t="s">
+      <c r="F95" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="G92" s="17" t="s">
+      <c r="G95" s="17" t="s">
         <v>123</v>
       </c>
-      <c r="H92" s="15" t="s">
+      <c r="H95" s="15" t="s">
         <v>82</v>
-      </c>
-    </row>
-    <row r="93" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B93" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="C93" s="11" t="s">
-        <v>153</v>
-      </c>
-      <c r="D93" s="11"/>
-      <c r="E93" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="F93" s="6">
-        <v>1.8</v>
-      </c>
-      <c r="G93" s="6"/>
-      <c r="H93" s="5" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="94" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B94" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C94" s="11" t="s">
-        <v>153</v>
-      </c>
-      <c r="D94" s="11" t="s">
-        <v>153</v>
-      </c>
-      <c r="E94" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="F94" s="6">
-        <v>1.4</v>
-      </c>
-      <c r="G94" s="6"/>
-      <c r="H94" s="5" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="95" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B95" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="C95" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="D95" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="E95" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="F95" s="6">
-        <v>10</v>
-      </c>
-      <c r="G95" s="6"/>
-      <c r="H95" s="5" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="96" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B96" s="5" t="s">
-        <v>127</v>
+        <v>73</v>
       </c>
       <c r="C96" s="11" t="s">
         <v>153</v>
       </c>
-      <c r="D96" s="11" t="s">
-        <v>196</v>
-      </c>
+      <c r="D96" s="11"/>
       <c r="E96" s="5" t="s">
-        <v>149</v>
+        <v>134</v>
       </c>
       <c r="F96" s="6">
-        <v>0.8</v>
+        <v>1.8</v>
       </c>
       <c r="G96" s="6"/>
       <c r="H96" s="5" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
     </row>
     <row r="97" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B97" s="5" t="s">
-        <v>128</v>
+        <v>74</v>
       </c>
       <c r="C97" s="11" t="s">
         <v>153</v>
       </c>
       <c r="D97" s="11" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E97" s="5" t="s">
-        <v>149</v>
+        <v>135</v>
       </c>
       <c r="F97" s="6">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="G97" s="6"/>
       <c r="H97" s="5" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="98" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B98" s="5" t="s">
-        <v>179</v>
+        <v>131</v>
       </c>
       <c r="C98" s="11" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D98" s="11" t="s">
-        <v>171</v>
+        <v>154</v>
       </c>
       <c r="E98" s="5" t="s">
-        <v>149</v>
+        <v>135</v>
       </c>
       <c r="F98" s="6">
-        <v>1.2</v>
+        <v>10</v>
       </c>
       <c r="G98" s="6"/>
       <c r="H98" s="5" t="s">
-        <v>178</v>
+        <v>132</v>
       </c>
     </row>
     <row r="99" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B99" s="5" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C99" s="11" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="D99" s="11" t="s">
-        <v>153</v>
+        <v>196</v>
       </c>
       <c r="E99" s="5" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
       <c r="F99" s="6">
-        <v>2</v>
+        <v>0.8</v>
       </c>
       <c r="G99" s="6"/>
       <c r="H99" s="5" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="100" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B100" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="C100" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="D100" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="E100" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="F100" s="6">
+        <v>1.2</v>
+      </c>
+      <c r="G100" s="6"/>
+      <c r="H100" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="101" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B101" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="C101" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="D101" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="E101" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="F101" s="6">
+        <v>1.2</v>
+      </c>
+      <c r="G101" s="6"/>
+      <c r="H101" s="5" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="102" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B102" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C102" s="11" t="s">
+        <v>155</v>
+      </c>
+      <c r="D102" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="E102" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F102" s="6">
+        <v>2</v>
+      </c>
+      <c r="G102" s="6"/>
+      <c r="H102" s="5" t="s">
         <v>110</v>
-      </c>
-    </row>
-    <row r="100" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B100" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="C100" s="13" t="s">
-        <v>156</v>
-      </c>
-      <c r="D100" s="13"/>
-      <c r="E100" s="8" t="s">
-        <v>162</v>
-      </c>
-      <c r="F100" s="9">
-        <v>1.4</v>
-      </c>
-      <c r="G100" s="9"/>
-      <c r="H100" s="8" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="101" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B101" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="C101" s="13" t="s">
-        <v>156</v>
-      </c>
-      <c r="D101" s="13" t="s">
-        <v>156</v>
-      </c>
-      <c r="E101" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="F101" s="9">
-        <v>1.5</v>
-      </c>
-      <c r="G101" s="9"/>
-      <c r="H101" s="8" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="102" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B102" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="C102" s="13" t="s">
-        <v>156</v>
-      </c>
-      <c r="D102" s="13" t="s">
-        <v>153</v>
-      </c>
-      <c r="E102" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="F102" s="9">
-        <v>1</v>
-      </c>
-      <c r="G102" s="9"/>
-      <c r="H102" s="8" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="103" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B103" s="8" t="s">
-        <v>221</v>
+        <v>75</v>
       </c>
       <c r="C103" s="13" t="s">
         <v>156</v>
       </c>
-      <c r="D103" s="13" t="s">
-        <v>205</v>
-      </c>
+      <c r="D103" s="13"/>
       <c r="E103" s="8" t="s">
-        <v>135</v>
+        <v>162</v>
       </c>
       <c r="F103" s="9">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="G103" s="9"/>
       <c r="H103" s="8" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
     </row>
     <row r="104" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B104" s="8" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C104" s="13" t="s">
         <v>156</v>
       </c>
       <c r="D104" s="13" t="s">
-        <v>147</v>
+        <v>156</v>
       </c>
       <c r="E104" s="8" t="s">
         <v>135</v>
       </c>
       <c r="F104" s="9">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="G104" s="9"/>
       <c r="H104" s="8" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
     </row>
     <row r="105" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B105" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C105" s="13" t="s">
         <v>156</v>
       </c>
       <c r="D105" s="13" t="s">
-        <v>171</v>
+        <v>153</v>
       </c>
       <c r="E105" s="8" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F105" s="9">
-        <v>1.4</v>
+        <v>1</v>
       </c>
       <c r="G105" s="9"/>
       <c r="H105" s="8" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="106" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B106" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="C106" s="13" t="s">
+        <v>156</v>
+      </c>
+      <c r="D106" s="13" t="s">
+        <v>205</v>
+      </c>
+      <c r="E106" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="F106" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="G106" s="9"/>
+      <c r="H106" s="8" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="107" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B107" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="C107" s="13" t="s">
+        <v>156</v>
+      </c>
+      <c r="D107" s="13" t="s">
+        <v>147</v>
+      </c>
+      <c r="E107" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="F107" s="9">
+        <v>1</v>
+      </c>
+      <c r="G107" s="9"/>
+      <c r="H107" s="8" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="108" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B108" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="C108" s="13" t="s">
+        <v>156</v>
+      </c>
+      <c r="D108" s="13" t="s">
+        <v>171</v>
+      </c>
+      <c r="E108" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="F108" s="9">
+        <v>1.4</v>
+      </c>
+      <c r="G108" s="9"/>
+      <c r="H108" s="8" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="106" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B106" s="5" t="s">
+    <row r="109" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B109" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="C106" s="11" t="s">
+      <c r="C109" s="11" t="s">
         <v>157</v>
       </c>
-      <c r="D106" s="11"/>
-      <c r="E106" s="5" t="s">
+      <c r="D109" s="11"/>
+      <c r="E109" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="F106" s="6">
+      <c r="F109" s="6">
         <v>3</v>
       </c>
-      <c r="G106" s="6"/>
-      <c r="H106" s="5" t="s">
+      <c r="G109" s="6"/>
+      <c r="H109" s="5" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="107" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B107" s="5" t="s">
+    <row r="110" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B110" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="C107" s="11" t="s">
+      <c r="C110" s="11" t="s">
         <v>157</v>
       </c>
-      <c r="D107" s="11" t="s">
+      <c r="D110" s="11" t="s">
         <v>157</v>
       </c>
-      <c r="E107" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="F107" s="6">
+      <c r="E110" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F110" s="6">
         <v>2</v>
       </c>
-      <c r="G107" s="6"/>
-      <c r="H107" s="5" t="s">
+      <c r="G110" s="6"/>
+      <c r="H110" s="5" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="108" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B108" s="5" t="s">
+    <row r="111" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B111" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="C108" s="11" t="s">
+      <c r="C111" s="11" t="s">
         <v>157</v>
       </c>
-      <c r="D108" s="11" t="s">
+      <c r="D111" s="11" t="s">
         <v>156</v>
       </c>
-      <c r="E108" s="5" t="s">
+      <c r="E111" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="F108" s="6">
+      <c r="F111" s="6">
         <v>1</v>
       </c>
-      <c r="G108" s="6"/>
-      <c r="H108" s="5" t="s">
+      <c r="G111" s="6"/>
+      <c r="H111" s="5" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="109" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B109" s="22" t="s">
+    <row r="112" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B112" s="22" t="s">
         <v>189</v>
       </c>
-      <c r="C109" s="18" t="s">
-        <v>228</v>
-      </c>
-      <c r="D109" s="23"/>
-      <c r="E109" s="22"/>
-      <c r="F109" s="24"/>
-      <c r="G109" s="24"/>
-      <c r="H109" s="22"/>
-    </row>
-    <row r="110" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B110" s="15" t="s">
+      <c r="C112" s="18" t="s">
+        <v>227</v>
+      </c>
+      <c r="D112" s="23"/>
+      <c r="E112" s="22"/>
+      <c r="F112" s="24"/>
+      <c r="G112" s="24"/>
+      <c r="H112" s="22"/>
+    </row>
+    <row r="113" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B113" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="C110" s="16" t="s">
+      <c r="C113" s="16" t="s">
         <v>163</v>
       </c>
-      <c r="D110" s="16" t="s">
+      <c r="D113" s="16" t="s">
         <v>164</v>
       </c>
-      <c r="E110" s="15" t="s">
+      <c r="E113" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="F110" s="17" t="s">
+      <c r="F113" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="G110" s="17" t="s">
+      <c r="G113" s="17" t="s">
         <v>123</v>
       </c>
-      <c r="H110" s="15" t="s">
+      <c r="H113" s="15" t="s">
         <v>82</v>
-      </c>
-    </row>
-    <row r="111" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B111" s="8" t="s">
-        <v>229</v>
-      </c>
-      <c r="C111" s="13" t="s">
-        <v>142</v>
-      </c>
-      <c r="D111" s="13" t="s">
-        <v>206</v>
-      </c>
-      <c r="E111" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="F111" s="9">
-        <v>11</v>
-      </c>
-      <c r="G111" s="9">
-        <v>60</v>
-      </c>
-      <c r="H111" s="8" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="112" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B112" s="8" t="s">
-        <v>230</v>
-      </c>
-      <c r="C112" s="13" t="s">
-        <v>142</v>
-      </c>
-      <c r="D112" s="13" t="s">
-        <v>207</v>
-      </c>
-      <c r="E112" s="8" t="s">
-        <v>140</v>
-      </c>
-      <c r="F112" s="9">
-        <v>2</v>
-      </c>
-      <c r="G112" s="9">
-        <v>30</v>
-      </c>
-      <c r="H112" s="8" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="113" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B113" s="8" t="s">
-        <v>233</v>
-      </c>
-      <c r="C113" s="13" t="s">
-        <v>234</v>
-      </c>
-      <c r="D113" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E113" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="F113" s="9">
-        <v>10</v>
-      </c>
-      <c r="G113" s="9"/>
-      <c r="H113" s="8" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="114" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B114" s="8" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="C114" s="13" t="s">
-        <v>234</v>
+        <v>291</v>
       </c>
       <c r="D114" s="13" t="s">
-        <v>181</v>
+        <v>292</v>
       </c>
       <c r="E114" s="8" t="s">
-        <v>180</v>
+        <v>136</v>
       </c>
       <c r="F114" s="9">
-        <v>1.4</v>
-      </c>
-      <c r="G114" s="9"/>
+        <v>11</v>
+      </c>
+      <c r="G114" s="9">
+        <v>60</v>
+      </c>
       <c r="H114" s="8" t="s">
-        <v>258</v>
+        <v>115</v>
       </c>
     </row>
     <row r="115" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B115" s="8" t="s">
-        <v>252</v>
+        <v>229</v>
       </c>
       <c r="C115" s="13" t="s">
-        <v>234</v>
+        <v>291</v>
       </c>
       <c r="D115" s="13" t="s">
-        <v>147</v>
+        <v>294</v>
       </c>
       <c r="E115" s="8" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="F115" s="9">
         <v>2</v>
       </c>
-      <c r="G115" s="9"/>
+      <c r="G115" s="9">
+        <v>30</v>
+      </c>
       <c r="H115" s="8" t="s">
-        <v>255</v>
+        <v>115</v>
       </c>
     </row>
     <row r="116" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B116" s="5" t="s">
-        <v>231</v>
-      </c>
-      <c r="C116" s="11" t="s">
-        <v>145</v>
-      </c>
-      <c r="D116" s="11" t="s">
-        <v>208</v>
-      </c>
-      <c r="E116" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="F116" s="6">
-        <v>11</v>
-      </c>
-      <c r="G116" s="6">
-        <v>60</v>
-      </c>
-      <c r="H116" s="5" t="s">
-        <v>115</v>
+      <c r="B116" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="C116" s="13" t="s">
+        <v>233</v>
+      </c>
+      <c r="D116" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E116" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="F116" s="9">
+        <v>10</v>
+      </c>
+      <c r="G116" s="9"/>
+      <c r="H116" s="8" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="117" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B117" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="C117" s="11" t="s">
-        <v>145</v>
-      </c>
-      <c r="D117" s="11" t="s">
-        <v>207</v>
-      </c>
-      <c r="E117" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="F117" s="6">
+      <c r="B117" s="8" t="s">
+        <v>234</v>
+      </c>
+      <c r="C117" s="13" t="s">
+        <v>233</v>
+      </c>
+      <c r="D117" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="E117" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="F117" s="9">
+        <v>1.4</v>
+      </c>
+      <c r="G117" s="9"/>
+      <c r="H117" s="8" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="118" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B118" s="8" t="s">
+        <v>251</v>
+      </c>
+      <c r="C118" s="13" t="s">
+        <v>233</v>
+      </c>
+      <c r="D118" s="13" t="s">
+        <v>147</v>
+      </c>
+      <c r="E118" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="F118" s="9">
         <v>2</v>
       </c>
-      <c r="G117" s="6">
-        <v>30</v>
-      </c>
-      <c r="H117" s="5" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="118" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B118" s="5" t="s">
-        <v>236</v>
-      </c>
-      <c r="C118" s="11" t="s">
-        <v>238</v>
-      </c>
-      <c r="D118" s="11" t="s">
-        <v>141</v>
-      </c>
-      <c r="E118" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="F118" s="6">
-        <v>10</v>
-      </c>
-      <c r="G118" s="6"/>
-      <c r="H118" s="5" t="s">
-        <v>260</v>
+      <c r="G118" s="9"/>
+      <c r="H118" s="8" t="s">
+        <v>254</v>
       </c>
     </row>
     <row r="119" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B119" s="5" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="C119" s="11" t="s">
-        <v>238</v>
+        <v>290</v>
       </c>
       <c r="D119" s="11" t="s">
-        <v>181</v>
+        <v>293</v>
       </c>
       <c r="E119" s="5" t="s">
-        <v>180</v>
+        <v>136</v>
       </c>
       <c r="F119" s="6">
-        <v>1.4</v>
-      </c>
-      <c r="G119" s="6"/>
+        <v>11</v>
+      </c>
+      <c r="G119" s="6">
+        <v>60</v>
+      </c>
       <c r="H119" s="5" t="s">
-        <v>259</v>
+        <v>115</v>
       </c>
     </row>
     <row r="120" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B120" s="5" t="s">
-        <v>253</v>
+        <v>231</v>
       </c>
       <c r="C120" s="11" t="s">
-        <v>238</v>
+        <v>290</v>
       </c>
       <c r="D120" s="11" t="s">
-        <v>147</v>
+        <v>294</v>
       </c>
       <c r="E120" s="5" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="F120" s="6">
         <v>2</v>
       </c>
-      <c r="G120" s="6"/>
+      <c r="G120" s="6">
+        <v>30</v>
+      </c>
       <c r="H120" s="5" t="s">
-        <v>254</v>
+        <v>115</v>
       </c>
     </row>
     <row r="121" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B121" s="8" t="s">
-        <v>239</v>
-      </c>
-      <c r="C121" s="13" t="s">
-        <v>240</v>
-      </c>
-      <c r="D121" s="13"/>
-      <c r="E121" s="8" t="s">
-        <v>162</v>
-      </c>
-      <c r="F121" s="9">
-        <v>3</v>
-      </c>
-      <c r="G121" s="9"/>
-      <c r="H121" s="8" t="s">
-        <v>256</v>
+      <c r="B121" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="C121" s="11" t="s">
+        <v>237</v>
+      </c>
+      <c r="D121" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="E121" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F121" s="6">
+        <v>10</v>
+      </c>
+      <c r="G121" s="6"/>
+      <c r="H121" s="5" t="s">
+        <v>259</v>
       </c>
     </row>
     <row r="122" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B122" s="8" t="s">
-        <v>241</v>
-      </c>
-      <c r="C122" s="13" t="s">
-        <v>240</v>
-      </c>
-      <c r="D122" s="13"/>
-      <c r="E122" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="F122" s="9">
-        <v>1.6</v>
-      </c>
-      <c r="G122" s="9"/>
-      <c r="H122" s="8" t="s">
-        <v>257</v>
+      <c r="B122" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="C122" s="11" t="s">
+        <v>237</v>
+      </c>
+      <c r="D122" s="11" t="s">
+        <v>181</v>
+      </c>
+      <c r="E122" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="F122" s="6">
+        <v>1.4</v>
+      </c>
+      <c r="G122" s="6"/>
+      <c r="H122" s="5" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="123" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B123" s="8" t="s">
-        <v>242</v>
-      </c>
-      <c r="C123" s="13" t="s">
-        <v>243</v>
-      </c>
-      <c r="D123" s="13" t="s">
-        <v>205</v>
-      </c>
-      <c r="E123" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="F123" s="9">
-        <v>7</v>
-      </c>
-      <c r="G123" s="9"/>
-      <c r="H123" s="8" t="s">
-        <v>246</v>
+      <c r="B123" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="C123" s="11" t="s">
+        <v>237</v>
+      </c>
+      <c r="D123" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="E123" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F123" s="6">
+        <v>2</v>
+      </c>
+      <c r="G123" s="6"/>
+      <c r="H123" s="5" t="s">
+        <v>253</v>
       </c>
     </row>
     <row r="124" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B124" s="8" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="C124" s="13" t="s">
-        <v>245</v>
-      </c>
-      <c r="D124" s="13" t="s">
-        <v>205</v>
-      </c>
+        <v>239</v>
+      </c>
+      <c r="D124" s="13"/>
       <c r="E124" s="8" t="s">
-        <v>135</v>
+        <v>162</v>
       </c>
       <c r="F124" s="9">
         <v>3</v>
       </c>
       <c r="G124" s="9"/>
       <c r="H124" s="8" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
     </row>
     <row r="125" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B125" s="8" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="C125" s="13" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="D125" s="13" t="s">
-        <v>141</v>
+        <v>239</v>
       </c>
       <c r="E125" s="8" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F125" s="9">
-        <v>4</v>
+        <v>1.6</v>
       </c>
       <c r="G125" s="9"/>
       <c r="H125" s="8" t="s">
-        <v>249</v>
+        <v>256</v>
       </c>
     </row>
     <row r="126" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B126" s="8" t="s">
-        <v>250</v>
+        <v>241</v>
       </c>
       <c r="C126" s="13" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="D126" s="13" t="s">
-        <v>144</v>
+        <v>205</v>
       </c>
       <c r="E126" s="8" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F126" s="9">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G126" s="9"/>
       <c r="H126" s="8" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
     </row>
     <row r="127" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B127" s="22" t="s">
+      <c r="B127" s="8" t="s">
+        <v>243</v>
+      </c>
+      <c r="C127" s="13" t="s">
+        <v>244</v>
+      </c>
+      <c r="D127" s="13" t="s">
+        <v>205</v>
+      </c>
+      <c r="E127" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="F127" s="9">
+        <v>3</v>
+      </c>
+      <c r="G127" s="9"/>
+      <c r="H127" s="8" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="128" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B128" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="C128" s="13" t="s">
+        <v>239</v>
+      </c>
+      <c r="D128" s="13" t="s">
+        <v>141</v>
+      </c>
+      <c r="E128" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="F128" s="9">
+        <v>4</v>
+      </c>
+      <c r="G128" s="9"/>
+      <c r="H128" s="8" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="129" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B129" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="C129" s="13" t="s">
+        <v>239</v>
+      </c>
+      <c r="D129" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E129" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="F129" s="9">
+        <v>4</v>
+      </c>
+      <c r="G129" s="9"/>
+      <c r="H129" s="8" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="130" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B130" s="22" t="s">
         <v>189</v>
       </c>
-      <c r="C127" s="18" t="s">
+      <c r="C130" s="18" t="s">
+        <v>261</v>
+      </c>
+      <c r="D130" s="23"/>
+      <c r="E130" s="22"/>
+      <c r="F130" s="24"/>
+      <c r="G130" s="24"/>
+      <c r="H130" s="22"/>
+    </row>
+    <row r="131" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B131" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="C131" s="16" t="s">
+        <v>163</v>
+      </c>
+      <c r="D131" s="16" t="s">
+        <v>164</v>
+      </c>
+      <c r="E131" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="F131" s="17" t="s">
+        <v>158</v>
+      </c>
+      <c r="G131" s="17" t="s">
+        <v>123</v>
+      </c>
+      <c r="H131" s="15" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="132" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B132" s="25" t="s">
         <v>262</v>
       </c>
-      <c r="D127" s="23"/>
-      <c r="E127" s="22"/>
-      <c r="F127" s="24"/>
-      <c r="G127" s="24"/>
-      <c r="H127" s="22"/>
-    </row>
-    <row r="128" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B128" s="15" t="s">
-        <v>81</v>
-      </c>
-      <c r="C128" s="16" t="s">
-        <v>163</v>
-      </c>
-      <c r="D128" s="16" t="s">
-        <v>164</v>
-      </c>
-      <c r="E128" s="15" t="s">
-        <v>133</v>
-      </c>
-      <c r="F128" s="17" t="s">
-        <v>158</v>
-      </c>
-      <c r="G128" s="17" t="s">
-        <v>123</v>
-      </c>
-      <c r="H128" s="15" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="129" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B129" s="25" t="s">
+      <c r="C132" s="26" t="s">
         <v>263</v>
       </c>
-      <c r="C129" s="26" t="s">
-        <v>264</v>
-      </c>
-      <c r="D129" s="26"/>
-      <c r="E129" s="25" t="s">
+      <c r="D132" s="26"/>
+      <c r="E132" s="25" t="s">
         <v>134</v>
       </c>
-      <c r="F129" s="28">
+      <c r="F132" s="28">
         <v>70</v>
       </c>
-      <c r="G129" s="27"/>
-      <c r="H129" s="25" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="130" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B130" s="25" t="s">
-        <v>265</v>
-      </c>
-      <c r="C130" s="26" t="s">
-        <v>264</v>
-      </c>
-      <c r="D130" s="26"/>
-      <c r="E130" s="25" t="s">
-        <v>135</v>
-      </c>
-      <c r="F130" s="28">
-        <v>64</v>
-      </c>
-      <c r="G130" s="27"/>
-      <c r="H130" s="25" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="131" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B131" s="5" t="s">
-        <v>290</v>
-      </c>
-      <c r="C131" s="11" t="s">
-        <v>269</v>
-      </c>
-      <c r="D131" s="11" t="s">
-        <v>264</v>
-      </c>
-      <c r="E131" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="F131" s="6">
-        <v>5</v>
-      </c>
-      <c r="G131" s="6"/>
-      <c r="H131" s="5" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="132" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B132" s="5" t="s">
-        <v>291</v>
-      </c>
-      <c r="C132" s="11" t="s">
-        <v>267</v>
-      </c>
-      <c r="D132" s="11" t="s">
-        <v>264</v>
-      </c>
-      <c r="E132" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="F132" s="6">
-        <v>5</v>
-      </c>
-      <c r="G132" s="6"/>
-      <c r="H132" s="5" t="s">
-        <v>281</v>
+      <c r="G132" s="27"/>
+      <c r="H132" s="25" t="s">
+        <v>276</v>
       </c>
     </row>
     <row r="133" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B133" s="25" t="s">
-        <v>288</v>
+        <v>264</v>
       </c>
       <c r="C133" s="26" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D133" s="26" t="s">
-        <v>156</v>
+        <v>263</v>
       </c>
       <c r="E133" s="25" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F133" s="28">
-        <v>10</v>
+        <v>64</v>
       </c>
       <c r="G133" s="27"/>
       <c r="H133" s="25" t="s">
-        <v>289</v>
+        <v>277</v>
       </c>
     </row>
     <row r="134" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B134" s="5" t="s">
-        <v>271</v>
+        <v>288</v>
       </c>
       <c r="C134" s="11" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="D134" s="11" t="s">
-        <v>141</v>
+        <v>263</v>
       </c>
       <c r="E134" s="5" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
       <c r="F134" s="6">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="G134" s="6"/>
       <c r="H134" s="5" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
     </row>
     <row r="135" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B135" s="5" t="s">
-        <v>270</v>
+        <v>289</v>
       </c>
       <c r="C135" s="11" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="D135" s="11" t="s">
-        <v>144</v>
+        <v>263</v>
       </c>
       <c r="E135" s="5" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
       <c r="F135" s="6">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="G135" s="6"/>
       <c r="H135" s="5" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
     </row>
     <row r="136" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B136" s="5" t="s">
-        <v>272</v>
-      </c>
-      <c r="C136" s="11" t="s">
-        <v>264</v>
-      </c>
-      <c r="D136" s="11" t="s">
-        <v>205</v>
-      </c>
-      <c r="E136" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="F136" s="6">
-        <v>14</v>
-      </c>
-      <c r="G136" s="6"/>
-      <c r="H136" s="5" t="s">
-        <v>285</v>
+      <c r="B136" s="25" t="s">
+        <v>286</v>
+      </c>
+      <c r="C136" s="26" t="s">
+        <v>263</v>
+      </c>
+      <c r="D136" s="26" t="s">
+        <v>304</v>
+      </c>
+      <c r="E136" s="25" t="s">
+        <v>137</v>
+      </c>
+      <c r="F136" s="28">
+        <v>10</v>
+      </c>
+      <c r="G136" s="27"/>
+      <c r="H136" s="25" t="s">
+        <v>287</v>
       </c>
     </row>
     <row r="137" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B137" s="5" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="C137" s="11" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D137" s="11" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="E137" s="5" t="s">
         <v>135</v>
@@ -4766,19 +4806,19 @@
         <v>14</v>
       </c>
       <c r="G137" s="6"/>
-      <c r="H137" s="25" t="s">
+      <c r="H137" s="5" t="s">
         <v>282</v>
       </c>
     </row>
     <row r="138" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B138" s="5" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C138" s="11" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D138" s="11" t="s">
-        <v>157</v>
+        <v>144</v>
       </c>
       <c r="E138" s="5" t="s">
         <v>135</v>
@@ -4787,89 +4827,210 @@
         <v>14</v>
       </c>
       <c r="G138" s="6"/>
-      <c r="H138" s="25" t="s">
-        <v>283</v>
+      <c r="H138" s="5" t="s">
+        <v>282</v>
       </c>
     </row>
     <row r="139" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B139" s="5" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C139" s="11" t="s">
-        <v>157</v>
+        <v>263</v>
       </c>
       <c r="D139" s="11" t="s">
-        <v>274</v>
-      </c>
-      <c r="E139" s="5"/>
+        <v>205</v>
+      </c>
+      <c r="E139" s="5" t="s">
+        <v>135</v>
+      </c>
       <c r="F139" s="6">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="G139" s="6"/>
       <c r="H139" s="5" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
     </row>
     <row r="140" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B140" s="5" t="s">
-        <v>275</v>
+        <v>265</v>
       </c>
       <c r="C140" s="11" t="s">
-        <v>157</v>
+        <v>263</v>
       </c>
       <c r="D140" s="11" t="s">
-        <v>274</v>
+        <v>153</v>
       </c>
       <c r="E140" s="5" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F140" s="6">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="G140" s="6"/>
-      <c r="H140" s="5" t="s">
-        <v>286</v>
+      <c r="H140" s="25" t="s">
+        <v>280</v>
       </c>
     </row>
     <row r="141" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B141" s="5" t="s">
-        <v>276</v>
+        <v>267</v>
       </c>
       <c r="C141" s="11" t="s">
+        <v>263</v>
+      </c>
+      <c r="D141" s="11" t="s">
         <v>157</v>
       </c>
-      <c r="D141" s="11" t="s">
-        <v>274</v>
-      </c>
-      <c r="E141" s="5"/>
+      <c r="E141" s="5" t="s">
+        <v>135</v>
+      </c>
       <c r="F141" s="6">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="G141" s="6"/>
-      <c r="H141" s="5" t="s">
-        <v>287</v>
+      <c r="H141" s="25" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="142" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B142" s="5" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="C142" s="11" t="s">
         <v>157</v>
       </c>
-      <c r="D142" s="11" t="s">
-        <v>274</v>
-      </c>
+      <c r="D142" s="11"/>
       <c r="E142" s="5" t="s">
-        <v>134</v>
+        <v>296</v>
       </c>
       <c r="F142" s="6">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="G142" s="6"/>
       <c r="H142" s="5" t="s">
-        <v>287</v>
-      </c>
+        <v>284</v>
+      </c>
+    </row>
+    <row r="143" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B143" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="C143" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="D143" s="11"/>
+      <c r="E143" s="5" t="s">
+        <v>295</v>
+      </c>
+      <c r="F143" s="6">
+        <v>40</v>
+      </c>
+      <c r="G143" s="6"/>
+      <c r="H143" s="5" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="144" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B144" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="C144" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="D144" s="11"/>
+      <c r="E144" s="5" t="s">
+        <v>296</v>
+      </c>
+      <c r="F144" s="6">
+        <v>19</v>
+      </c>
+      <c r="G144" s="6"/>
+      <c r="H144" s="5" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="145" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B145" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="C145" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="D145" s="11"/>
+      <c r="E145" s="5" t="s">
+        <v>295</v>
+      </c>
+      <c r="F145" s="6">
+        <v>40</v>
+      </c>
+      <c r="G145" s="6"/>
+      <c r="H145" s="5" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="146" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B146" s="22" t="s">
+        <v>189</v>
+      </c>
+      <c r="C146" s="18" t="s">
+        <v>299</v>
+      </c>
+      <c r="D146" s="23"/>
+      <c r="E146" s="22"/>
+      <c r="F146" s="24"/>
+      <c r="G146" s="24"/>
+      <c r="H146" s="22"/>
+    </row>
+    <row r="147" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B147" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="C147" s="16" t="s">
+        <v>163</v>
+      </c>
+      <c r="D147" s="16" t="s">
+        <v>164</v>
+      </c>
+      <c r="E147" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="F147" s="17" t="s">
+        <v>158</v>
+      </c>
+      <c r="G147" s="17" t="s">
+        <v>123</v>
+      </c>
+      <c r="H147" s="15" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="148" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B148" s="25" t="s">
+        <v>212</v>
+      </c>
+      <c r="C148" s="26" t="s">
+        <v>263</v>
+      </c>
+      <c r="D148" s="26"/>
+      <c r="E148" s="25" t="s">
+        <v>300</v>
+      </c>
+      <c r="F148" s="28">
+        <v>0</v>
+      </c>
+      <c r="G148" s="27"/>
+      <c r="H148" s="25"/>
+    </row>
+    <row r="149" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B149" s="25"/>
+      <c r="C149" s="26"/>
+      <c r="D149" s="26"/>
+      <c r="E149" s="25"/>
+      <c r="F149" s="28"/>
+      <c r="G149" s="27"/>
+      <c r="H149" s="25"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
20260111: Update DRC for AR GC TieDown
</commit_message>
<xml_diff>
--- a/Document/TR-1um_Drawing_Layer_DR_Table.xlsx
+++ b/Document/TR-1um_Drawing_Layer_DR_Table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/okamura/Library/CloudStorage/Dropbox/91_OpenPDK/TR-1um/Document/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE0B6A12-3D26-294A-97DB-4A7BD4673915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{853BFEFC-D2B5-A548-B488-6E7B65D7D185}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="800" yWindow="760" windowWidth="29440" windowHeight="18880" xr2:uid="{7F1200E8-B51D-9446-A5CE-CEA05B5231B7}"/>
+    <workbookView xWindow="900" yWindow="760" windowWidth="29440" windowHeight="18880" xr2:uid="{7F1200E8-B51D-9446-A5CE-CEA05B5231B7}"/>
   </bookViews>
   <sheets>
     <sheet name="TR-1um_Drawing_Layer_DR_Table" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="690" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="691" uniqueCount="307">
   <si>
     <t>WN.W1</t>
   </si>
@@ -692,9 +692,6 @@
     <t>AR.GC</t>
   </si>
   <si>
-    <t>GC(AR)</t>
-  </si>
-  <si>
     <t>GC.R1</t>
   </si>
   <si>
@@ -954,6 +951,12 @@
   </si>
   <si>
     <t>GC+GR</t>
+  </si>
+  <si>
+    <t>GC(R)</t>
+  </si>
+  <si>
+    <t>GC.ANT</t>
   </si>
 </sst>
 </file>
@@ -2047,7 +2050,7 @@
         <v>189</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D2" s="23"/>
       <c r="E2" s="22"/>
@@ -2124,7 +2127,7 @@
         <v>147</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>172</v>
@@ -2194,10 +2197,10 @@
     </row>
     <row r="10" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D10" s="11" t="s">
         <v>153</v>
@@ -2213,10 +2216,10 @@
     </row>
     <row r="11" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D11" s="11" t="s">
         <v>157</v>
@@ -2232,16 +2235,16 @@
     </row>
     <row r="12" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="5" t="s">
+        <v>301</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>262</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>303</v>
+      </c>
+      <c r="E12" s="5" t="s">
         <v>302</v>
-      </c>
-      <c r="C12" s="11" t="s">
-        <v>263</v>
-      </c>
-      <c r="D12" s="11" t="s">
-        <v>304</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>303</v>
       </c>
       <c r="F12" s="6">
         <v>0</v>
@@ -3470,7 +3473,7 @@
         <v>147</v>
       </c>
       <c r="D72" s="11" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="E72" s="5" t="s">
         <v>137</v>
@@ -3488,7 +3491,7 @@
         <v>189</v>
       </c>
       <c r="C73" s="18" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D73" s="23"/>
       <c r="E73" s="22"/>
@@ -3591,7 +3594,7 @@
         <v>125</v>
       </c>
       <c r="C78" s="13" t="s">
-        <v>218</v>
+        <v>305</v>
       </c>
       <c r="D78" s="13"/>
       <c r="E78" s="8" t="s">
@@ -3629,7 +3632,7 @@
         <v>212</v>
       </c>
       <c r="C80" s="13" t="s">
-        <v>218</v>
+        <v>305</v>
       </c>
       <c r="D80" s="13" t="s">
         <v>144</v>
@@ -3647,13 +3650,13 @@
     </row>
     <row r="81" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B81" s="8" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C81" s="13" t="s">
         <v>150</v>
       </c>
       <c r="D81" s="13" t="s">
-        <v>218</v>
+        <v>305</v>
       </c>
       <c r="E81" s="8" t="s">
         <v>166</v>
@@ -3666,15 +3669,17 @@
     </row>
     <row r="82" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B82" s="8" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C82" s="13" t="s">
-        <v>205</v>
+        <v>305</v>
       </c>
       <c r="D82" s="13" t="s">
+        <v>160</v>
+      </c>
+      <c r="E82" s="8" t="s">
         <v>167</v>
       </c>
-      <c r="E82" s="8"/>
       <c r="F82" s="9">
         <v>0</v>
       </c>
@@ -3683,7 +3688,7 @@
     </row>
     <row r="83" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B83" s="5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C83" s="11" t="s">
         <v>197</v>
@@ -3706,7 +3711,7 @@
     </row>
     <row r="84" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B84" s="5" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C84" s="11" t="s">
         <v>197</v>
@@ -3729,7 +3734,7 @@
     </row>
     <row r="85" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B85" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C85" s="11" t="s">
         <v>197</v>
@@ -4150,7 +4155,7 @@
     </row>
     <row r="106" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B106" s="8" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C106" s="13" t="s">
         <v>156</v>
@@ -4277,7 +4282,7 @@
         <v>189</v>
       </c>
       <c r="C112" s="18" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D112" s="23"/>
       <c r="E112" s="22"/>
@@ -4310,13 +4315,13 @@
     </row>
     <row r="114" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B114" s="8" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C114" s="13" t="s">
+        <v>290</v>
+      </c>
+      <c r="D114" s="13" t="s">
         <v>291</v>
-      </c>
-      <c r="D114" s="13" t="s">
-        <v>292</v>
       </c>
       <c r="E114" s="8" t="s">
         <v>136</v>
@@ -4333,13 +4338,13 @@
     </row>
     <row r="115" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B115" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C115" s="13" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D115" s="13" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E115" s="8" t="s">
         <v>140</v>
@@ -4356,10 +4361,10 @@
     </row>
     <row r="116" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B116" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="C116" s="13" t="s">
         <v>232</v>
-      </c>
-      <c r="C116" s="13" t="s">
-        <v>233</v>
       </c>
       <c r="D116" s="13" t="s">
         <v>144</v>
@@ -4372,15 +4377,15 @@
       </c>
       <c r="G116" s="9"/>
       <c r="H116" s="8" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="117" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B117" s="8" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C117" s="13" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D117" s="13" t="s">
         <v>181</v>
@@ -4393,15 +4398,15 @@
       </c>
       <c r="G117" s="9"/>
       <c r="H117" s="8" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="118" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B118" s="8" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C118" s="13" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D118" s="13" t="s">
         <v>147</v>
@@ -4414,18 +4419,18 @@
       </c>
       <c r="G118" s="9"/>
       <c r="H118" s="8" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="119" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B119" s="5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C119" s="11" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D119" s="11" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E119" s="5" t="s">
         <v>136</v>
@@ -4442,13 +4447,13 @@
     </row>
     <row r="120" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B120" s="5" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C120" s="11" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D120" s="11" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E120" s="5" t="s">
         <v>140</v>
@@ -4465,10 +4470,10 @@
     </row>
     <row r="121" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B121" s="5" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C121" s="11" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="D121" s="11" t="s">
         <v>141</v>
@@ -4481,15 +4486,15 @@
       </c>
       <c r="G121" s="6"/>
       <c r="H121" s="5" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="122" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B122" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="C122" s="11" t="s">
         <v>236</v>
-      </c>
-      <c r="C122" s="11" t="s">
-        <v>237</v>
       </c>
       <c r="D122" s="11" t="s">
         <v>181</v>
@@ -4502,15 +4507,15 @@
       </c>
       <c r="G122" s="6"/>
       <c r="H122" s="5" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="123" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B123" s="5" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C123" s="11" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="D123" s="11" t="s">
         <v>147</v>
@@ -4523,15 +4528,15 @@
       </c>
       <c r="G123" s="6"/>
       <c r="H123" s="5" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="124" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B124" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="C124" s="13" t="s">
         <v>238</v>
-      </c>
-      <c r="C124" s="13" t="s">
-        <v>239</v>
       </c>
       <c r="D124" s="13"/>
       <c r="E124" s="8" t="s">
@@ -4542,18 +4547,18 @@
       </c>
       <c r="G124" s="9"/>
       <c r="H124" s="8" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="125" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B125" s="8" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C125" s="13" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="D125" s="13" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E125" s="8" t="s">
         <v>135</v>
@@ -4563,15 +4568,15 @@
       </c>
       <c r="G125" s="9"/>
       <c r="H125" s="8" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="126" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B126" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="C126" s="13" t="s">
         <v>241</v>
-      </c>
-      <c r="C126" s="13" t="s">
-        <v>242</v>
       </c>
       <c r="D126" s="13" t="s">
         <v>205</v>
@@ -4584,15 +4589,15 @@
       </c>
       <c r="G126" s="9"/>
       <c r="H126" s="8" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="127" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B127" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="C127" s="13" t="s">
         <v>243</v>
-      </c>
-      <c r="C127" s="13" t="s">
-        <v>244</v>
       </c>
       <c r="D127" s="13" t="s">
         <v>205</v>
@@ -4605,15 +4610,15 @@
       </c>
       <c r="G127" s="9"/>
       <c r="H127" s="8" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="128" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B128" s="8" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C128" s="13" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="D128" s="13" t="s">
         <v>141</v>
@@ -4626,15 +4631,15 @@
       </c>
       <c r="G128" s="9"/>
       <c r="H128" s="8" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="129" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B129" s="8" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C129" s="13" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="D129" s="13" t="s">
         <v>144</v>
@@ -4647,7 +4652,7 @@
       </c>
       <c r="G129" s="9"/>
       <c r="H129" s="8" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="130" spans="2:8" ht="20" x14ac:dyDescent="0.2">
@@ -4655,7 +4660,7 @@
         <v>189</v>
       </c>
       <c r="C130" s="18" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D130" s="23"/>
       <c r="E130" s="22"/>
@@ -4688,10 +4693,10 @@
     </row>
     <row r="132" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B132" s="25" t="s">
+        <v>261</v>
+      </c>
+      <c r="C132" s="26" t="s">
         <v>262</v>
-      </c>
-      <c r="C132" s="26" t="s">
-        <v>263</v>
       </c>
       <c r="D132" s="26"/>
       <c r="E132" s="25" t="s">
@@ -4702,18 +4707,18 @@
       </c>
       <c r="G132" s="27"/>
       <c r="H132" s="25" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="133" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B133" s="25" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C133" s="26" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D133" s="26" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E133" s="25" t="s">
         <v>135</v>
@@ -4723,18 +4728,18 @@
       </c>
       <c r="G133" s="27"/>
       <c r="H133" s="25" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="134" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B134" s="5" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C134" s="11" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D134" s="11" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E134" s="5" t="s">
         <v>149</v>
@@ -4744,18 +4749,18 @@
       </c>
       <c r="G134" s="6"/>
       <c r="H134" s="5" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="135" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B135" s="5" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C135" s="11" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D135" s="11" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E135" s="5" t="s">
         <v>149</v>
@@ -4765,18 +4770,18 @@
       </c>
       <c r="G135" s="6"/>
       <c r="H135" s="5" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="136" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B136" s="25" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C136" s="26" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D136" s="26" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="E136" s="25" t="s">
         <v>137</v>
@@ -4786,15 +4791,15 @@
       </c>
       <c r="G136" s="27"/>
       <c r="H136" s="25" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="137" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B137" s="5" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C137" s="11" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D137" s="11" t="s">
         <v>141</v>
@@ -4807,15 +4812,15 @@
       </c>
       <c r="G137" s="6"/>
       <c r="H137" s="5" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="138" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B138" s="5" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C138" s="11" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D138" s="11" t="s">
         <v>144</v>
@@ -4828,15 +4833,15 @@
       </c>
       <c r="G138" s="6"/>
       <c r="H138" s="5" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="139" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B139" s="5" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C139" s="11" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D139" s="11" t="s">
         <v>205</v>
@@ -4849,15 +4854,15 @@
       </c>
       <c r="G139" s="6"/>
       <c r="H139" s="5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="140" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B140" s="5" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C140" s="11" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D140" s="11" t="s">
         <v>153</v>
@@ -4870,15 +4875,15 @@
       </c>
       <c r="G140" s="6"/>
       <c r="H140" s="25" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="141" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B141" s="5" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C141" s="11" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D141" s="11" t="s">
         <v>157</v>
@@ -4891,83 +4896,83 @@
       </c>
       <c r="G141" s="6"/>
       <c r="H141" s="25" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="142" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B142" s="5" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C142" s="11" t="s">
         <v>157</v>
       </c>
       <c r="D142" s="11"/>
       <c r="E142" s="5" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="F142" s="6">
         <v>19</v>
       </c>
       <c r="G142" s="6"/>
       <c r="H142" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="143" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B143" s="5" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C143" s="11" t="s">
         <v>157</v>
       </c>
       <c r="D143" s="11"/>
       <c r="E143" s="5" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F143" s="6">
         <v>40</v>
       </c>
       <c r="G143" s="6"/>
       <c r="H143" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="144" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B144" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C144" s="11" t="s">
         <v>157</v>
       </c>
       <c r="D144" s="11"/>
       <c r="E144" s="5" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="F144" s="6">
         <v>19</v>
       </c>
       <c r="G144" s="6"/>
       <c r="H144" s="5" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="145" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B145" s="5" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C145" s="11" t="s">
         <v>157</v>
       </c>
       <c r="D145" s="11"/>
       <c r="E145" s="5" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F145" s="6">
         <v>40</v>
       </c>
       <c r="G145" s="6"/>
       <c r="H145" s="5" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="146" spans="2:8" ht="20" x14ac:dyDescent="0.2">
@@ -4975,7 +4980,7 @@
         <v>189</v>
       </c>
       <c r="C146" s="18" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D146" s="23"/>
       <c r="E146" s="22"/>
@@ -5008,14 +5013,14 @@
     </row>
     <row r="148" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B148" s="25" t="s">
-        <v>212</v>
+        <v>306</v>
       </c>
       <c r="C148" s="26" t="s">
-        <v>263</v>
+        <v>304</v>
       </c>
       <c r="D148" s="26"/>
       <c r="E148" s="25" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="F148" s="28">
         <v>0</v>

</xml_diff>

<commit_message>
DRC run.drc revised for GC.W1
</commit_message>
<xml_diff>
--- a/Document/TR-1um_Drawing_Layer_DR_Table.xlsx
+++ b/Document/TR-1um_Drawing_Layer_DR_Table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/okamura/Dropbox/91_OpenPDK/TR-1um/Document/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{439FB1C9-0C98-1F41-9D86-FF4ED4B90AE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F25997B7-96D7-0A45-B11D-707DCB591EDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="860" yWindow="760" windowWidth="29380" windowHeight="18880" xr2:uid="{7F1200E8-B51D-9446-A5CE-CEA05B5231B7}"/>
   </bookViews>
@@ -3205,14 +3205,12 @@
       </c>
       <c r="D59" s="13"/>
       <c r="E59" s="8" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F59" s="9">
         <v>1</v>
       </c>
-      <c r="G59" s="9">
-        <v>30</v>
-      </c>
+      <c r="G59" s="9"/>
       <c r="H59" s="8" t="s">
         <v>83</v>
       </c>

</xml_diff>

<commit_message>
Update DRC related XLSX, CVS, PPT, and PDF.
</commit_message>
<xml_diff>
--- a/Document/TR-1um_Drawing_Layer_DR_Table.xlsx
+++ b/Document/TR-1um_Drawing_Layer_DR_Table.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/okamura/Dropbox/91_OpenPDK/TR-1um/Document/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7DEDE13-D27A-A84E-9F44-6EFB9E5FB4D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D292DF46-E6E0-E44A-9FE0-AB4BC713DCAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="860" yWindow="700" windowWidth="29380" windowHeight="18880" xr2:uid="{7F1200E8-B51D-9446-A5CE-CEA05B5231B7}"/>
+    <workbookView xWindow="9300" yWindow="960" windowWidth="29360" windowHeight="18880" xr2:uid="{7F1200E8-B51D-9446-A5CE-CEA05B5231B7}"/>
   </bookViews>
   <sheets>
     <sheet name="TR-1um_Drawing_Layer_DR_Table" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="691" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="695" uniqueCount="313">
   <si>
     <t>WN.W1</t>
   </si>
@@ -966,6 +966,15 @@
   </si>
   <si>
     <t>Cat-4: GC/CO related</t>
+  </si>
+  <si>
+    <t>Sfix</t>
+  </si>
+  <si>
+    <t>Efix</t>
+  </si>
+  <si>
+    <t>M1.W2</t>
   </si>
 </sst>
 </file>
@@ -2065,7 +2074,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4478C0F2-BA21-8B4B-B7C2-220C0E7FA6A8}">
-  <dimension ref="B2:H150"/>
+  <dimension ref="B2:H151"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="19" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.6640625" style="4" customWidth="1"/>
@@ -2706,7 +2715,7 @@
         <v>143</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>134</v>
+        <v>310</v>
       </c>
       <c r="F33" s="6">
         <v>2.8</v>
@@ -2727,7 +2736,7 @@
         <v>198</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>136</v>
+        <v>311</v>
       </c>
       <c r="F34" s="6">
         <v>1.4</v>
@@ -3377,7 +3386,7 @@
       </c>
       <c r="D66" s="11"/>
       <c r="E66" s="5" t="s">
-        <v>133</v>
+        <v>161</v>
       </c>
       <c r="F66" s="6">
         <v>1</v>
@@ -3884,7 +3893,7 @@
       </c>
       <c r="D91" s="13"/>
       <c r="E91" s="8" t="s">
-        <v>133</v>
+        <v>161</v>
       </c>
       <c r="F91" s="9">
         <v>1.2</v>
@@ -3905,7 +3914,7 @@
         <v>151</v>
       </c>
       <c r="E92" s="8" t="s">
-        <v>134</v>
+        <v>310</v>
       </c>
       <c r="F92" s="9">
         <v>1.2</v>
@@ -4002,404 +4011,402 @@
       </c>
       <c r="D97" s="11"/>
       <c r="E97" s="5" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="F97" s="6">
         <v>1.8</v>
       </c>
-      <c r="G97" s="6"/>
+      <c r="G97" s="6">
+        <v>10</v>
+      </c>
       <c r="H97" s="5" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="98" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B98" s="5" t="s">
-        <v>73</v>
+        <v>312</v>
       </c>
       <c r="C98" s="11" t="s">
-        <v>152</v>
-      </c>
-      <c r="D98" s="11" t="s">
-        <v>152</v>
-      </c>
+        <v>154</v>
+      </c>
+      <c r="D98" s="11"/>
       <c r="E98" s="5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F98" s="6">
-        <v>1.4</v>
+        <v>10</v>
       </c>
       <c r="G98" s="6"/>
       <c r="H98" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="99" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B99" s="5" t="s">
-        <v>130</v>
+        <v>73</v>
       </c>
       <c r="C99" s="11" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D99" s="11" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E99" s="5" t="s">
         <v>134</v>
       </c>
       <c r="F99" s="6">
-        <v>10</v>
+        <v>1.4</v>
       </c>
       <c r="G99" s="6"/>
       <c r="H99" s="5" t="s">
-        <v>131</v>
+        <v>102</v>
       </c>
     </row>
     <row r="100" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B100" s="5" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C100" s="11" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D100" s="11" t="s">
-        <v>189</v>
+        <v>153</v>
       </c>
       <c r="E100" s="5" t="s">
-        <v>148</v>
+        <v>310</v>
       </c>
       <c r="F100" s="6">
-        <v>0.8</v>
+        <v>10</v>
       </c>
       <c r="G100" s="6"/>
       <c r="H100" s="5" t="s">
-        <v>108</v>
+        <v>131</v>
       </c>
     </row>
     <row r="101" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B101" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C101" s="11" t="s">
         <v>152</v>
       </c>
       <c r="D101" s="11" t="s">
-        <v>151</v>
+        <v>189</v>
       </c>
       <c r="E101" s="5" t="s">
         <v>148</v>
       </c>
       <c r="F101" s="6">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="G101" s="6"/>
       <c r="H101" s="5" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
     </row>
     <row r="102" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B102" s="5" t="s">
-        <v>178</v>
+        <v>127</v>
       </c>
       <c r="C102" s="11" t="s">
         <v>152</v>
       </c>
       <c r="D102" s="11" t="s">
-        <v>170</v>
+        <v>151</v>
       </c>
       <c r="E102" s="5" t="s">
         <v>148</v>
       </c>
       <c r="F102" s="6">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="G102" s="6"/>
       <c r="H102" s="5" t="s">
-        <v>177</v>
+        <v>100</v>
       </c>
     </row>
     <row r="103" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B103" s="5" t="s">
-        <v>123</v>
+        <v>178</v>
       </c>
       <c r="C103" s="11" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D103" s="11" t="s">
-        <v>152</v>
+        <v>170</v>
       </c>
       <c r="E103" s="5" t="s">
-        <v>134</v>
+        <v>148</v>
       </c>
       <c r="F103" s="6">
-        <v>2</v>
+        <v>1.2</v>
       </c>
       <c r="G103" s="6"/>
       <c r="H103" s="5" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="104" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B104" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C104" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="D104" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="E104" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="F104" s="6">
+        <v>2</v>
+      </c>
+      <c r="G104" s="6"/>
+      <c r="H104" s="5" t="s">
         <v>109</v>
-      </c>
-    </row>
-    <row r="104" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B104" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="C104" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="D104" s="13"/>
-      <c r="E104" s="8" t="s">
-        <v>161</v>
-      </c>
-      <c r="F104" s="9">
-        <v>1.4</v>
-      </c>
-      <c r="G104" s="9"/>
-      <c r="H104" s="8" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="105" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B105" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C105" s="13" t="s">
         <v>155</v>
       </c>
-      <c r="D105" s="13" t="s">
-        <v>155</v>
-      </c>
+      <c r="D105" s="13"/>
       <c r="E105" s="8" t="s">
-        <v>134</v>
+        <v>161</v>
       </c>
       <c r="F105" s="9">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="G105" s="9"/>
       <c r="H105" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="106" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B106" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C106" s="13" t="s">
         <v>155</v>
       </c>
       <c r="D106" s="13" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="E106" s="8" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F106" s="9">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="G106" s="9"/>
       <c r="H106" s="8" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="107" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B107" s="8" t="s">
-        <v>213</v>
+        <v>76</v>
       </c>
       <c r="C107" s="13" t="s">
         <v>155</v>
       </c>
       <c r="D107" s="13" t="s">
-        <v>198</v>
+        <v>152</v>
       </c>
       <c r="E107" s="8" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F107" s="9">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="G107" s="9"/>
       <c r="H107" s="8" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="108" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B108" s="8" t="s">
-        <v>77</v>
+        <v>213</v>
       </c>
       <c r="C108" s="13" t="s">
         <v>155</v>
       </c>
       <c r="D108" s="13" t="s">
-        <v>146</v>
+        <v>198</v>
       </c>
       <c r="E108" s="8" t="s">
         <v>134</v>
       </c>
       <c r="F108" s="9">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="G108" s="9"/>
       <c r="H108" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="109" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B109" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C109" s="13" t="s">
         <v>155</v>
       </c>
       <c r="D109" s="13" t="s">
-        <v>170</v>
+        <v>146</v>
       </c>
       <c r="E109" s="8" t="s">
         <v>134</v>
       </c>
       <c r="F109" s="9">
-        <v>1.4</v>
+        <v>1</v>
       </c>
       <c r="G109" s="9"/>
       <c r="H109" s="8" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="110" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B110" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="C110" s="13" t="s">
+        <v>155</v>
+      </c>
+      <c r="D110" s="13" t="s">
+        <v>170</v>
+      </c>
+      <c r="E110" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="F110" s="9">
+        <v>1.4</v>
+      </c>
+      <c r="G110" s="9"/>
+      <c r="H110" s="8" t="s">
         <v>112</v>
-      </c>
-    </row>
-    <row r="110" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B110" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="C110" s="11" t="s">
-        <v>156</v>
-      </c>
-      <c r="D110" s="11"/>
-      <c r="E110" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="F110" s="6">
-        <v>3</v>
-      </c>
-      <c r="G110" s="6"/>
-      <c r="H110" s="5" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="111" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B111" s="5" t="s">
-        <v>120</v>
+        <v>79</v>
       </c>
       <c r="C111" s="11" t="s">
         <v>156</v>
       </c>
-      <c r="D111" s="11" t="s">
-        <v>156</v>
-      </c>
+      <c r="D111" s="11"/>
       <c r="E111" s="5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F111" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G111" s="6"/>
       <c r="H111" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="112" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B112" s="5" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="C112" s="11" t="s">
         <v>156</v>
       </c>
       <c r="D112" s="11" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E112" s="5" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="F112" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G112" s="6"/>
       <c r="H112" s="5" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="113" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B113" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="C113" s="11" t="s">
+        <v>156</v>
+      </c>
+      <c r="D113" s="11" t="s">
+        <v>155</v>
+      </c>
+      <c r="E113" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="F113" s="6">
+        <v>1</v>
+      </c>
+      <c r="G113" s="6"/>
+      <c r="H113" s="5" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="113" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B113" s="22" t="s">
+    <row r="114" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B114" s="22" t="s">
         <v>183</v>
       </c>
-      <c r="C113" s="18" t="s">
+      <c r="C114" s="18" t="s">
         <v>305</v>
       </c>
-      <c r="D113" s="23"/>
-      <c r="E113" s="22"/>
-      <c r="F113" s="24"/>
-      <c r="G113" s="24"/>
-      <c r="H113" s="22"/>
-    </row>
-    <row r="114" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B114" s="15" t="s">
+      <c r="D114" s="23"/>
+      <c r="E114" s="22"/>
+      <c r="F114" s="24"/>
+      <c r="G114" s="24"/>
+      <c r="H114" s="22"/>
+    </row>
+    <row r="115" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B115" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="C114" s="16" t="s">
+      <c r="C115" s="16" t="s">
         <v>162</v>
       </c>
-      <c r="D114" s="16" t="s">
+      <c r="D115" s="16" t="s">
         <v>163</v>
       </c>
-      <c r="E114" s="15" t="s">
+      <c r="E115" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="F114" s="17" t="s">
+      <c r="F115" s="17" t="s">
         <v>157</v>
       </c>
-      <c r="G114" s="17" t="s">
+      <c r="G115" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="H114" s="15" t="s">
+      <c r="H115" s="15" t="s">
         <v>81</v>
-      </c>
-    </row>
-    <row r="115" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B115" s="8" t="s">
-        <v>218</v>
-      </c>
-      <c r="C115" s="13" t="s">
-        <v>280</v>
-      </c>
-      <c r="D115" s="13" t="s">
-        <v>281</v>
-      </c>
-      <c r="E115" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="F115" s="9">
-        <v>11</v>
-      </c>
-      <c r="G115" s="9">
-        <v>60</v>
-      </c>
-      <c r="H115" s="8" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="116" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B116" s="8" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C116" s="13" t="s">
         <v>280</v>
       </c>
       <c r="D116" s="13" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="E116" s="8" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="F116" s="9">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="G116" s="9">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="H116" s="8" t="s">
         <v>114</v>
@@ -4407,108 +4414,108 @@
     </row>
     <row r="117" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B117" s="8" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="C117" s="13" t="s">
-        <v>223</v>
+        <v>280</v>
       </c>
       <c r="D117" s="13" t="s">
-        <v>143</v>
+        <v>283</v>
       </c>
       <c r="E117" s="8" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="F117" s="9">
-        <v>10</v>
-      </c>
-      <c r="G117" s="9"/>
+        <v>2</v>
+      </c>
+      <c r="G117" s="9">
+        <v>30</v>
+      </c>
       <c r="H117" s="8" t="s">
-        <v>250</v>
+        <v>114</v>
       </c>
     </row>
     <row r="118" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B118" s="8" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C118" s="13" t="s">
         <v>223</v>
       </c>
       <c r="D118" s="13" t="s">
-        <v>180</v>
+        <v>143</v>
       </c>
       <c r="E118" s="8" t="s">
-        <v>179</v>
+        <v>134</v>
       </c>
       <c r="F118" s="9">
-        <v>1.4</v>
+        <v>10</v>
       </c>
       <c r="G118" s="9"/>
       <c r="H118" s="8" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
     </row>
     <row r="119" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B119" s="8" t="s">
-        <v>241</v>
+        <v>224</v>
       </c>
       <c r="C119" s="13" t="s">
         <v>223</v>
       </c>
       <c r="D119" s="13" t="s">
-        <v>146</v>
+        <v>180</v>
       </c>
       <c r="E119" s="8" t="s">
-        <v>134</v>
+        <v>179</v>
       </c>
       <c r="F119" s="9">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="G119" s="9"/>
       <c r="H119" s="8" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="120" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B120" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="C120" s="13" t="s">
+        <v>223</v>
+      </c>
+      <c r="D120" s="13" t="s">
+        <v>146</v>
+      </c>
+      <c r="E120" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="F120" s="9">
+        <v>2</v>
+      </c>
+      <c r="G120" s="9"/>
+      <c r="H120" s="8" t="s">
         <v>244</v>
-      </c>
-    </row>
-    <row r="120" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B120" s="5" t="s">
-        <v>220</v>
-      </c>
-      <c r="C120" s="11" t="s">
-        <v>279</v>
-      </c>
-      <c r="D120" s="11" t="s">
-        <v>282</v>
-      </c>
-      <c r="E120" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="F120" s="6">
-        <v>11</v>
-      </c>
-      <c r="G120" s="6">
-        <v>60</v>
-      </c>
-      <c r="H120" s="5" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="121" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B121" s="5" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C121" s="11" t="s">
         <v>279</v>
       </c>
       <c r="D121" s="11" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="E121" s="5" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="F121" s="6">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="G121" s="6">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="H121" s="5" t="s">
         <v>114</v>
@@ -4516,134 +4523,136 @@
     </row>
     <row r="122" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B122" s="5" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="C122" s="11" t="s">
-        <v>227</v>
+        <v>279</v>
       </c>
       <c r="D122" s="11" t="s">
-        <v>140</v>
+        <v>283</v>
       </c>
       <c r="E122" s="5" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="F122" s="6">
-        <v>10</v>
-      </c>
-      <c r="G122" s="6"/>
+        <v>2</v>
+      </c>
+      <c r="G122" s="6">
+        <v>30</v>
+      </c>
       <c r="H122" s="5" t="s">
-        <v>249</v>
+        <v>114</v>
       </c>
     </row>
     <row r="123" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B123" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C123" s="11" t="s">
         <v>227</v>
       </c>
       <c r="D123" s="11" t="s">
-        <v>180</v>
+        <v>140</v>
       </c>
       <c r="E123" s="5" t="s">
-        <v>179</v>
+        <v>134</v>
       </c>
       <c r="F123" s="6">
-        <v>1.4</v>
+        <v>10</v>
       </c>
       <c r="G123" s="6"/>
       <c r="H123" s="5" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="124" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B124" s="5" t="s">
-        <v>242</v>
+        <v>226</v>
       </c>
       <c r="C124" s="11" t="s">
         <v>227</v>
       </c>
       <c r="D124" s="11" t="s">
-        <v>146</v>
+        <v>180</v>
       </c>
       <c r="E124" s="5" t="s">
-        <v>134</v>
+        <v>179</v>
       </c>
       <c r="F124" s="6">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="G124" s="6"/>
       <c r="H124" s="5" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="125" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B125" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="C125" s="11" t="s">
+        <v>227</v>
+      </c>
+      <c r="D125" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="E125" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="F125" s="6">
+        <v>2</v>
+      </c>
+      <c r="G125" s="6"/>
+      <c r="H125" s="5" t="s">
         <v>243</v>
-      </c>
-    </row>
-    <row r="125" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B125" s="8" t="s">
-        <v>228</v>
-      </c>
-      <c r="C125" s="13" t="s">
-        <v>229</v>
-      </c>
-      <c r="D125" s="13"/>
-      <c r="E125" s="8" t="s">
-        <v>161</v>
-      </c>
-      <c r="F125" s="9">
-        <v>3</v>
-      </c>
-      <c r="G125" s="9"/>
-      <c r="H125" s="8" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="126" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B126" s="8" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C126" s="13" t="s">
         <v>229</v>
       </c>
-      <c r="D126" s="13" t="s">
-        <v>229</v>
-      </c>
+      <c r="D126" s="13"/>
       <c r="E126" s="8" t="s">
-        <v>134</v>
+        <v>161</v>
       </c>
       <c r="F126" s="9">
-        <v>1.6</v>
+        <v>3</v>
       </c>
       <c r="G126" s="9"/>
       <c r="H126" s="8" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="127" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B127" s="8" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C127" s="13" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="D127" s="13" t="s">
-        <v>198</v>
+        <v>229</v>
       </c>
       <c r="E127" s="8" t="s">
         <v>134</v>
       </c>
       <c r="F127" s="9">
-        <v>7</v>
+        <v>1.6</v>
       </c>
       <c r="G127" s="9"/>
       <c r="H127" s="8" t="s">
-        <v>235</v>
+        <v>246</v>
       </c>
     </row>
     <row r="128" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B128" s="8" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C128" s="13" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="D128" s="13" t="s">
         <v>198</v>
@@ -4652,43 +4661,43 @@
         <v>134</v>
       </c>
       <c r="F128" s="9">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G128" s="9"/>
       <c r="H128" s="8" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="129" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B129" s="8" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="C129" s="13" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="D129" s="13" t="s">
-        <v>140</v>
+        <v>198</v>
       </c>
       <c r="E129" s="8" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F129" s="9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G129" s="9"/>
       <c r="H129" s="8" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="130" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B130" s="8" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C130" s="13" t="s">
         <v>229</v>
       </c>
       <c r="D130" s="13" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="E130" s="8" t="s">
         <v>136</v>
@@ -4698,112 +4707,112 @@
       </c>
       <c r="G130" s="9"/>
       <c r="H130" s="8" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="131" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B131" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="C131" s="13" t="s">
+        <v>229</v>
+      </c>
+      <c r="D131" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="E131" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="F131" s="9">
+        <v>4</v>
+      </c>
+      <c r="G131" s="9"/>
+      <c r="H131" s="8" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="131" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B131" s="22" t="s">
+    <row r="132" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B132" s="22" t="s">
         <v>183</v>
       </c>
-      <c r="C131" s="18" t="s">
+      <c r="C132" s="18" t="s">
         <v>306</v>
       </c>
-      <c r="D131" s="23"/>
-      <c r="E131" s="22"/>
-      <c r="F131" s="24"/>
-      <c r="G131" s="24"/>
-      <c r="H131" s="22"/>
-    </row>
-    <row r="132" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B132" s="15" t="s">
+      <c r="D132" s="23"/>
+      <c r="E132" s="22"/>
+      <c r="F132" s="24"/>
+      <c r="G132" s="24"/>
+      <c r="H132" s="22"/>
+    </row>
+    <row r="133" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B133" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="C132" s="16" t="s">
+      <c r="C133" s="16" t="s">
         <v>162</v>
       </c>
-      <c r="D132" s="16" t="s">
+      <c r="D133" s="16" t="s">
         <v>163</v>
       </c>
-      <c r="E132" s="15" t="s">
+      <c r="E133" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="F132" s="17" t="s">
+      <c r="F133" s="17" t="s">
         <v>157</v>
       </c>
-      <c r="G132" s="17" t="s">
+      <c r="G133" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="H132" s="15" t="s">
+      <c r="H133" s="15" t="s">
         <v>81</v>
-      </c>
-    </row>
-    <row r="133" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B133" s="25" t="s">
-        <v>251</v>
-      </c>
-      <c r="C133" s="26" t="s">
-        <v>252</v>
-      </c>
-      <c r="D133" s="26"/>
-      <c r="E133" s="25" t="s">
-        <v>133</v>
-      </c>
-      <c r="F133" s="28">
-        <v>70</v>
-      </c>
-      <c r="G133" s="27"/>
-      <c r="H133" s="25" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="134" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B134" s="25" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="C134" s="26" t="s">
         <v>252</v>
       </c>
-      <c r="D134" s="26" t="s">
-        <v>252</v>
-      </c>
+      <c r="D134" s="26"/>
       <c r="E134" s="25" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F134" s="28">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="G134" s="27"/>
       <c r="H134" s="25" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="135" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B135" s="25" t="s">
+        <v>253</v>
+      </c>
+      <c r="C135" s="26" t="s">
+        <v>252</v>
+      </c>
+      <c r="D135" s="26" t="s">
+        <v>252</v>
+      </c>
+      <c r="E135" s="25" t="s">
+        <v>134</v>
+      </c>
+      <c r="F135" s="28">
+        <v>64</v>
+      </c>
+      <c r="G135" s="27"/>
+      <c r="H135" s="25" t="s">
         <v>266</v>
-      </c>
-    </row>
-    <row r="135" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B135" s="5" t="s">
-        <v>277</v>
-      </c>
-      <c r="C135" s="11" t="s">
-        <v>257</v>
-      </c>
-      <c r="D135" s="11" t="s">
-        <v>252</v>
-      </c>
-      <c r="E135" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="F135" s="6">
-        <v>5</v>
-      </c>
-      <c r="G135" s="6"/>
-      <c r="H135" s="5" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="136" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B136" s="5" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C136" s="11" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="D136" s="11" t="s">
         <v>252</v>
@@ -4816,60 +4825,60 @@
       </c>
       <c r="G136" s="6"/>
       <c r="H136" s="5" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="137" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B137" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="C137" s="11" t="s">
+        <v>255</v>
+      </c>
+      <c r="D137" s="11" t="s">
+        <v>252</v>
+      </c>
+      <c r="E137" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="F137" s="6">
+        <v>5</v>
+      </c>
+      <c r="G137" s="6"/>
+      <c r="H137" s="5" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="137" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B137" s="25" t="s">
+    <row r="138" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B138" s="25" t="s">
         <v>275</v>
       </c>
-      <c r="C137" s="26" t="s">
+      <c r="C138" s="26" t="s">
         <v>252</v>
       </c>
-      <c r="D137" s="26" t="s">
+      <c r="D138" s="26" t="s">
         <v>290</v>
       </c>
-      <c r="E137" s="25" t="s">
+      <c r="E138" s="25" t="s">
         <v>136</v>
       </c>
-      <c r="F137" s="28">
+      <c r="F138" s="28">
         <v>10</v>
       </c>
-      <c r="G137" s="27"/>
-      <c r="H137" s="25" t="s">
+      <c r="G138" s="27"/>
+      <c r="H138" s="25" t="s">
         <v>276</v>
-      </c>
-    </row>
-    <row r="138" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B138" s="5" t="s">
-        <v>259</v>
-      </c>
-      <c r="C138" s="11" t="s">
-        <v>252</v>
-      </c>
-      <c r="D138" s="11" t="s">
-        <v>140</v>
-      </c>
-      <c r="E138" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="F138" s="6">
-        <v>14</v>
-      </c>
-      <c r="G138" s="6"/>
-      <c r="H138" s="5" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="139" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B139" s="5" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C139" s="11" t="s">
         <v>252</v>
       </c>
       <c r="D139" s="11" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="E139" s="5" t="s">
         <v>134</v>
@@ -4884,13 +4893,13 @@
     </row>
     <row r="140" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B140" s="5" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C140" s="11" t="s">
         <v>252</v>
       </c>
       <c r="D140" s="11" t="s">
-        <v>198</v>
+        <v>143</v>
       </c>
       <c r="E140" s="5" t="s">
         <v>134</v>
@@ -4900,18 +4909,18 @@
       </c>
       <c r="G140" s="6"/>
       <c r="H140" s="5" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="141" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B141" s="5" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="C141" s="11" t="s">
         <v>252</v>
       </c>
       <c r="D141" s="11" t="s">
-        <v>152</v>
+        <v>198</v>
       </c>
       <c r="E141" s="5" t="s">
         <v>134</v>
@@ -4920,19 +4929,19 @@
         <v>14</v>
       </c>
       <c r="G141" s="6"/>
-      <c r="H141" s="25" t="s">
-        <v>269</v>
+      <c r="H141" s="5" t="s">
+        <v>272</v>
       </c>
     </row>
     <row r="142" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B142" s="5" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="C142" s="11" t="s">
         <v>252</v>
       </c>
       <c r="D142" s="11" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="E142" s="5" t="s">
         <v>134</v>
@@ -4942,41 +4951,43 @@
       </c>
       <c r="G142" s="6"/>
       <c r="H142" s="25" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="143" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B143" s="5" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="C143" s="11" t="s">
+        <v>252</v>
+      </c>
+      <c r="D143" s="11" t="s">
         <v>156</v>
       </c>
-      <c r="D143" s="11"/>
       <c r="E143" s="5" t="s">
-        <v>285</v>
+        <v>134</v>
       </c>
       <c r="F143" s="6">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="G143" s="6"/>
-      <c r="H143" s="5" t="s">
-        <v>273</v>
+      <c r="H143" s="25" t="s">
+        <v>270</v>
       </c>
     </row>
     <row r="144" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B144" s="5" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C144" s="11" t="s">
         <v>156</v>
       </c>
       <c r="D144" s="11"/>
       <c r="E144" s="5" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="F144" s="6">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="G144" s="6"/>
       <c r="H144" s="5" t="s">
@@ -4985,36 +4996,36 @@
     </row>
     <row r="145" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B145" s="5" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C145" s="11" t="s">
         <v>156</v>
       </c>
       <c r="D145" s="11"/>
       <c r="E145" s="5" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F145" s="6">
-        <v>19</v>
+        <v>40</v>
       </c>
       <c r="G145" s="6"/>
       <c r="H145" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="146" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B146" s="5" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C146" s="11" t="s">
         <v>156</v>
       </c>
       <c r="D146" s="11"/>
       <c r="E146" s="5" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="F146" s="6">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="G146" s="6"/>
       <c r="H146" s="5" t="s">
@@ -5022,66 +5033,85 @@
       </c>
     </row>
     <row r="147" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B147" s="22" t="s">
+      <c r="B147" s="5" t="s">
+        <v>264</v>
+      </c>
+      <c r="C147" s="11" t="s">
+        <v>156</v>
+      </c>
+      <c r="D147" s="11"/>
+      <c r="E147" s="5" t="s">
+        <v>284</v>
+      </c>
+      <c r="F147" s="6">
+        <v>40</v>
+      </c>
+      <c r="G147" s="6"/>
+      <c r="H147" s="5" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="148" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B148" s="22" t="s">
         <v>183</v>
       </c>
-      <c r="C147" s="18" t="s">
+      <c r="C148" s="18" t="s">
         <v>307</v>
       </c>
-      <c r="D147" s="23"/>
-      <c r="E147" s="22"/>
-      <c r="F147" s="24"/>
-      <c r="G147" s="24"/>
-      <c r="H147" s="22"/>
-    </row>
-    <row r="148" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B148" s="15" t="s">
+      <c r="D148" s="23"/>
+      <c r="E148" s="22"/>
+      <c r="F148" s="24"/>
+      <c r="G148" s="24"/>
+      <c r="H148" s="22"/>
+    </row>
+    <row r="149" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B149" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="C148" s="16" t="s">
+      <c r="C149" s="16" t="s">
         <v>162</v>
       </c>
-      <c r="D148" s="16" t="s">
+      <c r="D149" s="16" t="s">
         <v>163</v>
       </c>
-      <c r="E148" s="15" t="s">
+      <c r="E149" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="F148" s="17" t="s">
+      <c r="F149" s="17" t="s">
         <v>157</v>
       </c>
-      <c r="G148" s="17" t="s">
+      <c r="G149" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="H148" s="15" t="s">
+      <c r="H149" s="15" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="149" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B149" s="31" t="s">
+    <row r="150" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B150" s="31" t="s">
         <v>293</v>
       </c>
-      <c r="C149" s="32" t="s">
+      <c r="C150" s="32" t="s">
         <v>198</v>
       </c>
-      <c r="D149" s="32"/>
-      <c r="E149" s="31" t="s">
+      <c r="D150" s="32"/>
+      <c r="E150" s="31" t="s">
         <v>295</v>
       </c>
-      <c r="F149" s="33">
+      <c r="F150" s="33">
         <v>0</v>
       </c>
-      <c r="G149" s="34"/>
-      <c r="H149" s="31"/>
-    </row>
-    <row r="150" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B150" s="31"/>
-      <c r="C150" s="32"/>
-      <c r="D150" s="32"/>
-      <c r="E150" s="31"/>
-      <c r="F150" s="33"/>
       <c r="G150" s="34"/>
       <c r="H150" s="31"/>
+    </row>
+    <row r="151" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B151" s="31"/>
+      <c r="C151" s="32"/>
+      <c r="D151" s="32"/>
+      <c r="E151" s="31"/>
+      <c r="F151" s="33"/>
+      <c r="G151" s="34"/>
+      <c r="H151" s="31"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Fix TYPO in the DRC  documents.
</commit_message>
<xml_diff>
--- a/Document/TR-1um_Drawing_Layer_DR_Table.xlsx
+++ b/Document/TR-1um_Drawing_Layer_DR_Table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/okamura/Dropbox/91_OpenPDK/TR-1um/Document/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D292DF46-E6E0-E44A-9FE0-AB4BC713DCAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC2BED15-A1FD-4A40-BE8E-D204E4EB1CB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9300" yWindow="960" windowWidth="29360" windowHeight="18880" xr2:uid="{7F1200E8-B51D-9446-A5CE-CEA05B5231B7}"/>
+    <workbookView xWindow="1200" yWindow="760" windowWidth="29340" windowHeight="18880" xr2:uid="{7F1200E8-B51D-9446-A5CE-CEA05B5231B7}"/>
   </bookViews>
   <sheets>
     <sheet name="TR-1um_Drawing_Layer_DR_Table" sheetId="2" r:id="rId1"/>
@@ -2720,7 +2720,9 @@
       <c r="F33" s="6">
         <v>2.8</v>
       </c>
-      <c r="G33" s="6"/>
+      <c r="G33" s="6">
+        <v>2.8</v>
+      </c>
       <c r="H33" s="5" t="s">
         <v>37</v>
       </c>
@@ -2741,7 +2743,9 @@
       <c r="F34" s="6">
         <v>1.4</v>
       </c>
-      <c r="G34" s="6"/>
+      <c r="G34" s="6">
+        <v>1.4</v>
+      </c>
       <c r="H34" s="5" t="s">
         <v>196</v>
       </c>
@@ -3391,7 +3395,9 @@
       <c r="F66" s="6">
         <v>1</v>
       </c>
-      <c r="G66" s="6"/>
+      <c r="G66" s="6">
+        <v>1</v>
+      </c>
       <c r="H66" s="5" t="s">
         <v>87</v>
       </c>
@@ -3431,7 +3437,9 @@
       <c r="F68" s="6">
         <v>1.2</v>
       </c>
-      <c r="G68" s="6"/>
+      <c r="G68" s="6">
+        <v>1.2</v>
+      </c>
       <c r="H68" s="5" t="s">
         <v>89</v>
       </c>
@@ -3898,7 +3906,9 @@
       <c r="F91" s="9">
         <v>1.2</v>
       </c>
-      <c r="G91" s="9"/>
+      <c r="G91" s="9">
+        <v>1.2</v>
+      </c>
       <c r="H91" s="8" t="s">
         <v>97</v>
       </c>
@@ -3919,7 +3929,9 @@
       <c r="F92" s="9">
         <v>1.2</v>
       </c>
-      <c r="G92" s="9"/>
+      <c r="G92" s="9">
+        <v>1.2</v>
+      </c>
       <c r="H92" s="8" t="s">
         <v>98</v>
       </c>
@@ -4079,7 +4091,9 @@
       <c r="F100" s="6">
         <v>10</v>
       </c>
-      <c r="G100" s="6"/>
+      <c r="G100" s="6">
+        <v>10</v>
+      </c>
       <c r="H100" s="5" t="s">
         <v>131</v>
       </c>
@@ -4182,7 +4196,9 @@
       <c r="F105" s="9">
         <v>1.4</v>
       </c>
-      <c r="G105" s="9"/>
+      <c r="G105" s="9">
+        <v>1.4</v>
+      </c>
       <c r="H105" s="8" t="s">
         <v>103</v>
       </c>
@@ -4621,7 +4637,9 @@
       <c r="F126" s="9">
         <v>3</v>
       </c>
-      <c r="G126" s="9"/>
+      <c r="G126" s="9">
+        <v>3</v>
+      </c>
       <c r="H126" s="8" t="s">
         <v>245</v>
       </c>

</xml_diff>

<commit_message>
More changes based on @H-Ojiro feedback.
Create new CO(CC) layer as CO & AC, and use this for M1.CC check.
Calculate M1W as -5 +5 and then use default derived to base spacing rule for M1.SW

Signed-off-by: Mitch Bailey <d.mitch.bailey@gmail.com>
</commit_message>
<xml_diff>
--- a/Document/TR-1um_Drawing_Layer_DR_Table.xlsx
+++ b/Document/TR-1um_Drawing_Layer_DR_Table.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="718" uniqueCount="324">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="718" uniqueCount="325">
   <si>
     <t>#</t>
   </si>
@@ -704,6 +704,9 @@
   </si>
   <si>
     <t>M1.CC</t>
+  </si>
+  <si>
+    <t>CO(CC)</t>
   </si>
   <si>
     <t>M1.CL</t>
@@ -6063,8 +6066,8 @@
       <c r="C108" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="D108" s="13" t="s">
-        <v>154</v>
+      <c r="D108" s="25" t="s">
+        <v>231</v>
       </c>
       <c r="E108" s="12" t="s">
         <v>228</v>
@@ -6098,7 +6101,7 @@
     <row r="109" ht="19.5" customHeight="1">
       <c r="A109" s="1"/>
       <c r="B109" s="12" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C109" s="13" t="s">
         <v>21</v>
@@ -6114,7 +6117,7 @@
       </c>
       <c r="G109" s="14"/>
       <c r="H109" s="12" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="I109" s="1"/>
       <c r="J109" s="1"/>
@@ -6138,7 +6141,7 @@
     <row r="110" ht="19.5" customHeight="1">
       <c r="A110" s="1"/>
       <c r="B110" s="12" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C110" s="13" t="s">
         <v>219</v>
@@ -6154,7 +6157,7 @@
       </c>
       <c r="G110" s="14"/>
       <c r="H110" s="12" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="I110" s="1"/>
       <c r="J110" s="1"/>
@@ -6178,7 +6181,7 @@
     <row r="111" ht="19.5" customHeight="1">
       <c r="A111" s="1"/>
       <c r="B111" s="19" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C111" s="20" t="s">
         <v>23</v>
@@ -6194,7 +6197,7 @@
         <v>1.4</v>
       </c>
       <c r="H111" s="19" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="I111" s="1"/>
       <c r="J111" s="1"/>
@@ -6218,7 +6221,7 @@
     <row r="112" ht="19.5" customHeight="1">
       <c r="A112" s="1"/>
       <c r="B112" s="19" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C112" s="20" t="s">
         <v>23</v>
@@ -6234,7 +6237,7 @@
       </c>
       <c r="G112" s="21"/>
       <c r="H112" s="19" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="I112" s="1"/>
       <c r="J112" s="1"/>
@@ -6258,7 +6261,7 @@
     <row r="113" ht="19.5" customHeight="1">
       <c r="A113" s="1"/>
       <c r="B113" s="19" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C113" s="20" t="s">
         <v>23</v>
@@ -6274,7 +6277,7 @@
       </c>
       <c r="G113" s="21"/>
       <c r="H113" s="19" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="I113" s="1"/>
       <c r="J113" s="1"/>
@@ -6298,7 +6301,7 @@
     <row r="114" ht="19.5" customHeight="1">
       <c r="A114" s="1"/>
       <c r="B114" s="19" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C114" s="20" t="s">
         <v>23</v>
@@ -6314,7 +6317,7 @@
       </c>
       <c r="G114" s="21"/>
       <c r="H114" s="19" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="I114" s="1"/>
       <c r="J114" s="1"/>
@@ -6338,7 +6341,7 @@
     <row r="115" ht="19.5" customHeight="1">
       <c r="A115" s="1"/>
       <c r="B115" s="19" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C115" s="20" t="s">
         <v>23</v>
@@ -6354,7 +6357,7 @@
       </c>
       <c r="G115" s="21"/>
       <c r="H115" s="19" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="I115" s="1"/>
       <c r="J115" s="1"/>
@@ -6378,7 +6381,7 @@
     <row r="116" ht="19.5" customHeight="1">
       <c r="A116" s="1"/>
       <c r="B116" s="19" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C116" s="20" t="s">
         <v>23</v>
@@ -6394,7 +6397,7 @@
       </c>
       <c r="G116" s="21"/>
       <c r="H116" s="19" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="I116" s="1"/>
       <c r="J116" s="1"/>
@@ -6418,7 +6421,7 @@
     <row r="117" ht="19.5" customHeight="1">
       <c r="A117" s="1"/>
       <c r="B117" s="12" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C117" s="13" t="s">
         <v>25</v>
@@ -6432,7 +6435,7 @@
       </c>
       <c r="G117" s="14"/>
       <c r="H117" s="12" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I117" s="1"/>
       <c r="J117" s="1"/>
@@ -6456,7 +6459,7 @@
     <row r="118" ht="19.5" customHeight="1">
       <c r="A118" s="1"/>
       <c r="B118" s="12" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C118" s="13" t="s">
         <v>25</v>
@@ -6472,7 +6475,7 @@
       </c>
       <c r="G118" s="14"/>
       <c r="H118" s="12" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="I118" s="1"/>
       <c r="J118" s="1"/>
@@ -6496,7 +6499,7 @@
     <row r="119" ht="19.5" customHeight="1">
       <c r="A119" s="1"/>
       <c r="B119" s="12" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C119" s="13" t="s">
         <v>25</v>
@@ -6512,7 +6515,7 @@
       </c>
       <c r="G119" s="14"/>
       <c r="H119" s="12" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="I119" s="1"/>
       <c r="J119" s="1"/>
@@ -6539,7 +6542,7 @@
         <v>0</v>
       </c>
       <c r="C120" s="5" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D120" s="6"/>
       <c r="E120" s="4"/>
@@ -6610,13 +6613,13 @@
     <row r="122" ht="18.75" customHeight="1">
       <c r="A122" s="1"/>
       <c r="B122" s="19" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C122" s="20" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D122" s="20" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E122" s="19" t="s">
         <v>67</v>
@@ -6652,13 +6655,13 @@
     <row r="123" ht="18.75" customHeight="1">
       <c r="A123" s="1"/>
       <c r="B123" s="19" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C123" s="20" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D123" s="20" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E123" s="19" t="s">
         <v>96</v>
@@ -6694,10 +6697,10 @@
     <row r="124" ht="18.75" customHeight="1">
       <c r="A124" s="1"/>
       <c r="B124" s="19" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C124" s="20" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D124" s="20" t="s">
         <v>53</v>
@@ -6710,7 +6713,7 @@
       </c>
       <c r="G124" s="21"/>
       <c r="H124" s="19" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="I124" s="1"/>
       <c r="J124" s="1"/>
@@ -6734,10 +6737,10 @@
     <row r="125" ht="18.75" customHeight="1">
       <c r="A125" s="1"/>
       <c r="B125" s="19" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C125" s="20" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D125" s="20" t="s">
         <v>185</v>
@@ -6750,7 +6753,7 @@
       </c>
       <c r="G125" s="21"/>
       <c r="H125" s="19" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="I125" s="1"/>
       <c r="J125" s="1"/>
@@ -6774,10 +6777,10 @@
     <row r="126" ht="18.75" customHeight="1">
       <c r="A126" s="1"/>
       <c r="B126" s="19" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C126" s="20" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D126" s="20" t="s">
         <v>18</v>
@@ -6790,7 +6793,7 @@
       </c>
       <c r="G126" s="21"/>
       <c r="H126" s="19" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="I126" s="1"/>
       <c r="J126" s="1"/>
@@ -6814,13 +6817,13 @@
     <row r="127" ht="18.75" customHeight="1">
       <c r="A127" s="1"/>
       <c r="B127" s="12" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C127" s="13" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D127" s="13" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E127" s="12" t="s">
         <v>67</v>
@@ -6856,13 +6859,13 @@
     <row r="128" ht="18.75" customHeight="1">
       <c r="A128" s="1"/>
       <c r="B128" s="12" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C128" s="13" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D128" s="13" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E128" s="12" t="s">
         <v>96</v>
@@ -6898,10 +6901,10 @@
     <row r="129" ht="18.75" customHeight="1">
       <c r="A129" s="1"/>
       <c r="B129" s="12" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C129" s="13" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D129" s="13" t="s">
         <v>11</v>
@@ -6914,7 +6917,7 @@
       </c>
       <c r="G129" s="14"/>
       <c r="H129" s="12" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="I129" s="1"/>
       <c r="J129" s="1"/>
@@ -6938,10 +6941,10 @@
     <row r="130" ht="18.75" customHeight="1">
       <c r="A130" s="1"/>
       <c r="B130" s="12" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C130" s="13" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D130" s="13" t="s">
         <v>185</v>
@@ -6954,7 +6957,7 @@
       </c>
       <c r="G130" s="14"/>
       <c r="H130" s="12" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="I130" s="1"/>
       <c r="J130" s="1"/>
@@ -6978,10 +6981,10 @@
     <row r="131" ht="18.75" customHeight="1">
       <c r="A131" s="1"/>
       <c r="B131" s="12" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C131" s="13" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D131" s="13" t="s">
         <v>18</v>
@@ -6994,7 +6997,7 @@
       </c>
       <c r="G131" s="14"/>
       <c r="H131" s="12" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="I131" s="1"/>
       <c r="J131" s="1"/>
@@ -7018,10 +7021,10 @@
     <row r="132" ht="18.75" customHeight="1">
       <c r="A132" s="1"/>
       <c r="B132" s="19" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C132" s="20" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D132" s="20"/>
       <c r="E132" s="19" t="s">
@@ -7034,7 +7037,7 @@
         <v>3.0</v>
       </c>
       <c r="H132" s="19" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="I132" s="1"/>
       <c r="J132" s="1"/>
@@ -7058,10 +7061,10 @@
     <row r="133" ht="18.75" customHeight="1">
       <c r="A133" s="1"/>
       <c r="B133" s="19" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C133" s="20" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D133" s="20" t="s">
         <v>18</v>
@@ -7074,7 +7077,7 @@
       </c>
       <c r="G133" s="21"/>
       <c r="H133" s="19" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="I133" s="1"/>
       <c r="J133" s="1"/>
@@ -7098,10 +7101,10 @@
     <row r="134" ht="18.75" customHeight="1">
       <c r="A134" s="1"/>
       <c r="B134" s="19" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C134" s="20" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D134" s="20" t="s">
         <v>78</v>
@@ -7114,7 +7117,7 @@
       </c>
       <c r="G134" s="21"/>
       <c r="H134" s="19" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="I134" s="1"/>
       <c r="J134" s="1"/>
@@ -7138,10 +7141,10 @@
     <row r="135" ht="18.75" customHeight="1">
       <c r="A135" s="1"/>
       <c r="B135" s="19" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C135" s="20" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D135" s="20" t="s">
         <v>78</v>
@@ -7154,7 +7157,7 @@
       </c>
       <c r="G135" s="21"/>
       <c r="H135" s="19" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="I135" s="1"/>
       <c r="J135" s="1"/>
@@ -7178,10 +7181,10 @@
     <row r="136" ht="18.75" customHeight="1">
       <c r="A136" s="1"/>
       <c r="B136" s="19" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C136" s="20" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D136" s="20" t="s">
         <v>11</v>
@@ -7194,7 +7197,7 @@
       </c>
       <c r="G136" s="21"/>
       <c r="H136" s="19" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="I136" s="1"/>
       <c r="J136" s="1"/>
@@ -7218,10 +7221,10 @@
     <row r="137" ht="18.75" customHeight="1">
       <c r="A137" s="1"/>
       <c r="B137" s="19" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C137" s="20" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D137" s="20" t="s">
         <v>53</v>
@@ -7234,7 +7237,7 @@
       </c>
       <c r="G137" s="21"/>
       <c r="H137" s="19" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="I137" s="1"/>
       <c r="J137" s="1"/>
@@ -7261,7 +7264,7 @@
         <v>0</v>
       </c>
       <c r="C138" s="5" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D138" s="6"/>
       <c r="E138" s="4"/>
@@ -7332,7 +7335,7 @@
     <row r="140" ht="18.75" customHeight="1">
       <c r="A140" s="1"/>
       <c r="B140" s="29" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C140" s="30" t="s">
         <v>27</v>
@@ -7346,7 +7349,7 @@
       </c>
       <c r="G140" s="32"/>
       <c r="H140" s="29" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="I140" s="1"/>
       <c r="J140" s="1"/>
@@ -7370,7 +7373,7 @@
     <row r="141" ht="18.75" customHeight="1">
       <c r="A141" s="1"/>
       <c r="B141" s="29" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C141" s="30" t="s">
         <v>27</v>
@@ -7386,7 +7389,7 @@
       </c>
       <c r="G141" s="32"/>
       <c r="H141" s="29" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="I141" s="1"/>
       <c r="J141" s="1"/>
@@ -7410,10 +7413,10 @@
     <row r="142" ht="18.75" customHeight="1">
       <c r="A142" s="1"/>
       <c r="B142" s="12" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C142" s="13" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D142" s="13" t="s">
         <v>27</v>
@@ -7426,7 +7429,7 @@
       </c>
       <c r="G142" s="14"/>
       <c r="H142" s="12" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="I142" s="1"/>
       <c r="J142" s="1"/>
@@ -7450,10 +7453,10 @@
     <row r="143" ht="18.75" customHeight="1">
       <c r="A143" s="1"/>
       <c r="B143" s="12" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C143" s="13" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D143" s="13" t="s">
         <v>27</v>
@@ -7466,7 +7469,7 @@
       </c>
       <c r="G143" s="14"/>
       <c r="H143" s="12" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="I143" s="1"/>
       <c r="J143" s="1"/>
@@ -7490,7 +7493,7 @@
     <row r="144" ht="18.75" customHeight="1">
       <c r="A144" s="1"/>
       <c r="B144" s="29" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C144" s="30" t="s">
         <v>27</v>
@@ -7506,7 +7509,7 @@
       </c>
       <c r="G144" s="32"/>
       <c r="H144" s="29" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="I144" s="1"/>
       <c r="J144" s="1"/>
@@ -7530,7 +7533,7 @@
     <row r="145" ht="18.75" customHeight="1">
       <c r="A145" s="1"/>
       <c r="B145" s="12" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C145" s="13" t="s">
         <v>27</v>
@@ -7546,7 +7549,7 @@
       </c>
       <c r="G145" s="14"/>
       <c r="H145" s="12" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="I145" s="1"/>
       <c r="J145" s="1"/>
@@ -7570,7 +7573,7 @@
     <row r="146" ht="18.75" customHeight="1">
       <c r="A146" s="1"/>
       <c r="B146" s="12" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C146" s="13" t="s">
         <v>27</v>
@@ -7586,7 +7589,7 @@
       </c>
       <c r="G146" s="14"/>
       <c r="H146" s="12" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="I146" s="1"/>
       <c r="J146" s="1"/>
@@ -7610,7 +7613,7 @@
     <row r="147" ht="18.75" customHeight="1">
       <c r="A147" s="1"/>
       <c r="B147" s="12" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C147" s="13" t="s">
         <v>27</v>
@@ -7626,7 +7629,7 @@
       </c>
       <c r="G147" s="14"/>
       <c r="H147" s="12" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="I147" s="1"/>
       <c r="J147" s="1"/>
@@ -7650,7 +7653,7 @@
     <row r="148" ht="18.75" customHeight="1">
       <c r="A148" s="1"/>
       <c r="B148" s="12" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C148" s="13" t="s">
         <v>27</v>
@@ -7666,7 +7669,7 @@
       </c>
       <c r="G148" s="14"/>
       <c r="H148" s="29" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="I148" s="1"/>
       <c r="J148" s="1"/>
@@ -7690,7 +7693,7 @@
     <row r="149" ht="18.75" customHeight="1">
       <c r="A149" s="1"/>
       <c r="B149" s="12" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C149" s="13" t="s">
         <v>27</v>
@@ -7706,7 +7709,7 @@
       </c>
       <c r="G149" s="14"/>
       <c r="H149" s="29" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="I149" s="1"/>
       <c r="J149" s="1"/>
@@ -7730,21 +7733,21 @@
     <row r="150" ht="18.75" customHeight="1">
       <c r="A150" s="1"/>
       <c r="B150" s="12" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C150" s="13" t="s">
         <v>25</v>
       </c>
       <c r="D150" s="13"/>
       <c r="E150" s="12" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="F150" s="14">
         <v>19.0</v>
       </c>
       <c r="G150" s="14"/>
       <c r="H150" s="12" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="I150" s="1"/>
       <c r="J150" s="1"/>
@@ -7768,21 +7771,21 @@
     <row r="151" ht="18.75" customHeight="1">
       <c r="A151" s="1"/>
       <c r="B151" s="12" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C151" s="13" t="s">
         <v>25</v>
       </c>
       <c r="D151" s="13"/>
       <c r="E151" s="12" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="F151" s="14">
         <v>40.0</v>
       </c>
       <c r="G151" s="14"/>
       <c r="H151" s="12" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="I151" s="1"/>
       <c r="J151" s="1"/>
@@ -7806,21 +7809,21 @@
     <row r="152" ht="18.75" customHeight="1">
       <c r="A152" s="1"/>
       <c r="B152" s="12" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C152" s="13" t="s">
         <v>25</v>
       </c>
       <c r="D152" s="13"/>
       <c r="E152" s="12" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="F152" s="14">
         <v>19.0</v>
       </c>
       <c r="G152" s="14"/>
       <c r="H152" s="12" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="I152" s="1"/>
       <c r="J152" s="1"/>
@@ -7844,21 +7847,21 @@
     <row r="153" ht="18.75" customHeight="1">
       <c r="A153" s="1"/>
       <c r="B153" s="12" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C153" s="13" t="s">
         <v>25</v>
       </c>
       <c r="D153" s="13"/>
       <c r="E153" s="12" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="F153" s="14">
         <v>40.0</v>
       </c>
       <c r="G153" s="14"/>
       <c r="H153" s="12" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="I153" s="1"/>
       <c r="J153" s="1"/>
@@ -7885,7 +7888,7 @@
         <v>0</v>
       </c>
       <c r="C154" s="5" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D154" s="6"/>
       <c r="E154" s="4"/>
@@ -7956,14 +7959,14 @@
     <row r="156" ht="18.75" customHeight="1">
       <c r="A156" s="1"/>
       <c r="B156" s="33" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C156" s="34" t="s">
         <v>78</v>
       </c>
       <c r="D156" s="34"/>
       <c r="E156" s="33" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="F156" s="35">
         <v>0.0</v>

</xml_diff>

<commit_message>
Add contact on GR checks.
Define small contacts as all contacts except diffusion resistance, diode, esd, and capacitor.
Update power point diagrams.

Signed-off-by: Mitch Bailey <d.mitch.bailey@gmail.com>
</commit_message>
<xml_diff>
--- a/Document/TR-1um_Drawing_Layer_DR_Table.xlsx
+++ b/Document/TR-1um_Drawing_Layer_DR_Table.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="718" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="707" uniqueCount="319">
   <si>
     <t>#</t>
   </si>
@@ -445,51 +445,36 @@
     <t>ER0020</t>
   </si>
   <si>
+    <t>CO.WS</t>
+  </si>
+  <si>
+    <t>CO(S)</t>
+  </si>
+  <si>
+    <t>Wfix</t>
+  </si>
+  <si>
     <t>CO.S1</t>
   </si>
   <si>
     <t>ER0044</t>
   </si>
   <si>
-    <t>CO.WM</t>
-  </si>
-  <si>
-    <t>CO(M)</t>
-  </si>
-  <si>
-    <t>Wfix</t>
-  </si>
-  <si>
-    <t>CO.WG</t>
-  </si>
-  <si>
-    <t>CO(G)</t>
-  </si>
-  <si>
-    <t>CO.WB</t>
-  </si>
-  <si>
-    <t>CO(B)</t>
-  </si>
-  <si>
-    <t>CO.WC</t>
+    <t>CO.WD</t>
+  </si>
+  <si>
+    <t>CO(D)</t>
+  </si>
+  <si>
+    <t>ERDP05/ERDN05</t>
+  </si>
+  <si>
+    <t>CO.SC</t>
   </si>
   <si>
     <t>CO(C)</t>
   </si>
   <si>
-    <t>CO.WD</t>
-  </si>
-  <si>
-    <t>CO(D)</t>
-  </si>
-  <si>
-    <t>ERDP05/ERDN05</t>
-  </si>
-  <si>
-    <t>CO.SC</t>
-  </si>
-  <si>
     <t>CO.SD</t>
   </si>
   <si>
@@ -692,9 +677,6 @@
   </si>
   <si>
     <t>M1.CO</t>
-  </si>
-  <si>
-    <t>CO(S)</t>
   </si>
   <si>
     <t>Fmin</t>
@@ -1077,7 +1059,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="40">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1155,6 +1137,15 @@
     </xf>
     <xf borderId="1" fillId="3" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="3" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -4408,21 +4399,21 @@
     </row>
     <row r="66" ht="19.5" customHeight="1">
       <c r="A66" s="1"/>
-      <c r="B66" s="12" t="s">
+      <c r="B66" s="24" t="s">
         <v>142</v>
       </c>
-      <c r="C66" s="13" t="s">
+      <c r="C66" s="25" t="s">
         <v>18</v>
       </c>
       <c r="D66" s="13"/>
-      <c r="E66" s="12" t="s">
+      <c r="E66" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="F66" s="14">
+      <c r="F66" s="26">
         <v>1.0</v>
       </c>
-      <c r="G66" s="14"/>
-      <c r="H66" s="12" t="s">
+      <c r="G66" s="26"/>
+      <c r="H66" s="24" t="s">
         <v>143</v>
       </c>
       <c r="I66" s="1"/>
@@ -4446,24 +4437,24 @@
     </row>
     <row r="67" ht="19.5" customHeight="1">
       <c r="A67" s="1"/>
-      <c r="B67" s="12" t="s">
+      <c r="B67" s="27" t="s">
         <v>144</v>
       </c>
-      <c r="C67" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="D67" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="E67" s="12" t="s">
-        <v>38</v>
+      <c r="C67" s="25" t="s">
+        <v>145</v>
+      </c>
+      <c r="D67" s="13"/>
+      <c r="E67" s="24" t="s">
+        <v>146</v>
       </c>
       <c r="F67" s="14">
         <v>1.0</v>
       </c>
-      <c r="G67" s="14"/>
+      <c r="G67" s="26">
+        <v>1.0</v>
+      </c>
       <c r="H67" s="12" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="I67" s="1"/>
       <c r="J67" s="1"/>
@@ -4485,25 +4476,25 @@
       <c r="Z67" s="1"/>
     </row>
     <row r="68" ht="19.5" customHeight="1">
-      <c r="A68" s="1"/>
+      <c r="A68" s="28"/>
       <c r="B68" s="12" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C68" s="13" t="s">
-        <v>147</v>
-      </c>
-      <c r="D68" s="13"/>
+        <v>18</v>
+      </c>
+      <c r="D68" s="13" t="s">
+        <v>18</v>
+      </c>
       <c r="E68" s="12" t="s">
-        <v>148</v>
+        <v>38</v>
       </c>
       <c r="F68" s="14">
         <v>1.0</v>
       </c>
-      <c r="G68" s="14">
-        <v>1.0</v>
-      </c>
+      <c r="G68" s="14"/>
       <c r="H68" s="12" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="I68" s="1"/>
       <c r="J68" s="1"/>
@@ -4534,16 +4525,16 @@
       </c>
       <c r="D69" s="13"/>
       <c r="E69" s="12" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="F69" s="14">
-        <v>1.0</v>
+        <v>1.2</v>
       </c>
       <c r="G69" s="14">
-        <v>1.0</v>
+        <v>1.2</v>
       </c>
       <c r="H69" s="12" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="I69" s="1"/>
       <c r="J69" s="1"/>
@@ -4566,25 +4557,23 @@
     </row>
     <row r="70" ht="19.5" customHeight="1">
       <c r="A70" s="1"/>
-      <c r="B70" s="24" t="s">
-        <v>151</v>
-      </c>
-      <c r="C70" s="25" t="s">
+      <c r="B70" s="12" t="s">
         <v>152</v>
       </c>
-      <c r="D70" s="13"/>
+      <c r="C70" s="13" t="s">
+        <v>153</v>
+      </c>
+      <c r="D70" s="13" t="s">
+        <v>18</v>
+      </c>
       <c r="E70" s="12" t="s">
-        <v>148</v>
+        <v>38</v>
       </c>
       <c r="F70" s="14">
-        <v>1.0</v>
-      </c>
-      <c r="G70" s="14">
-        <v>1.0</v>
-      </c>
-      <c r="H70" s="12" t="s">
-        <v>143</v>
-      </c>
+        <v>1.2</v>
+      </c>
+      <c r="G70" s="14"/>
+      <c r="H70" s="12"/>
       <c r="I70" s="1"/>
       <c r="J70" s="1"/>
       <c r="K70" s="1"/>
@@ -4607,21 +4596,21 @@
     <row r="71" ht="19.5" customHeight="1">
       <c r="A71" s="1"/>
       <c r="B71" s="12" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C71" s="13" t="s">
-        <v>154</v>
-      </c>
-      <c r="D71" s="13"/>
+        <v>150</v>
+      </c>
+      <c r="D71" s="13" t="s">
+        <v>18</v>
+      </c>
       <c r="E71" s="12" t="s">
-        <v>148</v>
+        <v>38</v>
       </c>
       <c r="F71" s="14">
         <v>1.2</v>
       </c>
-      <c r="G71" s="14">
-        <v>1.2</v>
-      </c>
+      <c r="G71" s="14"/>
       <c r="H71" s="12"/>
       <c r="I71" s="1"/>
       <c r="J71" s="1"/>
@@ -4648,18 +4637,18 @@
         <v>155</v>
       </c>
       <c r="C72" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="D72" s="13" t="s">
         <v>156</v>
       </c>
-      <c r="D72" s="13"/>
       <c r="E72" s="12" t="s">
-        <v>148</v>
+        <v>59</v>
       </c>
       <c r="F72" s="14">
         <v>1.2</v>
       </c>
-      <c r="G72" s="14">
-        <v>1.2</v>
-      </c>
+      <c r="G72" s="14"/>
       <c r="H72" s="12" t="s">
         <v>157</v>
       </c>
@@ -4688,19 +4677,21 @@
         <v>158</v>
       </c>
       <c r="C73" s="13" t="s">
-        <v>154</v>
+        <v>18</v>
       </c>
       <c r="D73" s="13" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="E73" s="12" t="s">
-        <v>38</v>
+        <v>59</v>
       </c>
       <c r="F73" s="14">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="G73" s="14"/>
-      <c r="H73" s="12"/>
+      <c r="H73" s="12" t="s">
+        <v>159</v>
+      </c>
       <c r="I73" s="1"/>
       <c r="J73" s="1"/>
       <c r="K73" s="1"/>
@@ -4723,22 +4714,24 @@
     <row r="74" ht="19.5" customHeight="1">
       <c r="A74" s="1"/>
       <c r="B74" s="12" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C74" s="13" t="s">
-        <v>156</v>
+        <v>18</v>
       </c>
       <c r="D74" s="13" t="s">
-        <v>18</v>
+        <v>53</v>
       </c>
       <c r="E74" s="12" t="s">
-        <v>38</v>
+        <v>59</v>
       </c>
       <c r="F74" s="14">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="G74" s="14"/>
-      <c r="H74" s="12"/>
+      <c r="H74" s="12" t="s">
+        <v>161</v>
+      </c>
       <c r="I74" s="1"/>
       <c r="J74" s="1"/>
       <c r="K74" s="1"/>
@@ -4761,23 +4754,23 @@
     <row r="75" ht="19.5" customHeight="1">
       <c r="A75" s="1"/>
       <c r="B75" s="12" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C75" s="13" t="s">
-        <v>156</v>
+        <v>18</v>
       </c>
       <c r="D75" s="13" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="E75" s="12" t="s">
-        <v>59</v>
+        <v>38</v>
       </c>
       <c r="F75" s="14">
-        <v>1.2</v>
+        <v>1.0</v>
       </c>
       <c r="G75" s="14"/>
       <c r="H75" s="12" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="I75" s="1"/>
       <c r="J75" s="1"/>
@@ -4801,13 +4794,13 @@
     <row r="76" ht="19.5" customHeight="1">
       <c r="A76" s="1"/>
       <c r="B76" s="12" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C76" s="13" t="s">
         <v>18</v>
       </c>
       <c r="D76" s="13" t="s">
-        <v>11</v>
+        <v>166</v>
       </c>
       <c r="E76" s="12" t="s">
         <v>59</v>
@@ -4817,7 +4810,7 @@
       </c>
       <c r="G76" s="14"/>
       <c r="H76" s="12" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="I76" s="1"/>
       <c r="J76" s="1"/>
@@ -4838,27 +4831,19 @@
       <c r="Y76" s="1"/>
       <c r="Z76" s="1"/>
     </row>
-    <row r="77" ht="19.5" customHeight="1">
+    <row r="77" ht="18.75" customHeight="1">
       <c r="A77" s="1"/>
-      <c r="B77" s="12" t="s">
-        <v>165</v>
-      </c>
-      <c r="C77" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="D77" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="E77" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="F77" s="14">
-        <v>0.8</v>
-      </c>
-      <c r="G77" s="14"/>
-      <c r="H77" s="12" t="s">
-        <v>166</v>
-      </c>
+      <c r="B77" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C77" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="D77" s="6"/>
+      <c r="E77" s="4"/>
+      <c r="F77" s="7"/>
+      <c r="G77" s="7"/>
+      <c r="H77" s="4"/>
       <c r="I77" s="1"/>
       <c r="J77" s="1"/>
       <c r="K77" s="1"/>
@@ -4880,24 +4865,26 @@
     </row>
     <row r="78" ht="19.5" customHeight="1">
       <c r="A78" s="1"/>
-      <c r="B78" s="12" t="s">
-        <v>167</v>
-      </c>
-      <c r="C78" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="D78" s="13" t="s">
-        <v>168</v>
-      </c>
-      <c r="E78" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="F78" s="14">
-        <v>1.0</v>
-      </c>
-      <c r="G78" s="14"/>
-      <c r="H78" s="12" t="s">
-        <v>169</v>
+      <c r="B78" s="29" t="s">
+        <v>2</v>
+      </c>
+      <c r="C78" s="30" t="s">
+        <v>3</v>
+      </c>
+      <c r="D78" s="30" t="s">
+        <v>4</v>
+      </c>
+      <c r="E78" s="29" t="s">
+        <v>5</v>
+      </c>
+      <c r="F78" s="31" t="s">
+        <v>6</v>
+      </c>
+      <c r="G78" s="31" t="s">
+        <v>7</v>
+      </c>
+      <c r="H78" s="29" t="s">
+        <v>8</v>
       </c>
       <c r="I78" s="1"/>
       <c r="J78" s="1"/>
@@ -4920,24 +4907,26 @@
     </row>
     <row r="79" ht="19.5" customHeight="1">
       <c r="A79" s="1"/>
-      <c r="B79" s="12" t="s">
+      <c r="B79" s="19" t="s">
+        <v>169</v>
+      </c>
+      <c r="C79" s="20" t="s">
         <v>170</v>
       </c>
-      <c r="C79" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="D79" s="13" t="s">
+      <c r="D79" s="20" t="s">
         <v>171</v>
       </c>
-      <c r="E79" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="F79" s="14">
-        <v>0.8</v>
-      </c>
-      <c r="G79" s="14"/>
-      <c r="H79" s="12" t="s">
-        <v>172</v>
+      <c r="E79" s="19" t="s">
+        <v>67</v>
+      </c>
+      <c r="F79" s="21">
+        <v>2.8</v>
+      </c>
+      <c r="G79" s="21">
+        <v>20.0</v>
+      </c>
+      <c r="H79" s="19" t="s">
+        <v>68</v>
       </c>
       <c r="I79" s="1"/>
       <c r="J79" s="1"/>
@@ -4958,19 +4947,29 @@
       <c r="Y79" s="1"/>
       <c r="Z79" s="1"/>
     </row>
-    <row r="80" ht="18.75" customHeight="1">
+    <row r="80" ht="19.5" customHeight="1">
       <c r="A80" s="1"/>
-      <c r="B80" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C80" s="5" t="s">
+      <c r="B80" s="19" t="s">
+        <v>172</v>
+      </c>
+      <c r="C80" s="20" t="s">
+        <v>170</v>
+      </c>
+      <c r="D80" s="20" t="s">
         <v>173</v>
       </c>
-      <c r="D80" s="6"/>
-      <c r="E80" s="4"/>
-      <c r="F80" s="7"/>
-      <c r="G80" s="7"/>
-      <c r="H80" s="4"/>
+      <c r="E80" s="19" t="s">
+        <v>96</v>
+      </c>
+      <c r="F80" s="21">
+        <v>13.0</v>
+      </c>
+      <c r="G80" s="21">
+        <v>100.0</v>
+      </c>
+      <c r="H80" s="19" t="s">
+        <v>68</v>
+      </c>
       <c r="I80" s="1"/>
       <c r="J80" s="1"/>
       <c r="K80" s="1"/>
@@ -4992,26 +4991,24 @@
     </row>
     <row r="81" ht="19.5" customHeight="1">
       <c r="A81" s="1"/>
-      <c r="B81" s="26" t="s">
-        <v>2</v>
-      </c>
-      <c r="C81" s="27" t="s">
-        <v>3</v>
-      </c>
-      <c r="D81" s="27" t="s">
-        <v>4</v>
-      </c>
-      <c r="E81" s="26" t="s">
-        <v>5</v>
-      </c>
-      <c r="F81" s="28" t="s">
-        <v>6</v>
-      </c>
-      <c r="G81" s="28" t="s">
-        <v>7</v>
-      </c>
-      <c r="H81" s="26" t="s">
-        <v>8</v>
+      <c r="B81" s="19" t="s">
+        <v>174</v>
+      </c>
+      <c r="C81" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="D81" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="E81" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="F81" s="21">
+        <v>1.0</v>
+      </c>
+      <c r="G81" s="21"/>
+      <c r="H81" s="19" t="s">
+        <v>175</v>
       </c>
       <c r="I81" s="1"/>
       <c r="J81" s="1"/>
@@ -5035,25 +5032,21 @@
     <row r="82" ht="19.5" customHeight="1">
       <c r="A82" s="1"/>
       <c r="B82" s="19" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C82" s="20" t="s">
-        <v>175</v>
-      </c>
-      <c r="D82" s="20" t="s">
-        <v>176</v>
-      </c>
+        <v>177</v>
+      </c>
+      <c r="D82" s="20"/>
       <c r="E82" s="19" t="s">
-        <v>67</v>
+        <v>35</v>
       </c>
       <c r="F82" s="21">
-        <v>2.8</v>
-      </c>
-      <c r="G82" s="21">
-        <v>20.0</v>
-      </c>
+        <v>2.0</v>
+      </c>
+      <c r="G82" s="21"/>
       <c r="H82" s="19" t="s">
-        <v>68</v>
+        <v>178</v>
       </c>
       <c r="I82" s="1"/>
       <c r="J82" s="1"/>
@@ -5077,26 +5070,22 @@
     <row r="83" ht="19.5" customHeight="1">
       <c r="A83" s="1"/>
       <c r="B83" s="19" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C83" s="20" t="s">
-        <v>175</v>
+        <v>16</v>
       </c>
       <c r="D83" s="20" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="E83" s="19" t="s">
-        <v>96</v>
+        <v>181</v>
       </c>
       <c r="F83" s="21">
-        <v>13.0</v>
-      </c>
-      <c r="G83" s="21">
-        <v>100.0</v>
-      </c>
-      <c r="H83" s="19" t="s">
-        <v>68</v>
-      </c>
+        <v>1.0</v>
+      </c>
+      <c r="G83" s="21"/>
+      <c r="H83" s="19"/>
       <c r="I83" s="1"/>
       <c r="J83" s="1"/>
       <c r="K83" s="1"/>
@@ -5119,24 +5108,24 @@
     <row r="84" ht="19.5" customHeight="1">
       <c r="A84" s="1"/>
       <c r="B84" s="19" t="s">
-        <v>179</v>
+        <v>135</v>
       </c>
       <c r="C84" s="20" t="s">
-        <v>78</v>
+        <v>177</v>
       </c>
       <c r="D84" s="20" t="s">
-        <v>16</v>
+        <v>53</v>
       </c>
       <c r="E84" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="F84" s="21">
-        <v>1.0</v>
-      </c>
-      <c r="G84" s="21"/>
-      <c r="H84" s="19" t="s">
-        <v>180</v>
-      </c>
+      <c r="F84" s="21" t="s">
+        <v>70</v>
+      </c>
+      <c r="G84" s="21" t="s">
+        <v>70</v>
+      </c>
+      <c r="H84" s="19"/>
       <c r="I84" s="1"/>
       <c r="J84" s="1"/>
       <c r="K84" s="1"/>
@@ -5159,22 +5148,22 @@
     <row r="85" ht="19.5" customHeight="1">
       <c r="A85" s="1"/>
       <c r="B85" s="19" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C85" s="20" t="s">
-        <v>182</v>
-      </c>
-      <c r="D85" s="20"/>
+        <v>16</v>
+      </c>
+      <c r="D85" s="20" t="s">
+        <v>177</v>
+      </c>
       <c r="E85" s="19" t="s">
-        <v>35</v>
+        <v>83</v>
       </c>
       <c r="F85" s="21">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="G85" s="21"/>
-      <c r="H85" s="19" t="s">
-        <v>183</v>
-      </c>
+      <c r="H85" s="19"/>
       <c r="I85" s="1"/>
       <c r="J85" s="1"/>
       <c r="K85" s="1"/>
@@ -5197,19 +5186,19 @@
     <row r="86" ht="19.5" customHeight="1">
       <c r="A86" s="1"/>
       <c r="B86" s="19" t="s">
+        <v>183</v>
+      </c>
+      <c r="C86" s="20" t="s">
+        <v>177</v>
+      </c>
+      <c r="D86" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="E86" s="19" t="s">
         <v>184</v>
       </c>
-      <c r="C86" s="20" t="s">
-        <v>16</v>
-      </c>
-      <c r="D86" s="20" t="s">
-        <v>185</v>
-      </c>
-      <c r="E86" s="19" t="s">
-        <v>186</v>
-      </c>
       <c r="F86" s="21">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="G86" s="21"/>
       <c r="H86" s="19"/>
@@ -5234,25 +5223,27 @@
     </row>
     <row r="87" ht="19.5" customHeight="1">
       <c r="A87" s="1"/>
-      <c r="B87" s="19" t="s">
-        <v>135</v>
-      </c>
-      <c r="C87" s="20" t="s">
-        <v>182</v>
-      </c>
-      <c r="D87" s="20" t="s">
-        <v>53</v>
-      </c>
-      <c r="E87" s="19" t="s">
-        <v>38</v>
-      </c>
-      <c r="F87" s="21" t="s">
-        <v>70</v>
-      </c>
-      <c r="G87" s="21" t="s">
-        <v>70</v>
-      </c>
-      <c r="H87" s="19"/>
+      <c r="B87" s="12" t="s">
+        <v>185</v>
+      </c>
+      <c r="C87" s="13" t="s">
+        <v>186</v>
+      </c>
+      <c r="D87" s="13" t="s">
+        <v>187</v>
+      </c>
+      <c r="E87" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F87" s="14">
+        <v>4.0</v>
+      </c>
+      <c r="G87" s="14">
+        <v>20.0</v>
+      </c>
+      <c r="H87" s="12" t="s">
+        <v>68</v>
+      </c>
       <c r="I87" s="1"/>
       <c r="J87" s="1"/>
       <c r="K87" s="1"/>
@@ -5274,23 +5265,27 @@
     </row>
     <row r="88" ht="19.5" customHeight="1">
       <c r="A88" s="1"/>
-      <c r="B88" s="19" t="s">
-        <v>187</v>
-      </c>
-      <c r="C88" s="20" t="s">
-        <v>16</v>
-      </c>
-      <c r="D88" s="20" t="s">
-        <v>182</v>
-      </c>
-      <c r="E88" s="19" t="s">
-        <v>83</v>
-      </c>
-      <c r="F88" s="21">
-        <v>0.0</v>
-      </c>
-      <c r="G88" s="21"/>
-      <c r="H88" s="19"/>
+      <c r="B88" s="12" t="s">
+        <v>188</v>
+      </c>
+      <c r="C88" s="13" t="s">
+        <v>186</v>
+      </c>
+      <c r="D88" s="13" t="s">
+        <v>189</v>
+      </c>
+      <c r="E88" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="F88" s="14">
+        <v>20.0</v>
+      </c>
+      <c r="G88" s="14">
+        <v>100.0</v>
+      </c>
+      <c r="H88" s="12" t="s">
+        <v>68</v>
+      </c>
       <c r="I88" s="1"/>
       <c r="J88" s="1"/>
       <c r="K88" s="1"/>
@@ -5312,23 +5307,25 @@
     </row>
     <row r="89" ht="19.5" customHeight="1">
       <c r="A89" s="1"/>
-      <c r="B89" s="19" t="s">
-        <v>188</v>
-      </c>
-      <c r="C89" s="20" t="s">
-        <v>182</v>
-      </c>
-      <c r="D89" s="20" t="s">
-        <v>10</v>
-      </c>
-      <c r="E89" s="19" t="s">
-        <v>189</v>
-      </c>
-      <c r="F89" s="21">
-        <v>0.0</v>
-      </c>
-      <c r="G89" s="21"/>
-      <c r="H89" s="19"/>
+      <c r="B89" s="12" t="s">
+        <v>190</v>
+      </c>
+      <c r="C89" s="13" t="s">
+        <v>186</v>
+      </c>
+      <c r="D89" s="13" t="s">
+        <v>186</v>
+      </c>
+      <c r="E89" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F89" s="14">
+        <v>2.0</v>
+      </c>
+      <c r="G89" s="14"/>
+      <c r="H89" s="12" t="s">
+        <v>191</v>
+      </c>
       <c r="I89" s="1"/>
       <c r="J89" s="1"/>
       <c r="K89" s="1"/>
@@ -5350,27 +5347,21 @@
     </row>
     <row r="90" ht="19.5" customHeight="1">
       <c r="A90" s="1"/>
-      <c r="B90" s="12" t="s">
-        <v>190</v>
-      </c>
-      <c r="C90" s="13" t="s">
-        <v>191</v>
-      </c>
-      <c r="D90" s="13" t="s">
+      <c r="B90" s="19" t="s">
         <v>192</v>
       </c>
-      <c r="E90" s="12" t="s">
-        <v>67</v>
-      </c>
-      <c r="F90" s="14">
-        <v>4.0</v>
-      </c>
-      <c r="G90" s="14">
-        <v>20.0</v>
-      </c>
-      <c r="H90" s="12" t="s">
-        <v>68</v>
-      </c>
+      <c r="C90" s="20" t="s">
+        <v>193</v>
+      </c>
+      <c r="D90" s="20"/>
+      <c r="E90" s="19" t="s">
+        <v>35</v>
+      </c>
+      <c r="F90" s="21">
+        <v>1.0</v>
+      </c>
+      <c r="G90" s="21"/>
+      <c r="H90" s="19"/>
       <c r="I90" s="1"/>
       <c r="J90" s="1"/>
       <c r="K90" s="1"/>
@@ -5392,26 +5383,24 @@
     </row>
     <row r="91" ht="19.5" customHeight="1">
       <c r="A91" s="1"/>
-      <c r="B91" s="12" t="s">
-        <v>193</v>
-      </c>
-      <c r="C91" s="13" t="s">
-        <v>191</v>
-      </c>
-      <c r="D91" s="13" t="s">
+      <c r="B91" s="19" t="s">
         <v>194</v>
       </c>
-      <c r="E91" s="12" t="s">
-        <v>96</v>
-      </c>
-      <c r="F91" s="14">
-        <v>20.0</v>
-      </c>
-      <c r="G91" s="14">
-        <v>100.0</v>
-      </c>
-      <c r="H91" s="12" t="s">
-        <v>68</v>
+      <c r="C91" s="20" t="s">
+        <v>195</v>
+      </c>
+      <c r="D91" s="20"/>
+      <c r="E91" s="19" t="s">
+        <v>67</v>
+      </c>
+      <c r="F91" s="21">
+        <v>1.0</v>
+      </c>
+      <c r="G91" s="21">
+        <v>97.5</v>
+      </c>
+      <c r="H91" s="19" t="s">
+        <v>196</v>
       </c>
       <c r="I91" s="1"/>
       <c r="J91" s="1"/>
@@ -5434,25 +5423,23 @@
     </row>
     <row r="92" ht="19.5" customHeight="1">
       <c r="A92" s="1"/>
-      <c r="B92" s="12" t="s">
-        <v>195</v>
-      </c>
-      <c r="C92" s="13" t="s">
-        <v>191</v>
-      </c>
-      <c r="D92" s="13" t="s">
-        <v>191</v>
-      </c>
-      <c r="E92" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="F92" s="14">
-        <v>2.0</v>
-      </c>
-      <c r="G92" s="14"/>
-      <c r="H92" s="12" t="s">
-        <v>196</v>
-      </c>
+      <c r="B92" s="19" t="s">
+        <v>197</v>
+      </c>
+      <c r="C92" s="20" t="s">
+        <v>193</v>
+      </c>
+      <c r="D92" s="20" t="s">
+        <v>198</v>
+      </c>
+      <c r="E92" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="F92" s="21">
+        <v>1.5</v>
+      </c>
+      <c r="G92" s="21"/>
+      <c r="H92" s="19"/>
       <c r="I92" s="1"/>
       <c r="J92" s="1"/>
       <c r="K92" s="1"/>
@@ -5475,14 +5462,16 @@
     <row r="93" ht="19.5" customHeight="1">
       <c r="A93" s="1"/>
       <c r="B93" s="19" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C93" s="20" t="s">
-        <v>198</v>
-      </c>
-      <c r="D93" s="20"/>
+        <v>193</v>
+      </c>
+      <c r="D93" s="20" t="s">
+        <v>200</v>
+      </c>
       <c r="E93" s="19" t="s">
-        <v>35</v>
+        <v>59</v>
       </c>
       <c r="F93" s="21">
         <v>1.0</v>
@@ -5511,23 +5500,23 @@
     <row r="94" ht="19.5" customHeight="1">
       <c r="A94" s="1"/>
       <c r="B94" s="19" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C94" s="20" t="s">
-        <v>200</v>
+        <v>153</v>
       </c>
       <c r="D94" s="20"/>
       <c r="E94" s="19" t="s">
-        <v>67</v>
+        <v>146</v>
       </c>
       <c r="F94" s="21">
-        <v>1.0</v>
+        <v>1.2</v>
       </c>
       <c r="G94" s="21">
-        <v>97.5</v>
+        <v>1.2</v>
       </c>
       <c r="H94" s="19" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="I94" s="1"/>
       <c r="J94" s="1"/>
@@ -5551,22 +5540,26 @@
     <row r="95" ht="19.5" customHeight="1">
       <c r="A95" s="1"/>
       <c r="B95" s="19" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C95" s="20" t="s">
-        <v>198</v>
+        <v>153</v>
       </c>
       <c r="D95" s="20" t="s">
-        <v>203</v>
+        <v>153</v>
       </c>
       <c r="E95" s="19" t="s">
-        <v>59</v>
+        <v>204</v>
       </c>
       <c r="F95" s="21">
-        <v>1.5</v>
-      </c>
-      <c r="G95" s="21"/>
-      <c r="H95" s="19"/>
+        <v>1.2</v>
+      </c>
+      <c r="G95" s="21">
+        <v>1.2</v>
+      </c>
+      <c r="H95" s="19" t="s">
+        <v>205</v>
+      </c>
       <c r="I95" s="1"/>
       <c r="J95" s="1"/>
       <c r="K95" s="1"/>
@@ -5589,22 +5582,24 @@
     <row r="96" ht="19.5" customHeight="1">
       <c r="A96" s="1"/>
       <c r="B96" s="19" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C96" s="20" t="s">
-        <v>198</v>
+        <v>153</v>
       </c>
       <c r="D96" s="20" t="s">
-        <v>205</v>
+        <v>66</v>
       </c>
       <c r="E96" s="19" t="s">
         <v>59</v>
       </c>
       <c r="F96" s="21">
-        <v>1.0</v>
+        <v>2.9</v>
       </c>
       <c r="G96" s="21"/>
-      <c r="H96" s="19"/>
+      <c r="H96" s="19" t="s">
+        <v>207</v>
+      </c>
       <c r="I96" s="1"/>
       <c r="J96" s="1"/>
       <c r="K96" s="1"/>
@@ -5627,23 +5622,23 @@
     <row r="97" ht="19.5" customHeight="1">
       <c r="A97" s="1"/>
       <c r="B97" s="19" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="C97" s="20" t="s">
-        <v>154</v>
-      </c>
-      <c r="D97" s="20"/>
+        <v>153</v>
+      </c>
+      <c r="D97" s="20" t="s">
+        <v>53</v>
+      </c>
       <c r="E97" s="19" t="s">
-        <v>148</v>
+        <v>59</v>
       </c>
       <c r="F97" s="21">
         <v>1.2</v>
       </c>
-      <c r="G97" s="21">
-        <v>1.2</v>
-      </c>
+      <c r="G97" s="21"/>
       <c r="H97" s="19" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="I97" s="1"/>
       <c r="J97" s="1"/>
@@ -5664,29 +5659,19 @@
       <c r="Y97" s="1"/>
       <c r="Z97" s="1"/>
     </row>
-    <row r="98" ht="19.5" customHeight="1">
+    <row r="98" ht="18.75" customHeight="1">
       <c r="A98" s="1"/>
-      <c r="B98" s="19" t="s">
-        <v>208</v>
-      </c>
-      <c r="C98" s="20" t="s">
-        <v>154</v>
-      </c>
-      <c r="D98" s="20" t="s">
-        <v>154</v>
-      </c>
-      <c r="E98" s="19" t="s">
-        <v>209</v>
-      </c>
-      <c r="F98" s="21">
-        <v>1.2</v>
-      </c>
-      <c r="G98" s="21">
-        <v>1.2</v>
-      </c>
-      <c r="H98" s="19" t="s">
+      <c r="B98" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C98" s="5" t="s">
         <v>210</v>
       </c>
+      <c r="D98" s="6"/>
+      <c r="E98" s="4"/>
+      <c r="F98" s="7"/>
+      <c r="G98" s="7"/>
+      <c r="H98" s="4"/>
       <c r="I98" s="1"/>
       <c r="J98" s="1"/>
       <c r="K98" s="1"/>
@@ -5708,24 +5693,26 @@
     </row>
     <row r="99" ht="19.5" customHeight="1">
       <c r="A99" s="1"/>
-      <c r="B99" s="19" t="s">
-        <v>211</v>
-      </c>
-      <c r="C99" s="20" t="s">
-        <v>154</v>
-      </c>
-      <c r="D99" s="20" t="s">
-        <v>66</v>
-      </c>
-      <c r="E99" s="19" t="s">
-        <v>59</v>
-      </c>
-      <c r="F99" s="21">
-        <v>2.9</v>
-      </c>
-      <c r="G99" s="21"/>
-      <c r="H99" s="19" t="s">
-        <v>212</v>
+      <c r="B99" s="29" t="s">
+        <v>2</v>
+      </c>
+      <c r="C99" s="30" t="s">
+        <v>3</v>
+      </c>
+      <c r="D99" s="30" t="s">
+        <v>4</v>
+      </c>
+      <c r="E99" s="29" t="s">
+        <v>5</v>
+      </c>
+      <c r="F99" s="31" t="s">
+        <v>6</v>
+      </c>
+      <c r="G99" s="31" t="s">
+        <v>7</v>
+      </c>
+      <c r="H99" s="29" t="s">
+        <v>8</v>
       </c>
       <c r="I99" s="1"/>
       <c r="J99" s="1"/>
@@ -5748,24 +5735,22 @@
     </row>
     <row r="100" ht="19.5" customHeight="1">
       <c r="A100" s="1"/>
-      <c r="B100" s="19" t="s">
-        <v>213</v>
-      </c>
-      <c r="C100" s="20" t="s">
-        <v>154</v>
-      </c>
-      <c r="D100" s="20" t="s">
-        <v>53</v>
-      </c>
-      <c r="E100" s="19" t="s">
-        <v>59</v>
-      </c>
-      <c r="F100" s="21">
-        <v>1.2</v>
-      </c>
-      <c r="G100" s="21"/>
-      <c r="H100" s="19" t="s">
-        <v>214</v>
+      <c r="B100" s="12" t="s">
+        <v>211</v>
+      </c>
+      <c r="C100" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D100" s="13"/>
+      <c r="E100" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="F100" s="14">
+        <v>1.8</v>
+      </c>
+      <c r="G100" s="14"/>
+      <c r="H100" s="12" t="s">
+        <v>212</v>
       </c>
       <c r="I100" s="1"/>
       <c r="J100" s="1"/>
@@ -5786,19 +5771,25 @@
       <c r="Y100" s="1"/>
       <c r="Z100" s="1"/>
     </row>
-    <row r="101" ht="18.75" customHeight="1">
+    <row r="101" ht="19.5" customHeight="1">
       <c r="A101" s="1"/>
-      <c r="B101" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C101" s="5" t="s">
-        <v>215</v>
-      </c>
-      <c r="D101" s="6"/>
-      <c r="E101" s="4"/>
-      <c r="F101" s="7"/>
-      <c r="G101" s="7"/>
-      <c r="H101" s="4"/>
+      <c r="B101" s="12" t="s">
+        <v>213</v>
+      </c>
+      <c r="C101" s="13" t="s">
+        <v>214</v>
+      </c>
+      <c r="D101" s="13"/>
+      <c r="E101" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="F101" s="14">
+        <v>10.0</v>
+      </c>
+      <c r="G101" s="14"/>
+      <c r="H101" s="12" t="s">
+        <v>212</v>
+      </c>
       <c r="I101" s="1"/>
       <c r="J101" s="1"/>
       <c r="K101" s="1"/>
@@ -5820,26 +5811,24 @@
     </row>
     <row r="102" ht="19.5" customHeight="1">
       <c r="A102" s="1"/>
-      <c r="B102" s="26" t="s">
-        <v>2</v>
-      </c>
-      <c r="C102" s="27" t="s">
-        <v>3</v>
-      </c>
-      <c r="D102" s="27" t="s">
-        <v>4</v>
-      </c>
-      <c r="E102" s="26" t="s">
-        <v>5</v>
-      </c>
-      <c r="F102" s="28" t="s">
-        <v>6</v>
-      </c>
-      <c r="G102" s="28" t="s">
-        <v>7</v>
-      </c>
-      <c r="H102" s="26" t="s">
-        <v>8</v>
+      <c r="B102" s="12" t="s">
+        <v>215</v>
+      </c>
+      <c r="C102" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D102" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="E102" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F102" s="14">
+        <v>1.4</v>
+      </c>
+      <c r="G102" s="14"/>
+      <c r="H102" s="12" t="s">
+        <v>216</v>
       </c>
       <c r="I102" s="1"/>
       <c r="J102" s="1"/>
@@ -5863,21 +5852,25 @@
     <row r="103" ht="19.5" customHeight="1">
       <c r="A103" s="1"/>
       <c r="B103" s="12" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C103" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="D103" s="13"/>
+        <v>218</v>
+      </c>
+      <c r="D103" s="13" t="s">
+        <v>218</v>
+      </c>
       <c r="E103" s="12" t="s">
-        <v>35</v>
+        <v>219</v>
       </c>
       <c r="F103" s="14">
-        <v>1.8</v>
-      </c>
-      <c r="G103" s="14"/>
+        <v>10.0</v>
+      </c>
+      <c r="G103" s="14">
+        <v>10.0</v>
+      </c>
       <c r="H103" s="12" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="I103" s="1"/>
       <c r="J103" s="1"/>
@@ -5901,21 +5894,23 @@
     <row r="104" ht="19.5" customHeight="1">
       <c r="A104" s="1"/>
       <c r="B104" s="12" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="C104" s="13" t="s">
-        <v>219</v>
-      </c>
-      <c r="D104" s="13"/>
+        <v>21</v>
+      </c>
+      <c r="D104" s="13" t="s">
+        <v>145</v>
+      </c>
       <c r="E104" s="12" t="s">
-        <v>35</v>
+        <v>222</v>
       </c>
       <c r="F104" s="14">
-        <v>10.0</v>
+        <v>0.8</v>
       </c>
       <c r="G104" s="14"/>
       <c r="H104" s="12" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="I104" s="1"/>
       <c r="J104" s="1"/>
@@ -5939,23 +5934,23 @@
     <row r="105" ht="19.5" customHeight="1">
       <c r="A105" s="1"/>
       <c r="B105" s="12" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="C105" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="D105" s="13" t="s">
-        <v>21</v>
+      <c r="D105" s="25" t="s">
+        <v>225</v>
       </c>
       <c r="E105" s="12" t="s">
-        <v>38</v>
+        <v>222</v>
       </c>
       <c r="F105" s="14">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="G105" s="14"/>
       <c r="H105" s="12" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
       <c r="I105" s="1"/>
       <c r="J105" s="1"/>
@@ -5979,25 +5974,23 @@
     <row r="106" ht="19.5" customHeight="1">
       <c r="A106" s="1"/>
       <c r="B106" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="C106" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D106" s="13" t="s">
+        <v>196</v>
+      </c>
+      <c r="E106" s="12" t="s">
         <v>222</v>
       </c>
-      <c r="C106" s="13" t="s">
-        <v>223</v>
-      </c>
-      <c r="D106" s="13" t="s">
-        <v>223</v>
-      </c>
-      <c r="E106" s="12" t="s">
-        <v>224</v>
-      </c>
       <c r="F106" s="14">
-        <v>10.0</v>
-      </c>
-      <c r="G106" s="14">
-        <v>10.0</v>
-      </c>
+        <v>1.2</v>
+      </c>
+      <c r="G106" s="14"/>
       <c r="H106" s="12" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="I106" s="1"/>
       <c r="J106" s="1"/>
@@ -6021,19 +6014,19 @@
     <row r="107" ht="19.5" customHeight="1">
       <c r="A107" s="1"/>
       <c r="B107" s="12" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="C107" s="13" t="s">
+        <v>214</v>
+      </c>
+      <c r="D107" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="D107" s="13" t="s">
-        <v>227</v>
-      </c>
       <c r="E107" s="12" t="s">
-        <v>228</v>
+        <v>38</v>
       </c>
       <c r="F107" s="14">
-        <v>0.8</v>
+        <v>2.0</v>
       </c>
       <c r="G107" s="14"/>
       <c r="H107" s="12" t="s">
@@ -6060,24 +6053,24 @@
     </row>
     <row r="108" ht="19.5" customHeight="1">
       <c r="A108" s="1"/>
-      <c r="B108" s="12" t="s">
+      <c r="B108" s="19" t="s">
         <v>230</v>
       </c>
-      <c r="C108" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="D108" s="25" t="s">
+      <c r="C108" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="D108" s="20"/>
+      <c r="E108" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="F108" s="21">
+        <v>1.4</v>
+      </c>
+      <c r="G108" s="21">
+        <v>1.4</v>
+      </c>
+      <c r="H108" s="19" t="s">
         <v>231</v>
-      </c>
-      <c r="E108" s="12" t="s">
-        <v>228</v>
-      </c>
-      <c r="F108" s="14">
-        <v>1.3</v>
-      </c>
-      <c r="G108" s="14"/>
-      <c r="H108" s="12" t="s">
-        <v>214</v>
       </c>
       <c r="I108" s="1"/>
       <c r="J108" s="1"/>
@@ -6100,23 +6093,23 @@
     </row>
     <row r="109" ht="19.5" customHeight="1">
       <c r="A109" s="1"/>
-      <c r="B109" s="12" t="s">
+      <c r="B109" s="19" t="s">
         <v>232</v>
       </c>
-      <c r="C109" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="D109" s="13" t="s">
-        <v>201</v>
-      </c>
-      <c r="E109" s="12" t="s">
-        <v>228</v>
-      </c>
-      <c r="F109" s="14">
-        <v>1.2</v>
-      </c>
-      <c r="G109" s="14"/>
-      <c r="H109" s="12" t="s">
+      <c r="C109" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="D109" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="E109" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="F109" s="21">
+        <v>1.5</v>
+      </c>
+      <c r="G109" s="21"/>
+      <c r="H109" s="19" t="s">
         <v>233</v>
       </c>
       <c r="I109" s="1"/>
@@ -6140,23 +6133,23 @@
     </row>
     <row r="110" ht="19.5" customHeight="1">
       <c r="A110" s="1"/>
-      <c r="B110" s="12" t="s">
+      <c r="B110" s="19" t="s">
         <v>234</v>
       </c>
-      <c r="C110" s="13" t="s">
-        <v>219</v>
-      </c>
-      <c r="D110" s="13" t="s">
+      <c r="C110" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="D110" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="E110" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="F110" s="14">
-        <v>2.0</v>
-      </c>
-      <c r="G110" s="14"/>
-      <c r="H110" s="12" t="s">
+      <c r="E110" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="F110" s="21">
+        <v>1.0</v>
+      </c>
+      <c r="G110" s="21"/>
+      <c r="H110" s="19" t="s">
         <v>235</v>
       </c>
       <c r="I110" s="1"/>
@@ -6186,16 +6179,16 @@
       <c r="C111" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="D111" s="20"/>
+      <c r="D111" s="20" t="s">
+        <v>78</v>
+      </c>
       <c r="E111" s="19" t="s">
-        <v>148</v>
+        <v>38</v>
       </c>
       <c r="F111" s="21">
-        <v>1.4</v>
-      </c>
-      <c r="G111" s="21">
-        <v>1.4</v>
-      </c>
+        <v>1.2</v>
+      </c>
+      <c r="G111" s="21"/>
       <c r="H111" s="19" t="s">
         <v>237</v>
       </c>
@@ -6227,13 +6220,13 @@
         <v>23</v>
       </c>
       <c r="D112" s="20" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="E112" s="19" t="s">
         <v>38</v>
       </c>
       <c r="F112" s="21">
-        <v>1.5</v>
+        <v>1.0</v>
       </c>
       <c r="G112" s="21"/>
       <c r="H112" s="19" t="s">
@@ -6267,13 +6260,13 @@
         <v>23</v>
       </c>
       <c r="D113" s="20" t="s">
-        <v>21</v>
+        <v>196</v>
       </c>
       <c r="E113" s="19" t="s">
-        <v>59</v>
+        <v>38</v>
       </c>
       <c r="F113" s="21">
-        <v>1.0</v>
+        <v>1.4</v>
       </c>
       <c r="G113" s="21"/>
       <c r="H113" s="19" t="s">
@@ -6300,23 +6293,21 @@
     </row>
     <row r="114" ht="19.5" customHeight="1">
       <c r="A114" s="1"/>
-      <c r="B114" s="19" t="s">
+      <c r="B114" s="12" t="s">
         <v>242</v>
       </c>
-      <c r="C114" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="D114" s="20" t="s">
-        <v>78</v>
-      </c>
-      <c r="E114" s="19" t="s">
-        <v>38</v>
-      </c>
-      <c r="F114" s="21">
-        <v>1.2</v>
-      </c>
-      <c r="G114" s="21"/>
-      <c r="H114" s="19" t="s">
+      <c r="C114" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D114" s="13"/>
+      <c r="E114" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="F114" s="14">
+        <v>3.0</v>
+      </c>
+      <c r="G114" s="14"/>
+      <c r="H114" s="12" t="s">
         <v>243</v>
       </c>
       <c r="I114" s="1"/>
@@ -6340,23 +6331,23 @@
     </row>
     <row r="115" ht="19.5" customHeight="1">
       <c r="A115" s="1"/>
-      <c r="B115" s="19" t="s">
+      <c r="B115" s="12" t="s">
         <v>244</v>
       </c>
-      <c r="C115" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="D115" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="E115" s="19" t="s">
+      <c r="C115" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D115" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="E115" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="F115" s="21">
-        <v>1.0</v>
-      </c>
-      <c r="G115" s="21"/>
-      <c r="H115" s="19" t="s">
+      <c r="F115" s="14">
+        <v>2.0</v>
+      </c>
+      <c r="G115" s="14"/>
+      <c r="H115" s="12" t="s">
         <v>245</v>
       </c>
       <c r="I115" s="1"/>
@@ -6380,24 +6371,24 @@
     </row>
     <row r="116" ht="19.5" customHeight="1">
       <c r="A116" s="1"/>
-      <c r="B116" s="19" t="s">
+      <c r="B116" s="12" t="s">
         <v>246</v>
       </c>
-      <c r="C116" s="20" t="s">
+      <c r="C116" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D116" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="D116" s="20" t="s">
-        <v>201</v>
-      </c>
-      <c r="E116" s="19" t="s">
-        <v>38</v>
-      </c>
-      <c r="F116" s="21">
-        <v>1.4</v>
-      </c>
-      <c r="G116" s="21"/>
-      <c r="H116" s="19" t="s">
-        <v>247</v>
+      <c r="E116" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="F116" s="14">
+        <v>1.0</v>
+      </c>
+      <c r="G116" s="14"/>
+      <c r="H116" s="12" t="s">
+        <v>235</v>
       </c>
       <c r="I116" s="1"/>
       <c r="J116" s="1"/>
@@ -6418,25 +6409,19 @@
       <c r="Y116" s="1"/>
       <c r="Z116" s="1"/>
     </row>
-    <row r="117" ht="19.5" customHeight="1">
+    <row r="117" ht="18.75" customHeight="1">
       <c r="A117" s="1"/>
-      <c r="B117" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="C117" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="D117" s="13"/>
-      <c r="E117" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="F117" s="14">
-        <v>3.0</v>
-      </c>
-      <c r="G117" s="14"/>
-      <c r="H117" s="12" t="s">
-        <v>249</v>
-      </c>
+      <c r="B117" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C117" s="5" t="s">
+        <v>247</v>
+      </c>
+      <c r="D117" s="6"/>
+      <c r="E117" s="4"/>
+      <c r="F117" s="7"/>
+      <c r="G117" s="7"/>
+      <c r="H117" s="4"/>
       <c r="I117" s="1"/>
       <c r="J117" s="1"/>
       <c r="K117" s="1"/>
@@ -6456,26 +6441,28 @@
       <c r="Y117" s="1"/>
       <c r="Z117" s="1"/>
     </row>
-    <row r="118" ht="19.5" customHeight="1">
+    <row r="118" ht="18.75" customHeight="1">
       <c r="A118" s="1"/>
-      <c r="B118" s="12" t="s">
-        <v>250</v>
-      </c>
-      <c r="C118" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="D118" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="E118" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="F118" s="14">
-        <v>2.0</v>
-      </c>
-      <c r="G118" s="14"/>
-      <c r="H118" s="12" t="s">
-        <v>251</v>
+      <c r="B118" s="29" t="s">
+        <v>2</v>
+      </c>
+      <c r="C118" s="30" t="s">
+        <v>3</v>
+      </c>
+      <c r="D118" s="30" t="s">
+        <v>4</v>
+      </c>
+      <c r="E118" s="29" t="s">
+        <v>5</v>
+      </c>
+      <c r="F118" s="31" t="s">
+        <v>6</v>
+      </c>
+      <c r="G118" s="31" t="s">
+        <v>7</v>
+      </c>
+      <c r="H118" s="29" t="s">
+        <v>8</v>
       </c>
       <c r="I118" s="1"/>
       <c r="J118" s="1"/>
@@ -6496,26 +6483,28 @@
       <c r="Y118" s="1"/>
       <c r="Z118" s="1"/>
     </row>
-    <row r="119" ht="19.5" customHeight="1">
+    <row r="119" ht="18.75" customHeight="1">
       <c r="A119" s="1"/>
-      <c r="B119" s="12" t="s">
-        <v>252</v>
-      </c>
-      <c r="C119" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="D119" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="E119" s="12" t="s">
-        <v>228</v>
-      </c>
-      <c r="F119" s="14">
-        <v>1.0</v>
-      </c>
-      <c r="G119" s="14"/>
-      <c r="H119" s="12" t="s">
-        <v>241</v>
+      <c r="B119" s="19" t="s">
+        <v>248</v>
+      </c>
+      <c r="C119" s="20" t="s">
+        <v>249</v>
+      </c>
+      <c r="D119" s="20" t="s">
+        <v>250</v>
+      </c>
+      <c r="E119" s="19" t="s">
+        <v>67</v>
+      </c>
+      <c r="F119" s="21">
+        <v>11.0</v>
+      </c>
+      <c r="G119" s="21">
+        <v>60.0</v>
+      </c>
+      <c r="H119" s="19" t="s">
+        <v>68</v>
       </c>
       <c r="I119" s="1"/>
       <c r="J119" s="1"/>
@@ -6538,17 +6527,27 @@
     </row>
     <row r="120" ht="18.75" customHeight="1">
       <c r="A120" s="1"/>
-      <c r="B120" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C120" s="5" t="s">
-        <v>253</v>
-      </c>
-      <c r="D120" s="6"/>
-      <c r="E120" s="4"/>
-      <c r="F120" s="7"/>
-      <c r="G120" s="7"/>
-      <c r="H120" s="4"/>
+      <c r="B120" s="19" t="s">
+        <v>251</v>
+      </c>
+      <c r="C120" s="20" t="s">
+        <v>249</v>
+      </c>
+      <c r="D120" s="20" t="s">
+        <v>252</v>
+      </c>
+      <c r="E120" s="19" t="s">
+        <v>96</v>
+      </c>
+      <c r="F120" s="21">
+        <v>2.0</v>
+      </c>
+      <c r="G120" s="21">
+        <v>30.0</v>
+      </c>
+      <c r="H120" s="19" t="s">
+        <v>68</v>
+      </c>
       <c r="I120" s="1"/>
       <c r="J120" s="1"/>
       <c r="K120" s="1"/>
@@ -6570,26 +6569,24 @@
     </row>
     <row r="121" ht="18.75" customHeight="1">
       <c r="A121" s="1"/>
-      <c r="B121" s="26" t="s">
-        <v>2</v>
-      </c>
-      <c r="C121" s="27" t="s">
-        <v>3</v>
-      </c>
-      <c r="D121" s="27" t="s">
-        <v>4</v>
-      </c>
-      <c r="E121" s="26" t="s">
-        <v>5</v>
-      </c>
-      <c r="F121" s="28" t="s">
-        <v>6</v>
-      </c>
-      <c r="G121" s="28" t="s">
-        <v>7</v>
-      </c>
-      <c r="H121" s="26" t="s">
-        <v>8</v>
+      <c r="B121" s="19" t="s">
+        <v>253</v>
+      </c>
+      <c r="C121" s="20" t="s">
+        <v>254</v>
+      </c>
+      <c r="D121" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="E121" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="F121" s="21">
+        <v>10.0</v>
+      </c>
+      <c r="G121" s="21"/>
+      <c r="H121" s="19" t="s">
+        <v>255</v>
       </c>
       <c r="I121" s="1"/>
       <c r="J121" s="1"/>
@@ -6613,25 +6610,23 @@
     <row r="122" ht="18.75" customHeight="1">
       <c r="A122" s="1"/>
       <c r="B122" s="19" t="s">
+        <v>256</v>
+      </c>
+      <c r="C122" s="20" t="s">
         <v>254</v>
       </c>
-      <c r="C122" s="20" t="s">
-        <v>255</v>
-      </c>
       <c r="D122" s="20" t="s">
-        <v>256</v>
+        <v>180</v>
       </c>
       <c r="E122" s="19" t="s">
-        <v>67</v>
+        <v>181</v>
       </c>
       <c r="F122" s="21">
-        <v>11.0</v>
-      </c>
-      <c r="G122" s="21">
-        <v>60.0</v>
-      </c>
+        <v>1.4</v>
+      </c>
+      <c r="G122" s="21"/>
       <c r="H122" s="19" t="s">
-        <v>68</v>
+        <v>257</v>
       </c>
       <c r="I122" s="1"/>
       <c r="J122" s="1"/>
@@ -6655,25 +6650,23 @@
     <row r="123" ht="18.75" customHeight="1">
       <c r="A123" s="1"/>
       <c r="B123" s="19" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C123" s="20" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D123" s="20" t="s">
-        <v>258</v>
+        <v>18</v>
       </c>
       <c r="E123" s="19" t="s">
-        <v>96</v>
+        <v>38</v>
       </c>
       <c r="F123" s="21">
         <v>2.0</v>
       </c>
-      <c r="G123" s="21">
-        <v>30.0</v>
-      </c>
+      <c r="G123" s="21"/>
       <c r="H123" s="19" t="s">
-        <v>68</v>
+        <v>259</v>
       </c>
       <c r="I123" s="1"/>
       <c r="J123" s="1"/>
@@ -6696,24 +6689,26 @@
     </row>
     <row r="124" ht="18.75" customHeight="1">
       <c r="A124" s="1"/>
-      <c r="B124" s="19" t="s">
-        <v>259</v>
-      </c>
-      <c r="C124" s="20" t="s">
+      <c r="B124" s="12" t="s">
         <v>260</v>
       </c>
-      <c r="D124" s="20" t="s">
-        <v>53</v>
-      </c>
-      <c r="E124" s="19" t="s">
-        <v>38</v>
-      </c>
-      <c r="F124" s="21">
-        <v>10.0</v>
-      </c>
-      <c r="G124" s="21"/>
-      <c r="H124" s="19" t="s">
+      <c r="C124" s="13" t="s">
         <v>261</v>
+      </c>
+      <c r="D124" s="13" t="s">
+        <v>262</v>
+      </c>
+      <c r="E124" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F124" s="14">
+        <v>11.0</v>
+      </c>
+      <c r="G124" s="14">
+        <v>60.0</v>
+      </c>
+      <c r="H124" s="12" t="s">
+        <v>68</v>
       </c>
       <c r="I124" s="1"/>
       <c r="J124" s="1"/>
@@ -6736,24 +6731,26 @@
     </row>
     <row r="125" ht="18.75" customHeight="1">
       <c r="A125" s="1"/>
-      <c r="B125" s="19" t="s">
-        <v>262</v>
-      </c>
-      <c r="C125" s="20" t="s">
-        <v>260</v>
-      </c>
-      <c r="D125" s="20" t="s">
-        <v>185</v>
-      </c>
-      <c r="E125" s="19" t="s">
-        <v>186</v>
-      </c>
-      <c r="F125" s="21">
-        <v>1.4</v>
-      </c>
-      <c r="G125" s="21"/>
-      <c r="H125" s="19" t="s">
+      <c r="B125" s="12" t="s">
         <v>263</v>
+      </c>
+      <c r="C125" s="13" t="s">
+        <v>261</v>
+      </c>
+      <c r="D125" s="13" t="s">
+        <v>252</v>
+      </c>
+      <c r="E125" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="F125" s="14">
+        <v>2.0</v>
+      </c>
+      <c r="G125" s="14">
+        <v>30.0</v>
+      </c>
+      <c r="H125" s="12" t="s">
+        <v>68</v>
       </c>
       <c r="I125" s="1"/>
       <c r="J125" s="1"/>
@@ -6776,24 +6773,24 @@
     </row>
     <row r="126" ht="18.75" customHeight="1">
       <c r="A126" s="1"/>
-      <c r="B126" s="19" t="s">
+      <c r="B126" s="12" t="s">
         <v>264</v>
       </c>
-      <c r="C126" s="20" t="s">
-        <v>260</v>
-      </c>
-      <c r="D126" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="E126" s="19" t="s">
+      <c r="C126" s="13" t="s">
+        <v>265</v>
+      </c>
+      <c r="D126" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E126" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="F126" s="21">
-        <v>2.0</v>
-      </c>
-      <c r="G126" s="21"/>
-      <c r="H126" s="19" t="s">
-        <v>265</v>
+      <c r="F126" s="14">
+        <v>10.0</v>
+      </c>
+      <c r="G126" s="14"/>
+      <c r="H126" s="12" t="s">
+        <v>266</v>
       </c>
       <c r="I126" s="1"/>
       <c r="J126" s="1"/>
@@ -6817,25 +6814,23 @@
     <row r="127" ht="18.75" customHeight="1">
       <c r="A127" s="1"/>
       <c r="B127" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C127" s="13" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D127" s="13" t="s">
+        <v>180</v>
+      </c>
+      <c r="E127" s="12" t="s">
+        <v>181</v>
+      </c>
+      <c r="F127" s="14">
+        <v>1.4</v>
+      </c>
+      <c r="G127" s="14"/>
+      <c r="H127" s="12" t="s">
         <v>268</v>
-      </c>
-      <c r="E127" s="12" t="s">
-        <v>67</v>
-      </c>
-      <c r="F127" s="14">
-        <v>11.0</v>
-      </c>
-      <c r="G127" s="14">
-        <v>60.0</v>
-      </c>
-      <c r="H127" s="12" t="s">
-        <v>68</v>
       </c>
       <c r="I127" s="1"/>
       <c r="J127" s="1"/>
@@ -6862,22 +6857,20 @@
         <v>269</v>
       </c>
       <c r="C128" s="13" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D128" s="13" t="s">
-        <v>258</v>
+        <v>18</v>
       </c>
       <c r="E128" s="12" t="s">
-        <v>96</v>
+        <v>38</v>
       </c>
       <c r="F128" s="14">
         <v>2.0</v>
       </c>
-      <c r="G128" s="14">
-        <v>30.0</v>
-      </c>
+      <c r="G128" s="14"/>
       <c r="H128" s="12" t="s">
-        <v>68</v>
+        <v>270</v>
       </c>
       <c r="I128" s="1"/>
       <c r="J128" s="1"/>
@@ -6900,24 +6893,24 @@
     </row>
     <row r="129" ht="18.75" customHeight="1">
       <c r="A129" s="1"/>
-      <c r="B129" s="12" t="s">
-        <v>270</v>
-      </c>
-      <c r="C129" s="13" t="s">
+      <c r="B129" s="19" t="s">
         <v>271</v>
       </c>
-      <c r="D129" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="E129" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="F129" s="14">
-        <v>10.0</v>
-      </c>
-      <c r="G129" s="14"/>
-      <c r="H129" s="12" t="s">
+      <c r="C129" s="20" t="s">
         <v>272</v>
+      </c>
+      <c r="D129" s="20"/>
+      <c r="E129" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="F129" s="21">
+        <v>3.0</v>
+      </c>
+      <c r="G129" s="21">
+        <v>3.0</v>
+      </c>
+      <c r="H129" s="19" t="s">
+        <v>273</v>
       </c>
       <c r="I129" s="1"/>
       <c r="J129" s="1"/>
@@ -6940,24 +6933,24 @@
     </row>
     <row r="130" ht="18.75" customHeight="1">
       <c r="A130" s="1"/>
-      <c r="B130" s="12" t="s">
-        <v>273</v>
-      </c>
-      <c r="C130" s="13" t="s">
-        <v>271</v>
-      </c>
-      <c r="D130" s="13" t="s">
-        <v>185</v>
-      </c>
-      <c r="E130" s="12" t="s">
-        <v>186</v>
-      </c>
-      <c r="F130" s="14">
-        <v>1.4</v>
-      </c>
-      <c r="G130" s="14"/>
-      <c r="H130" s="12" t="s">
+      <c r="B130" s="19" t="s">
         <v>274</v>
+      </c>
+      <c r="C130" s="20" t="s">
+        <v>272</v>
+      </c>
+      <c r="D130" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="E130" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="F130" s="21">
+        <v>1.6</v>
+      </c>
+      <c r="G130" s="21"/>
+      <c r="H130" s="19" t="s">
+        <v>275</v>
       </c>
       <c r="I130" s="1"/>
       <c r="J130" s="1"/>
@@ -6980,24 +6973,24 @@
     </row>
     <row r="131" ht="18.75" customHeight="1">
       <c r="A131" s="1"/>
-      <c r="B131" s="12" t="s">
-        <v>275</v>
-      </c>
-      <c r="C131" s="13" t="s">
-        <v>271</v>
-      </c>
-      <c r="D131" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="E131" s="12" t="s">
+      <c r="B131" s="19" t="s">
+        <v>276</v>
+      </c>
+      <c r="C131" s="20" t="s">
+        <v>277</v>
+      </c>
+      <c r="D131" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="E131" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="F131" s="14">
-        <v>2.0</v>
-      </c>
-      <c r="G131" s="14"/>
-      <c r="H131" s="12" t="s">
-        <v>276</v>
+      <c r="F131" s="21">
+        <v>7.0</v>
+      </c>
+      <c r="G131" s="21"/>
+      <c r="H131" s="19" t="s">
+        <v>278</v>
       </c>
       <c r="I131" s="1"/>
       <c r="J131" s="1"/>
@@ -7021,23 +7014,23 @@
     <row r="132" ht="18.75" customHeight="1">
       <c r="A132" s="1"/>
       <c r="B132" s="19" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C132" s="20" t="s">
-        <v>278</v>
-      </c>
-      <c r="D132" s="20"/>
+        <v>280</v>
+      </c>
+      <c r="D132" s="20" t="s">
+        <v>78</v>
+      </c>
       <c r="E132" s="19" t="s">
-        <v>148</v>
+        <v>38</v>
       </c>
       <c r="F132" s="21">
         <v>3.0</v>
       </c>
-      <c r="G132" s="21">
-        <v>3.0</v>
-      </c>
+      <c r="G132" s="21"/>
       <c r="H132" s="19" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="I132" s="1"/>
       <c r="J132" s="1"/>
@@ -7061,23 +7054,23 @@
     <row r="133" ht="18.75" customHeight="1">
       <c r="A133" s="1"/>
       <c r="B133" s="19" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C133" s="20" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="D133" s="20" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="E133" s="19" t="s">
-        <v>38</v>
+        <v>59</v>
       </c>
       <c r="F133" s="21">
-        <v>1.6</v>
+        <v>4.0</v>
       </c>
       <c r="G133" s="21"/>
       <c r="H133" s="19" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="I133" s="1"/>
       <c r="J133" s="1"/>
@@ -7101,23 +7094,23 @@
     <row r="134" ht="18.75" customHeight="1">
       <c r="A134" s="1"/>
       <c r="B134" s="19" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C134" s="20" t="s">
-        <v>283</v>
+        <v>272</v>
       </c>
       <c r="D134" s="20" t="s">
-        <v>78</v>
+        <v>53</v>
       </c>
       <c r="E134" s="19" t="s">
-        <v>38</v>
+        <v>59</v>
       </c>
       <c r="F134" s="21">
-        <v>7.0</v>
+        <v>4.0</v>
       </c>
       <c r="G134" s="21"/>
       <c r="H134" s="19" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="I134" s="1"/>
       <c r="J134" s="1"/>
@@ -7140,25 +7133,17 @@
     </row>
     <row r="135" ht="18.75" customHeight="1">
       <c r="A135" s="1"/>
-      <c r="B135" s="19" t="s">
-        <v>285</v>
-      </c>
-      <c r="C135" s="20" t="s">
+      <c r="B135" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C135" s="5" t="s">
         <v>286</v>
       </c>
-      <c r="D135" s="20" t="s">
-        <v>78</v>
-      </c>
-      <c r="E135" s="19" t="s">
-        <v>38</v>
-      </c>
-      <c r="F135" s="21">
-        <v>3.0</v>
-      </c>
-      <c r="G135" s="21"/>
-      <c r="H135" s="19" t="s">
-        <v>287</v>
-      </c>
+      <c r="D135" s="6"/>
+      <c r="E135" s="4"/>
+      <c r="F135" s="7"/>
+      <c r="G135" s="7"/>
+      <c r="H135" s="4"/>
       <c r="I135" s="1"/>
       <c r="J135" s="1"/>
       <c r="K135" s="1"/>
@@ -7180,24 +7165,26 @@
     </row>
     <row r="136" ht="18.75" customHeight="1">
       <c r="A136" s="1"/>
-      <c r="B136" s="19" t="s">
-        <v>288</v>
-      </c>
-      <c r="C136" s="20" t="s">
-        <v>278</v>
-      </c>
-      <c r="D136" s="20" t="s">
-        <v>11</v>
-      </c>
-      <c r="E136" s="19" t="s">
-        <v>59</v>
-      </c>
-      <c r="F136" s="21">
-        <v>4.0</v>
-      </c>
-      <c r="G136" s="21"/>
-      <c r="H136" s="19" t="s">
-        <v>289</v>
+      <c r="B136" s="29" t="s">
+        <v>2</v>
+      </c>
+      <c r="C136" s="30" t="s">
+        <v>3</v>
+      </c>
+      <c r="D136" s="30" t="s">
+        <v>4</v>
+      </c>
+      <c r="E136" s="29" t="s">
+        <v>5</v>
+      </c>
+      <c r="F136" s="31" t="s">
+        <v>6</v>
+      </c>
+      <c r="G136" s="31" t="s">
+        <v>7</v>
+      </c>
+      <c r="H136" s="29" t="s">
+        <v>8</v>
       </c>
       <c r="I136" s="1"/>
       <c r="J136" s="1"/>
@@ -7220,24 +7207,22 @@
     </row>
     <row r="137" ht="18.75" customHeight="1">
       <c r="A137" s="1"/>
-      <c r="B137" s="19" t="s">
-        <v>290</v>
-      </c>
-      <c r="C137" s="20" t="s">
-        <v>278</v>
-      </c>
-      <c r="D137" s="20" t="s">
-        <v>53</v>
-      </c>
-      <c r="E137" s="19" t="s">
-        <v>59</v>
-      </c>
-      <c r="F137" s="21">
-        <v>4.0</v>
-      </c>
-      <c r="G137" s="21"/>
-      <c r="H137" s="19" t="s">
-        <v>291</v>
+      <c r="B137" s="32" t="s">
+        <v>287</v>
+      </c>
+      <c r="C137" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="D137" s="33"/>
+      <c r="E137" s="32" t="s">
+        <v>35</v>
+      </c>
+      <c r="F137" s="34">
+        <v>70.0</v>
+      </c>
+      <c r="G137" s="35"/>
+      <c r="H137" s="32" t="s">
+        <v>288</v>
       </c>
       <c r="I137" s="1"/>
       <c r="J137" s="1"/>
@@ -7260,17 +7245,25 @@
     </row>
     <row r="138" ht="18.75" customHeight="1">
       <c r="A138" s="1"/>
-      <c r="B138" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C138" s="5" t="s">
-        <v>292</v>
-      </c>
-      <c r="D138" s="6"/>
-      <c r="E138" s="4"/>
-      <c r="F138" s="7"/>
-      <c r="G138" s="7"/>
-      <c r="H138" s="4"/>
+      <c r="B138" s="32" t="s">
+        <v>289</v>
+      </c>
+      <c r="C138" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="D138" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="E138" s="32" t="s">
+        <v>38</v>
+      </c>
+      <c r="F138" s="34">
+        <v>64.0</v>
+      </c>
+      <c r="G138" s="35"/>
+      <c r="H138" s="32" t="s">
+        <v>290</v>
+      </c>
       <c r="I138" s="1"/>
       <c r="J138" s="1"/>
       <c r="K138" s="1"/>
@@ -7292,26 +7285,24 @@
     </row>
     <row r="139" ht="18.75" customHeight="1">
       <c r="A139" s="1"/>
-      <c r="B139" s="26" t="s">
-        <v>2</v>
-      </c>
-      <c r="C139" s="27" t="s">
-        <v>3</v>
-      </c>
-      <c r="D139" s="27" t="s">
-        <v>4</v>
-      </c>
-      <c r="E139" s="26" t="s">
-        <v>5</v>
-      </c>
-      <c r="F139" s="28" t="s">
-        <v>6</v>
-      </c>
-      <c r="G139" s="28" t="s">
-        <v>7</v>
-      </c>
-      <c r="H139" s="26" t="s">
-        <v>8</v>
+      <c r="B139" s="12" t="s">
+        <v>291</v>
+      </c>
+      <c r="C139" s="13" t="s">
+        <v>292</v>
+      </c>
+      <c r="D139" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="E139" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="F139" s="14">
+        <v>5.0</v>
+      </c>
+      <c r="G139" s="14"/>
+      <c r="H139" s="12" t="s">
+        <v>293</v>
       </c>
       <c r="I139" s="1"/>
       <c r="J139" s="1"/>
@@ -7334,22 +7325,24 @@
     </row>
     <row r="140" ht="18.75" customHeight="1">
       <c r="A140" s="1"/>
-      <c r="B140" s="29" t="s">
-        <v>293</v>
-      </c>
-      <c r="C140" s="30" t="s">
+      <c r="B140" s="12" t="s">
+        <v>294</v>
+      </c>
+      <c r="C140" s="13" t="s">
+        <v>295</v>
+      </c>
+      <c r="D140" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="D140" s="30"/>
-      <c r="E140" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="F140" s="31">
-        <v>70.0</v>
-      </c>
-      <c r="G140" s="32"/>
-      <c r="H140" s="29" t="s">
-        <v>294</v>
+      <c r="E140" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="F140" s="14">
+        <v>5.0</v>
+      </c>
+      <c r="G140" s="14"/>
+      <c r="H140" s="12" t="s">
+        <v>296</v>
       </c>
       <c r="I140" s="1"/>
       <c r="J140" s="1"/>
@@ -7372,24 +7365,24 @@
     </row>
     <row r="141" ht="18.75" customHeight="1">
       <c r="A141" s="1"/>
-      <c r="B141" s="29" t="s">
-        <v>295</v>
-      </c>
-      <c r="C141" s="30" t="s">
+      <c r="B141" s="32" t="s">
+        <v>297</v>
+      </c>
+      <c r="C141" s="33" t="s">
         <v>27</v>
       </c>
-      <c r="D141" s="30" t="s">
-        <v>27</v>
-      </c>
-      <c r="E141" s="29" t="s">
-        <v>38</v>
-      </c>
-      <c r="F141" s="31">
-        <v>64.0</v>
-      </c>
-      <c r="G141" s="32"/>
-      <c r="H141" s="29" t="s">
-        <v>296</v>
+      <c r="D141" s="33" t="s">
+        <v>30</v>
+      </c>
+      <c r="E141" s="32" t="s">
+        <v>59</v>
+      </c>
+      <c r="F141" s="34">
+        <v>10.0</v>
+      </c>
+      <c r="G141" s="35"/>
+      <c r="H141" s="32" t="s">
+        <v>298</v>
       </c>
       <c r="I141" s="1"/>
       <c r="J141" s="1"/>
@@ -7413,23 +7406,23 @@
     <row r="142" ht="18.75" customHeight="1">
       <c r="A142" s="1"/>
       <c r="B142" s="12" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="C142" s="13" t="s">
-        <v>298</v>
+        <v>27</v>
       </c>
       <c r="D142" s="13" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="E142" s="12" t="s">
-        <v>228</v>
+        <v>38</v>
       </c>
       <c r="F142" s="14">
-        <v>5.0</v>
+        <v>14.0</v>
       </c>
       <c r="G142" s="14"/>
       <c r="H142" s="12" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="I142" s="1"/>
       <c r="J142" s="1"/>
@@ -7453,23 +7446,23 @@
     <row r="143" ht="18.75" customHeight="1">
       <c r="A143" s="1"/>
       <c r="B143" s="12" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C143" s="13" t="s">
-        <v>301</v>
+        <v>27</v>
       </c>
       <c r="D143" s="13" t="s">
-        <v>27</v>
+        <v>53</v>
       </c>
       <c r="E143" s="12" t="s">
-        <v>228</v>
+        <v>38</v>
       </c>
       <c r="F143" s="14">
-        <v>5.0</v>
+        <v>14.0</v>
       </c>
       <c r="G143" s="14"/>
       <c r="H143" s="12" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="I143" s="1"/>
       <c r="J143" s="1"/>
@@ -7492,24 +7485,24 @@
     </row>
     <row r="144" ht="18.75" customHeight="1">
       <c r="A144" s="1"/>
-      <c r="B144" s="29" t="s">
+      <c r="B144" s="12" t="s">
+        <v>302</v>
+      </c>
+      <c r="C144" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="D144" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="E144" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F144" s="14">
+        <v>14.0</v>
+      </c>
+      <c r="G144" s="14"/>
+      <c r="H144" s="12" t="s">
         <v>303</v>
-      </c>
-      <c r="C144" s="30" t="s">
-        <v>27</v>
-      </c>
-      <c r="D144" s="30" t="s">
-        <v>30</v>
-      </c>
-      <c r="E144" s="29" t="s">
-        <v>59</v>
-      </c>
-      <c r="F144" s="31">
-        <v>10.0</v>
-      </c>
-      <c r="G144" s="32"/>
-      <c r="H144" s="29" t="s">
-        <v>304</v>
       </c>
       <c r="I144" s="1"/>
       <c r="J144" s="1"/>
@@ -7533,13 +7526,13 @@
     <row r="145" ht="18.75" customHeight="1">
       <c r="A145" s="1"/>
       <c r="B145" s="12" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C145" s="13" t="s">
         <v>27</v>
       </c>
       <c r="D145" s="13" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="E145" s="12" t="s">
         <v>38</v>
@@ -7548,8 +7541,8 @@
         <v>14.0</v>
       </c>
       <c r="G145" s="14"/>
-      <c r="H145" s="12" t="s">
-        <v>306</v>
+      <c r="H145" s="32" t="s">
+        <v>305</v>
       </c>
       <c r="I145" s="1"/>
       <c r="J145" s="1"/>
@@ -7573,13 +7566,13 @@
     <row r="146" ht="18.75" customHeight="1">
       <c r="A146" s="1"/>
       <c r="B146" s="12" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C146" s="13" t="s">
         <v>27</v>
       </c>
       <c r="D146" s="13" t="s">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="E146" s="12" t="s">
         <v>38</v>
@@ -7588,8 +7581,8 @@
         <v>14.0</v>
       </c>
       <c r="G146" s="14"/>
-      <c r="H146" s="12" t="s">
-        <v>306</v>
+      <c r="H146" s="32" t="s">
+        <v>307</v>
       </c>
       <c r="I146" s="1"/>
       <c r="J146" s="1"/>
@@ -7616,20 +7609,18 @@
         <v>308</v>
       </c>
       <c r="C147" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="D147" s="13" t="s">
-        <v>78</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="D147" s="13"/>
       <c r="E147" s="12" t="s">
-        <v>38</v>
+        <v>309</v>
       </c>
       <c r="F147" s="14">
-        <v>14.0</v>
+        <v>19.0</v>
       </c>
       <c r="G147" s="14"/>
       <c r="H147" s="12" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="I147" s="1"/>
       <c r="J147" s="1"/>
@@ -7653,23 +7644,21 @@
     <row r="148" ht="18.75" customHeight="1">
       <c r="A148" s="1"/>
       <c r="B148" s="12" t="s">
+        <v>311</v>
+      </c>
+      <c r="C148" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D148" s="13"/>
+      <c r="E148" s="12" t="s">
+        <v>312</v>
+      </c>
+      <c r="F148" s="14">
+        <v>40.0</v>
+      </c>
+      <c r="G148" s="14"/>
+      <c r="H148" s="12" t="s">
         <v>310</v>
-      </c>
-      <c r="C148" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="D148" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="E148" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="F148" s="14">
-        <v>14.0</v>
-      </c>
-      <c r="G148" s="14"/>
-      <c r="H148" s="29" t="s">
-        <v>311</v>
       </c>
       <c r="I148" s="1"/>
       <c r="J148" s="1"/>
@@ -7693,23 +7682,21 @@
     <row r="149" ht="18.75" customHeight="1">
       <c r="A149" s="1"/>
       <c r="B149" s="12" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C149" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="D149" s="13" t="s">
         <v>25</v>
       </c>
+      <c r="D149" s="13"/>
       <c r="E149" s="12" t="s">
-        <v>38</v>
+        <v>309</v>
       </c>
       <c r="F149" s="14">
-        <v>14.0</v>
+        <v>19.0</v>
       </c>
       <c r="G149" s="14"/>
-      <c r="H149" s="29" t="s">
-        <v>313</v>
+      <c r="H149" s="12" t="s">
+        <v>314</v>
       </c>
       <c r="I149" s="1"/>
       <c r="J149" s="1"/>
@@ -7733,21 +7720,21 @@
     <row r="150" ht="18.75" customHeight="1">
       <c r="A150" s="1"/>
       <c r="B150" s="12" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C150" s="13" t="s">
         <v>25</v>
       </c>
       <c r="D150" s="13"/>
       <c r="E150" s="12" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="F150" s="14">
-        <v>19.0</v>
+        <v>40.0</v>
       </c>
       <c r="G150" s="14"/>
       <c r="H150" s="12" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="I150" s="1"/>
       <c r="J150" s="1"/>
@@ -7770,23 +7757,17 @@
     </row>
     <row r="151" ht="18.75" customHeight="1">
       <c r="A151" s="1"/>
-      <c r="B151" s="12" t="s">
-        <v>317</v>
-      </c>
-      <c r="C151" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="D151" s="13"/>
-      <c r="E151" s="12" t="s">
-        <v>318</v>
-      </c>
-      <c r="F151" s="14">
-        <v>40.0</v>
-      </c>
-      <c r="G151" s="14"/>
-      <c r="H151" s="12" t="s">
+      <c r="B151" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C151" s="5" t="s">
         <v>316</v>
       </c>
+      <c r="D151" s="6"/>
+      <c r="E151" s="4"/>
+      <c r="F151" s="7"/>
+      <c r="G151" s="7"/>
+      <c r="H151" s="4"/>
       <c r="I151" s="1"/>
       <c r="J151" s="1"/>
       <c r="K151" s="1"/>
@@ -7808,22 +7789,26 @@
     </row>
     <row r="152" ht="18.75" customHeight="1">
       <c r="A152" s="1"/>
-      <c r="B152" s="12" t="s">
-        <v>319</v>
-      </c>
-      <c r="C152" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="D152" s="13"/>
-      <c r="E152" s="12" t="s">
-        <v>315</v>
-      </c>
-      <c r="F152" s="14">
-        <v>19.0</v>
-      </c>
-      <c r="G152" s="14"/>
-      <c r="H152" s="12" t="s">
-        <v>320</v>
+      <c r="B152" s="29" t="s">
+        <v>2</v>
+      </c>
+      <c r="C152" s="30" t="s">
+        <v>3</v>
+      </c>
+      <c r="D152" s="30" t="s">
+        <v>4</v>
+      </c>
+      <c r="E152" s="29" t="s">
+        <v>5</v>
+      </c>
+      <c r="F152" s="31" t="s">
+        <v>6</v>
+      </c>
+      <c r="G152" s="31" t="s">
+        <v>7</v>
+      </c>
+      <c r="H152" s="29" t="s">
+        <v>8</v>
       </c>
       <c r="I152" s="1"/>
       <c r="J152" s="1"/>
@@ -7846,23 +7831,21 @@
     </row>
     <row r="153" ht="18.75" customHeight="1">
       <c r="A153" s="1"/>
-      <c r="B153" s="12" t="s">
-        <v>321</v>
-      </c>
-      <c r="C153" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="D153" s="13"/>
-      <c r="E153" s="12" t="s">
+      <c r="B153" s="36" t="s">
+        <v>317</v>
+      </c>
+      <c r="C153" s="37" t="s">
+        <v>78</v>
+      </c>
+      <c r="D153" s="37"/>
+      <c r="E153" s="36" t="s">
         <v>318</v>
       </c>
-      <c r="F153" s="14">
-        <v>40.0</v>
-      </c>
-      <c r="G153" s="14"/>
-      <c r="H153" s="12" t="s">
-        <v>320</v>
-      </c>
+      <c r="F153" s="38">
+        <v>0.0</v>
+      </c>
+      <c r="G153" s="39"/>
+      <c r="H153" s="36"/>
       <c r="I153" s="1"/>
       <c r="J153" s="1"/>
       <c r="K153" s="1"/>
@@ -7884,17 +7867,13 @@
     </row>
     <row r="154" ht="18.75" customHeight="1">
       <c r="A154" s="1"/>
-      <c r="B154" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C154" s="5" t="s">
-        <v>322</v>
-      </c>
-      <c r="D154" s="6"/>
-      <c r="E154" s="4"/>
-      <c r="F154" s="7"/>
-      <c r="G154" s="7"/>
-      <c r="H154" s="4"/>
+      <c r="B154" s="36"/>
+      <c r="C154" s="37"/>
+      <c r="D154" s="37"/>
+      <c r="E154" s="36"/>
+      <c r="F154" s="38"/>
+      <c r="G154" s="39"/>
+      <c r="H154" s="36"/>
       <c r="I154" s="1"/>
       <c r="J154" s="1"/>
       <c r="K154" s="1"/>
@@ -7916,27 +7895,13 @@
     </row>
     <row r="155" ht="18.75" customHeight="1">
       <c r="A155" s="1"/>
-      <c r="B155" s="26" t="s">
-        <v>2</v>
-      </c>
-      <c r="C155" s="27" t="s">
-        <v>3</v>
-      </c>
-      <c r="D155" s="27" t="s">
-        <v>4</v>
-      </c>
-      <c r="E155" s="26" t="s">
-        <v>5</v>
-      </c>
-      <c r="F155" s="28" t="s">
-        <v>6</v>
-      </c>
-      <c r="G155" s="28" t="s">
-        <v>7</v>
-      </c>
-      <c r="H155" s="26" t="s">
-        <v>8</v>
-      </c>
+      <c r="B155" s="1"/>
+      <c r="C155" s="2"/>
+      <c r="D155" s="2"/>
+      <c r="E155" s="1"/>
+      <c r="F155" s="3"/>
+      <c r="G155" s="3"/>
+      <c r="H155" s="1"/>
       <c r="I155" s="1"/>
       <c r="J155" s="1"/>
       <c r="K155" s="1"/>
@@ -7958,21 +7923,13 @@
     </row>
     <row r="156" ht="18.75" customHeight="1">
       <c r="A156" s="1"/>
-      <c r="B156" s="33" t="s">
-        <v>323</v>
-      </c>
-      <c r="C156" s="34" t="s">
-        <v>78</v>
-      </c>
-      <c r="D156" s="34"/>
-      <c r="E156" s="33" t="s">
-        <v>324</v>
-      </c>
-      <c r="F156" s="35">
-        <v>0.0</v>
-      </c>
-      <c r="G156" s="36"/>
-      <c r="H156" s="33"/>
+      <c r="B156" s="1"/>
+      <c r="C156" s="2"/>
+      <c r="D156" s="2"/>
+      <c r="E156" s="1"/>
+      <c r="F156" s="3"/>
+      <c r="G156" s="3"/>
+      <c r="H156" s="1"/>
       <c r="I156" s="1"/>
       <c r="J156" s="1"/>
       <c r="K156" s="1"/>
@@ -7994,13 +7951,13 @@
     </row>
     <row r="157" ht="18.75" customHeight="1">
       <c r="A157" s="1"/>
-      <c r="B157" s="33"/>
-      <c r="C157" s="34"/>
-      <c r="D157" s="34"/>
-      <c r="E157" s="33"/>
-      <c r="F157" s="35"/>
-      <c r="G157" s="36"/>
-      <c r="H157" s="33"/>
+      <c r="B157" s="1"/>
+      <c r="C157" s="2"/>
+      <c r="D157" s="2"/>
+      <c r="E157" s="1"/>
+      <c r="F157" s="3"/>
+      <c r="G157" s="3"/>
+      <c r="H157" s="1"/>
       <c r="I157" s="1"/>
       <c r="J157" s="1"/>
       <c r="K157" s="1"/>
@@ -13508,90 +13465,9 @@
       <c r="Y353" s="1"/>
       <c r="Z353" s="1"/>
     </row>
-    <row r="354" ht="18.75" customHeight="1">
-      <c r="A354" s="1"/>
-      <c r="B354" s="1"/>
-      <c r="C354" s="2"/>
-      <c r="D354" s="2"/>
-      <c r="E354" s="1"/>
-      <c r="F354" s="3"/>
-      <c r="G354" s="3"/>
-      <c r="H354" s="1"/>
-      <c r="I354" s="1"/>
-      <c r="J354" s="1"/>
-      <c r="K354" s="1"/>
-      <c r="L354" s="1"/>
-      <c r="M354" s="1"/>
-      <c r="N354" s="1"/>
-      <c r="O354" s="1"/>
-      <c r="P354" s="1"/>
-      <c r="Q354" s="1"/>
-      <c r="R354" s="1"/>
-      <c r="S354" s="1"/>
-      <c r="T354" s="1"/>
-      <c r="U354" s="1"/>
-      <c r="V354" s="1"/>
-      <c r="W354" s="1"/>
-      <c r="X354" s="1"/>
-      <c r="Y354" s="1"/>
-      <c r="Z354" s="1"/>
-    </row>
-    <row r="355" ht="18.75" customHeight="1">
-      <c r="A355" s="1"/>
-      <c r="B355" s="1"/>
-      <c r="C355" s="2"/>
-      <c r="D355" s="2"/>
-      <c r="E355" s="1"/>
-      <c r="F355" s="3"/>
-      <c r="G355" s="3"/>
-      <c r="H355" s="1"/>
-      <c r="I355" s="1"/>
-      <c r="J355" s="1"/>
-      <c r="K355" s="1"/>
-      <c r="L355" s="1"/>
-      <c r="M355" s="1"/>
-      <c r="N355" s="1"/>
-      <c r="O355" s="1"/>
-      <c r="P355" s="1"/>
-      <c r="Q355" s="1"/>
-      <c r="R355" s="1"/>
-      <c r="S355" s="1"/>
-      <c r="T355" s="1"/>
-      <c r="U355" s="1"/>
-      <c r="V355" s="1"/>
-      <c r="W355" s="1"/>
-      <c r="X355" s="1"/>
-      <c r="Y355" s="1"/>
-      <c r="Z355" s="1"/>
-    </row>
-    <row r="356" ht="18.75" customHeight="1">
-      <c r="A356" s="1"/>
-      <c r="B356" s="1"/>
-      <c r="C356" s="2"/>
-      <c r="D356" s="2"/>
-      <c r="E356" s="1"/>
-      <c r="F356" s="3"/>
-      <c r="G356" s="3"/>
-      <c r="H356" s="1"/>
-      <c r="I356" s="1"/>
-      <c r="J356" s="1"/>
-      <c r="K356" s="1"/>
-      <c r="L356" s="1"/>
-      <c r="M356" s="1"/>
-      <c r="N356" s="1"/>
-      <c r="O356" s="1"/>
-      <c r="P356" s="1"/>
-      <c r="Q356" s="1"/>
-      <c r="R356" s="1"/>
-      <c r="S356" s="1"/>
-      <c r="T356" s="1"/>
-      <c r="U356" s="1"/>
-      <c r="V356" s="1"/>
-      <c r="W356" s="1"/>
-      <c r="X356" s="1"/>
-      <c r="Y356" s="1"/>
-      <c r="Z356" s="1"/>
-    </row>
+    <row r="354" ht="15.75" customHeight="1"/>
+    <row r="355" ht="15.75" customHeight="1"/>
+    <row r="356" ht="15.75" customHeight="1"/>
     <row r="357" ht="15.75" customHeight="1"/>
     <row r="358" ht="15.75" customHeight="1"/>
     <row r="359" ht="15.75" customHeight="1"/>
@@ -14232,9 +14108,6 @@
     <row r="994" ht="15.75" customHeight="1"/>
     <row r="995" ht="15.75" customHeight="1"/>
     <row r="996" ht="15.75" customHeight="1"/>
-    <row r="997" ht="15.75" customHeight="1"/>
-    <row r="998" ht="15.75" customHeight="1"/>
-    <row r="999" ht="15.75" customHeight="1"/>
   </sheetData>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.25" right="0.25" top="0.75"/>

</xml_diff>